<commit_message>
build out composite risk free rate tools
</commit_message>
<xml_diff>
--- a/epsilon-phi-core/src/resources/templates/MSCI Index Construction.xlsx
+++ b/epsilon-phi-core/src/resources/templates/MSCI Index Construction.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11008"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26827"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/francisbarker/Repositories/Python/epsilon-phi/epsilon-phi-core/src/resources/templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fabar\repos\epsilon-phi\epsilon-phi-core\src\resources\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{197DB83C-936F-4B4D-8DDA-2C013717079C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A34E9905-6548-44B1-87C6-AC183A1F094D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="57600" windowHeight="32400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13096" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rules" sheetId="40" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="762" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="971" uniqueCount="372">
   <si>
     <r>
       <rPr>
@@ -1053,6 +1053,516 @@
   </si>
   <si>
     <t>Symbol</t>
+  </si>
+  <si>
+    <t>Region</t>
+  </si>
+  <si>
+    <t>MSCI Region</t>
+  </si>
+  <si>
+    <t>Currency</t>
+  </si>
+  <si>
+    <t>ARS</t>
+  </si>
+  <si>
+    <t>AUD</t>
+  </si>
+  <si>
+    <t>ATS</t>
+  </si>
+  <si>
+    <t>BEF</t>
+  </si>
+  <si>
+    <t>BRL</t>
+  </si>
+  <si>
+    <t>CAD</t>
+  </si>
+  <si>
+    <t>CNY</t>
+  </si>
+  <si>
+    <t>COP</t>
+  </si>
+  <si>
+    <t>CZK</t>
+  </si>
+  <si>
+    <t>DKK</t>
+  </si>
+  <si>
+    <t>FIM</t>
+  </si>
+  <si>
+    <t>FRF</t>
+  </si>
+  <si>
+    <t>DEM</t>
+  </si>
+  <si>
+    <t>GRD</t>
+  </si>
+  <si>
+    <t>HKD</t>
+  </si>
+  <si>
+    <t>HUF</t>
+  </si>
+  <si>
+    <t>INR</t>
+  </si>
+  <si>
+    <t>IDR</t>
+  </si>
+  <si>
+    <t>ILS</t>
+  </si>
+  <si>
+    <t>ITL</t>
+  </si>
+  <si>
+    <t>JPY</t>
+  </si>
+  <si>
+    <t>JOD</t>
+  </si>
+  <si>
+    <t>KRW</t>
+  </si>
+  <si>
+    <t>LUF</t>
+  </si>
+  <si>
+    <t>MYR</t>
+  </si>
+  <si>
+    <t>MXN</t>
+  </si>
+  <si>
+    <t>MAD</t>
+  </si>
+  <si>
+    <t>NZD</t>
+  </si>
+  <si>
+    <t>NOK</t>
+  </si>
+  <si>
+    <t>PKR</t>
+  </si>
+  <si>
+    <t>PEN</t>
+  </si>
+  <si>
+    <t>PHP</t>
+  </si>
+  <si>
+    <t>PLN</t>
+  </si>
+  <si>
+    <t>PTE</t>
+  </si>
+  <si>
+    <t>QAD</t>
+  </si>
+  <si>
+    <t>RUB</t>
+  </si>
+  <si>
+    <t>SAR</t>
+  </si>
+  <si>
+    <t>SGD</t>
+  </si>
+  <si>
+    <t>ZAR</t>
+  </si>
+  <si>
+    <t>ESP</t>
+  </si>
+  <si>
+    <t>SEK</t>
+  </si>
+  <si>
+    <t>CHF</t>
+  </si>
+  <si>
+    <t>TWD</t>
+  </si>
+  <si>
+    <t>THB</t>
+  </si>
+  <si>
+    <t>AED</t>
+  </si>
+  <si>
+    <t>GBP</t>
+  </si>
+  <si>
+    <t>USD</t>
+  </si>
+  <si>
+    <t>VEF</t>
+  </si>
+  <si>
+    <t>CLP</t>
+  </si>
+  <si>
+    <t>EGP</t>
+  </si>
+  <si>
+    <t>IEP</t>
+  </si>
+  <si>
+    <t>KWD</t>
+  </si>
+  <si>
+    <t>NLG</t>
+  </si>
+  <si>
+    <t>TRY</t>
+  </si>
+  <si>
+    <t>LKR</t>
+  </si>
+  <si>
+    <t>Local</t>
+  </si>
+  <si>
+    <t>MSASTR$</t>
+  </si>
+  <si>
+    <t>MSASTRL</t>
+  </si>
+  <si>
+    <t>MSAUST$</t>
+  </si>
+  <si>
+    <t>MSAUSTL</t>
+  </si>
+  <si>
+    <t>MSBELG$</t>
+  </si>
+  <si>
+    <t>MSBELGL</t>
+  </si>
+  <si>
+    <t>MSBRAZ$</t>
+  </si>
+  <si>
+    <t>MSBRAZL</t>
+  </si>
+  <si>
+    <t>MSCHIL$</t>
+  </si>
+  <si>
+    <t>MSCHILL</t>
+  </si>
+  <si>
+    <t>MSCHIN$</t>
+  </si>
+  <si>
+    <t>MSCHINL</t>
+  </si>
+  <si>
+    <t>MSCNDA$</t>
+  </si>
+  <si>
+    <t>MSCNDAL</t>
+  </si>
+  <si>
+    <t>MSCOLM$</t>
+  </si>
+  <si>
+    <t>MSCOLML</t>
+  </si>
+  <si>
+    <t>MSCZCH$</t>
+  </si>
+  <si>
+    <t>MSCZCHL</t>
+  </si>
+  <si>
+    <t>MSDNMK$</t>
+  </si>
+  <si>
+    <t>MSDNMKL</t>
+  </si>
+  <si>
+    <t>MSEGYT$</t>
+  </si>
+  <si>
+    <t>MSEGYTL</t>
+  </si>
+  <si>
+    <t>MSEIRE$</t>
+  </si>
+  <si>
+    <t>MSEIREL</t>
+  </si>
+  <si>
+    <t>MSFIND$</t>
+  </si>
+  <si>
+    <t>MSFINDL</t>
+  </si>
+  <si>
+    <t>MSFRNC$</t>
+  </si>
+  <si>
+    <t>MSFRNCL</t>
+  </si>
+  <si>
+    <t>MSGERM$</t>
+  </si>
+  <si>
+    <t>MSGERML</t>
+  </si>
+  <si>
+    <t>MSGREE$</t>
+  </si>
+  <si>
+    <t>MSGREEL</t>
+  </si>
+  <si>
+    <t>MSHGKG$</t>
+  </si>
+  <si>
+    <t>MSHGKGL</t>
+  </si>
+  <si>
+    <t>MSHUNG$</t>
+  </si>
+  <si>
+    <t>MSHUNGL</t>
+  </si>
+  <si>
+    <t>MSINDF$</t>
+  </si>
+  <si>
+    <t>MSINDFL</t>
+  </si>
+  <si>
+    <t>MSINDI$</t>
+  </si>
+  <si>
+    <t>MSINDIL</t>
+  </si>
+  <si>
+    <t>MSISRL$</t>
+  </si>
+  <si>
+    <t>MSISRLL</t>
+  </si>
+  <si>
+    <t>MSITAL$</t>
+  </si>
+  <si>
+    <t>MSITALL</t>
+  </si>
+  <si>
+    <t>MSJPAN$</t>
+  </si>
+  <si>
+    <t>MSJPANL</t>
+  </si>
+  <si>
+    <t>MSKORE$</t>
+  </si>
+  <si>
+    <t>MSKOREL</t>
+  </si>
+  <si>
+    <t>MSKUWA$</t>
+  </si>
+  <si>
+    <t>MSKUWAL</t>
+  </si>
+  <si>
+    <t>MSMALF$</t>
+  </si>
+  <si>
+    <t>MSMALFL</t>
+  </si>
+  <si>
+    <t>MSMEXF$</t>
+  </si>
+  <si>
+    <t>MSMEXFL</t>
+  </si>
+  <si>
+    <t>MSNETH$</t>
+  </si>
+  <si>
+    <t>MSNETHL</t>
+  </si>
+  <si>
+    <t>MSNWAY$</t>
+  </si>
+  <si>
+    <t>MSNWAYL</t>
+  </si>
+  <si>
+    <t>MSNZEA$</t>
+  </si>
+  <si>
+    <t>MSNZEAL</t>
+  </si>
+  <si>
+    <t>MSPERU$</t>
+  </si>
+  <si>
+    <t>MSPERUL</t>
+  </si>
+  <si>
+    <t>MSPHLF$</t>
+  </si>
+  <si>
+    <t>MSPHLFL</t>
+  </si>
+  <si>
+    <t>MSPLND$</t>
+  </si>
+  <si>
+    <t>MSPLNDL</t>
+  </si>
+  <si>
+    <t>MSPORD$</t>
+  </si>
+  <si>
+    <t>MSPORDL</t>
+  </si>
+  <si>
+    <t>MSQATA$</t>
+  </si>
+  <si>
+    <t>MSQATAL</t>
+  </si>
+  <si>
+    <t>MSSARF$</t>
+  </si>
+  <si>
+    <t>MSSARFL</t>
+  </si>
+  <si>
+    <t>MSSAUD$</t>
+  </si>
+  <si>
+    <t>MSSAUDL</t>
+  </si>
+  <si>
+    <t>MSSING$</t>
+  </si>
+  <si>
+    <t>MSSINGL</t>
+  </si>
+  <si>
+    <t>MSSPAN$</t>
+  </si>
+  <si>
+    <t>MSSPANL</t>
+  </si>
+  <si>
+    <t>MSSWDN$</t>
+  </si>
+  <si>
+    <t>MSSWDNL</t>
+  </si>
+  <si>
+    <t>MSSWIT$</t>
+  </si>
+  <si>
+    <t>MSSWITL</t>
+  </si>
+  <si>
+    <t>MSTAIW$</t>
+  </si>
+  <si>
+    <t>MSTAIWL</t>
+  </si>
+  <si>
+    <t>MSTHAF$</t>
+  </si>
+  <si>
+    <t>MSTHAFL</t>
+  </si>
+  <si>
+    <t>MSTURK$</t>
+  </si>
+  <si>
+    <t>MSTURKL</t>
+  </si>
+  <si>
+    <t>MSUAEI$</t>
+  </si>
+  <si>
+    <t>MSUAEIL</t>
+  </si>
+  <si>
+    <t>MSUSAM$</t>
+  </si>
+  <si>
+    <t>MSUSAML</t>
+  </si>
+  <si>
+    <t>MSUTDK$</t>
+  </si>
+  <si>
+    <t>MSUTDKL</t>
+  </si>
+  <si>
+    <t>MSARGT$</t>
+  </si>
+  <si>
+    <t>MSARGTL</t>
+  </si>
+  <si>
+    <t>MSJORD$</t>
+  </si>
+  <si>
+    <t>MSJORDL</t>
+  </si>
+  <si>
+    <t>MSLUXB$</t>
+  </si>
+  <si>
+    <t>MSLUXBL</t>
+  </si>
+  <si>
+    <t>MSMORC$</t>
+  </si>
+  <si>
+    <t>MSMORCL</t>
+  </si>
+  <si>
+    <t>MSPAKI$</t>
+  </si>
+  <si>
+    <t>MSPAKIL</t>
+  </si>
+  <si>
+    <t>MSRUSS$</t>
+  </si>
+  <si>
+    <t>MSRUSSL</t>
+  </si>
+  <si>
+    <t>MSSRIL$</t>
+  </si>
+  <si>
+    <t>MSSRILL</t>
+  </si>
+  <si>
+    <t>MSVENF$</t>
+  </si>
+  <si>
+    <t>MSVENFL</t>
+  </si>
+  <si>
+    <t>Dollar</t>
   </si>
 </sst>
 </file>
@@ -1150,7 +1660,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -1178,9 +1688,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -1189,6 +1696,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1496,15 +2009,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{398A9000-FE9A-0D49-BC15-66DEE1B3B201}">
   <dimension ref="A1:J70"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="13"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="13.15"/>
   <cols>
-    <col min="1" max="1" width="31.796875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="21.19921875" style="6" customWidth="1"/>
-    <col min="3" max="10" width="17.796875" style="6" customWidth="1"/>
+    <col min="1" max="1" width="31.78515625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="21.2109375" style="6" customWidth="1"/>
+    <col min="3" max="10" width="17.78515625" style="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="12" customFormat="1" ht="19" customHeight="1">
-      <c r="A1" s="11" t="s">
+    <row r="1" spans="1:10" s="11" customFormat="1" ht="19.05" customHeight="1">
+      <c r="A1" s="10" t="s">
         <v>200</v>
       </c>
       <c r="B1" s="4" t="s">
@@ -1535,8 +2048,8 @@
         <v>122</v>
       </c>
     </row>
-    <row r="2" spans="1:10" s="12" customFormat="1" ht="19" customHeight="1">
-      <c r="A2" s="11" t="s">
+    <row r="2" spans="1:10" s="11" customFormat="1" ht="19.05" customHeight="1">
+      <c r="A2" s="10" t="s">
         <v>201</v>
       </c>
       <c r="B2" s="4" t="s">
@@ -1567,7 +2080,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="16" customHeight="1">
+    <row r="3" spans="1:10" ht="16.05" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>0</v>
       </c>
@@ -1599,7 +2112,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="16" customHeight="1">
+    <row r="4" spans="1:10" ht="16.05" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>1</v>
       </c>
@@ -1631,7 +2144,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="16" customHeight="1">
+    <row r="5" spans="1:10" ht="16.05" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>2</v>
       </c>
@@ -1663,7 +2176,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="16" customHeight="1">
+    <row r="6" spans="1:10" ht="16.05" customHeight="1">
       <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
@@ -1695,7 +2208,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="16" customHeight="1">
+    <row r="7" spans="1:10" ht="16.05" customHeight="1">
       <c r="A7" s="2" t="s">
         <v>4</v>
       </c>
@@ -1727,7 +2240,7 @@
         <v>32143</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="16" customHeight="1">
+    <row r="8" spans="1:10" ht="16.05" customHeight="1">
       <c r="A8" s="3" t="s">
         <v>123</v>
       </c>
@@ -1759,7 +2272,7 @@
         <v>32143</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="16" customHeight="1">
+    <row r="9" spans="1:10" ht="16.05" customHeight="1">
       <c r="A9" s="2" t="s">
         <v>5</v>
       </c>
@@ -1791,7 +2304,7 @@
         <v>32143</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="16" customHeight="1">
+    <row r="10" spans="1:10" ht="16.05" customHeight="1">
       <c r="A10" s="2" t="s">
         <v>6</v>
       </c>
@@ -1823,7 +2336,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="16" customHeight="1">
+    <row r="11" spans="1:10" ht="16.05" customHeight="1">
       <c r="A11" s="2" t="s">
         <v>7</v>
       </c>
@@ -1855,7 +2368,7 @@
         <v>34367</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="16" customHeight="1">
+    <row r="12" spans="1:10" ht="16.05" customHeight="1">
       <c r="A12" s="2" t="s">
         <v>8</v>
       </c>
@@ -1887,7 +2400,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="16" customHeight="1">
+    <row r="13" spans="1:10" ht="16.05" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>9</v>
       </c>
@@ -1919,7 +2432,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="16" customHeight="1">
+    <row r="14" spans="1:10" ht="16.05" customHeight="1">
       <c r="A14" s="2" t="s">
         <v>10</v>
       </c>
@@ -1951,7 +2464,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="16" customHeight="1">
+    <row r="15" spans="1:10" ht="16.05" customHeight="1">
       <c r="A15" s="2" t="s">
         <v>11</v>
       </c>
@@ -1983,7 +2496,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="16" customHeight="1">
+    <row r="16" spans="1:10" ht="16.05" customHeight="1">
       <c r="A16" s="2" t="s">
         <v>12</v>
       </c>
@@ -2015,7 +2528,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="16" customHeight="1">
+    <row r="17" spans="1:10" ht="16.05" customHeight="1">
       <c r="A17" s="2" t="s">
         <v>13</v>
       </c>
@@ -2047,7 +2560,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="16" customHeight="1">
+    <row r="18" spans="1:10" ht="16.05" customHeight="1">
       <c r="A18" s="2" t="s">
         <v>14</v>
       </c>
@@ -2079,7 +2592,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="16" customHeight="1">
+    <row r="19" spans="1:10" ht="16.05" customHeight="1">
       <c r="A19" s="2" t="s">
         <v>15</v>
       </c>
@@ -2111,7 +2624,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="16" customHeight="1">
+    <row r="20" spans="1:10" ht="16.05" customHeight="1">
       <c r="A20" s="2" t="s">
         <v>16</v>
       </c>
@@ -2143,7 +2656,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="16" customHeight="1">
+    <row r="21" spans="1:10" ht="16.05" customHeight="1">
       <c r="A21" s="2" t="s">
         <v>17</v>
       </c>
@@ -2175,7 +2688,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="16" customHeight="1">
+    <row r="22" spans="1:10" ht="16.05" customHeight="1">
       <c r="A22" s="2" t="s">
         <v>18</v>
       </c>
@@ -2207,7 +2720,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="16" customHeight="1">
+    <row r="23" spans="1:10" ht="16.05" customHeight="1">
       <c r="A23" s="2" t="s">
         <v>19</v>
       </c>
@@ -2239,7 +2752,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="16" customHeight="1">
+    <row r="24" spans="1:10" ht="16.05" customHeight="1">
       <c r="A24" s="2" t="s">
         <v>20</v>
       </c>
@@ -2271,7 +2784,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="16" customHeight="1">
+    <row r="25" spans="1:10" ht="16.05" customHeight="1">
       <c r="A25" s="3" t="s">
         <v>124</v>
       </c>
@@ -2303,7 +2816,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="16" customHeight="1">
+    <row r="26" spans="1:10" ht="16.05" customHeight="1">
       <c r="A26" s="2" t="s">
         <v>21</v>
       </c>
@@ -2335,7 +2848,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="16" customHeight="1">
+    <row r="27" spans="1:10" ht="16.05" customHeight="1">
       <c r="A27" s="2" t="s">
         <v>22</v>
       </c>
@@ -2367,7 +2880,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="16" customHeight="1">
+    <row r="28" spans="1:10" ht="16.05" customHeight="1">
       <c r="A28" s="2" t="s">
         <v>23</v>
       </c>
@@ -2399,7 +2912,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="16" customHeight="1">
+    <row r="29" spans="1:10" ht="16.05" customHeight="1">
       <c r="A29" s="2" t="s">
         <v>24</v>
       </c>
@@ -2431,7 +2944,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="16" customHeight="1">
+    <row r="30" spans="1:10" ht="16.05" customHeight="1">
       <c r="A30" s="2" t="s">
         <v>25</v>
       </c>
@@ -2463,7 +2976,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="16" customHeight="1">
+    <row r="31" spans="1:10" ht="16.05" customHeight="1">
       <c r="A31" s="3" t="s">
         <v>125</v>
       </c>
@@ -2495,7 +3008,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="16" customHeight="1">
+    <row r="32" spans="1:10" ht="16.05" customHeight="1">
       <c r="A32" s="2" t="s">
         <v>26</v>
       </c>
@@ -2527,7 +3040,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ht="16" customHeight="1">
+    <row r="33" spans="1:10" ht="16.05" customHeight="1">
       <c r="A33" s="2" t="s">
         <v>27</v>
       </c>
@@ -2559,7 +3072,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="16" customHeight="1">
+    <row r="34" spans="1:10" ht="16.05" customHeight="1">
       <c r="A34" s="2" t="s">
         <v>28</v>
       </c>
@@ -2591,7 +3104,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="35" spans="1:10" ht="16" customHeight="1">
+    <row r="35" spans="1:10" ht="16.05" customHeight="1">
       <c r="A35" s="2" t="s">
         <v>29</v>
       </c>
@@ -2623,7 +3136,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="36" spans="1:10" ht="16" customHeight="1">
+    <row r="36" spans="1:10" ht="16.05" customHeight="1">
       <c r="A36" s="2" t="s">
         <v>30</v>
       </c>
@@ -2655,7 +3168,7 @@
         <v>32143</v>
       </c>
     </row>
-    <row r="37" spans="1:10" ht="16" customHeight="1">
+    <row r="37" spans="1:10" ht="16.05" customHeight="1">
       <c r="A37" s="2" t="s">
         <v>31</v>
       </c>
@@ -2687,7 +3200,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="38" spans="1:10" ht="16" customHeight="1">
+    <row r="38" spans="1:10" ht="16.05" customHeight="1">
       <c r="A38" s="2" t="s">
         <v>32</v>
       </c>
@@ -2719,7 +3232,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="39" spans="1:10" ht="16" customHeight="1">
+    <row r="39" spans="1:10" ht="16.05" customHeight="1">
       <c r="A39" s="2" t="s">
         <v>33</v>
       </c>
@@ -2751,7 +3264,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="40" spans="1:10" ht="16" customHeight="1">
+    <row r="40" spans="1:10" ht="16.05" customHeight="1">
       <c r="A40" s="2" t="s">
         <v>34</v>
       </c>
@@ -2783,7 +3296,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="41" spans="1:10" ht="16" customHeight="1">
+    <row r="41" spans="1:10" ht="16.05" customHeight="1">
       <c r="A41" s="2" t="s">
         <v>35</v>
       </c>
@@ -2815,7 +3328,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="42" spans="1:10" ht="16" customHeight="1">
+    <row r="42" spans="1:10" ht="16.05" customHeight="1">
       <c r="A42" s="3" t="s">
         <v>126</v>
       </c>
@@ -2847,7 +3360,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="43" spans="1:10" ht="16" customHeight="1">
+    <row r="43" spans="1:10" ht="16.05" customHeight="1">
       <c r="A43" s="2" t="s">
         <v>36</v>
       </c>
@@ -2879,7 +3392,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="44" spans="1:10" ht="16" customHeight="1">
+    <row r="44" spans="1:10" ht="16.05" customHeight="1">
       <c r="A44" s="2" t="s">
         <v>37</v>
       </c>
@@ -2911,7 +3424,7 @@
         <v>34367</v>
       </c>
     </row>
-    <row r="45" spans="1:10" ht="16" customHeight="1">
+    <row r="45" spans="1:10" ht="16.05" customHeight="1">
       <c r="A45" s="2" t="s">
         <v>38</v>
       </c>
@@ -2943,7 +3456,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="46" spans="1:10" ht="16" customHeight="1">
+    <row r="46" spans="1:10" ht="16.05" customHeight="1">
       <c r="A46" s="2" t="s">
         <v>39</v>
       </c>
@@ -2975,7 +3488,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="47" spans="1:10" ht="16" customHeight="1">
+    <row r="47" spans="1:10" ht="16.05" customHeight="1">
       <c r="A47" s="2" t="s">
         <v>40</v>
       </c>
@@ -3007,7 +3520,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="48" spans="1:10" ht="16" customHeight="1">
+    <row r="48" spans="1:10" ht="16.05" customHeight="1">
       <c r="A48" s="2" t="s">
         <v>41</v>
       </c>
@@ -3039,7 +3552,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="49" spans="1:10" ht="16" customHeight="1">
+    <row r="49" spans="1:10" ht="16.05" customHeight="1">
       <c r="A49" s="2" t="s">
         <v>42</v>
       </c>
@@ -3071,7 +3584,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="50" spans="1:10" ht="16" customHeight="1">
+    <row r="50" spans="1:10" ht="16.05" customHeight="1">
       <c r="A50" s="2" t="s">
         <v>43</v>
       </c>
@@ -3103,7 +3616,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="51" spans="1:10" ht="16" customHeight="1">
+    <row r="51" spans="1:10" ht="16.05" customHeight="1">
       <c r="A51" s="3" t="s">
         <v>59</v>
       </c>
@@ -3135,7 +3648,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="52" spans="1:10" ht="16" customHeight="1">
+    <row r="52" spans="1:10" ht="16.05" customHeight="1">
       <c r="A52" s="2" t="s">
         <v>44</v>
       </c>
@@ -3167,7 +3680,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="53" spans="1:10" ht="16" customHeight="1">
+    <row r="53" spans="1:10" ht="16.05" customHeight="1">
       <c r="A53" s="3" t="s">
         <v>127</v>
       </c>
@@ -3199,7 +3712,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="54" spans="1:10" ht="16" customHeight="1">
+    <row r="54" spans="1:10" ht="16.05" customHeight="1">
       <c r="A54" s="2" t="s">
         <v>45</v>
       </c>
@@ -3231,7 +3744,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="55" spans="1:10" ht="16" customHeight="1">
+    <row r="55" spans="1:10" ht="16.05" customHeight="1">
       <c r="A55" s="3" t="s">
         <v>128</v>
       </c>
@@ -3263,7 +3776,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="56" spans="1:10" ht="16" customHeight="1">
+    <row r="56" spans="1:10" ht="16.05" customHeight="1">
       <c r="A56" s="2" t="s">
         <v>46</v>
       </c>
@@ -3295,7 +3808,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="57" spans="1:10" ht="16" customHeight="1">
+    <row r="57" spans="1:10" ht="16.05" customHeight="1">
       <c r="A57" s="2" t="s">
         <v>47</v>
       </c>
@@ -3327,7 +3840,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="58" spans="1:10" ht="16" customHeight="1">
+    <row r="58" spans="1:10" ht="16.05" customHeight="1">
       <c r="A58" s="2" t="s">
         <v>48</v>
       </c>
@@ -3359,7 +3872,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="59" spans="1:10" ht="16" customHeight="1">
+    <row r="59" spans="1:10" ht="16.05" customHeight="1">
       <c r="A59" s="2" t="s">
         <v>49</v>
       </c>
@@ -3391,7 +3904,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="60" spans="1:10" ht="16" customHeight="1">
+    <row r="60" spans="1:10" ht="16.05" customHeight="1">
       <c r="A60" s="2" t="s">
         <v>50</v>
       </c>
@@ -3423,7 +3936,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="61" spans="1:10" ht="16" customHeight="1">
+    <row r="61" spans="1:10" ht="16.05" customHeight="1">
       <c r="A61" s="2" t="s">
         <v>51</v>
       </c>
@@ -3455,7 +3968,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="62" spans="1:10" ht="16" customHeight="1">
+    <row r="62" spans="1:10" ht="16.05" customHeight="1">
       <c r="A62" s="2" t="s">
         <v>52</v>
       </c>
@@ -3487,7 +4000,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="63" spans="1:10" ht="16" customHeight="1">
+    <row r="63" spans="1:10" ht="16.05" customHeight="1">
       <c r="A63" s="7" t="s">
         <v>129</v>
       </c>
@@ -3519,7 +4032,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="64" spans="1:10" ht="16" customHeight="1">
+    <row r="64" spans="1:10" ht="16.05" customHeight="1">
       <c r="A64" s="2" t="s">
         <v>53</v>
       </c>
@@ -3551,7 +4064,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="65" spans="1:10" ht="16" customHeight="1">
+    <row r="65" spans="1:10" ht="16.05" customHeight="1">
       <c r="A65" s="2" t="s">
         <v>54</v>
       </c>
@@ -3583,7 +4096,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="66" spans="1:10" ht="16" customHeight="1">
+    <row r="66" spans="1:10" ht="16.05" customHeight="1">
       <c r="A66" s="2" t="s">
         <v>55</v>
       </c>
@@ -3615,7 +4128,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="67" spans="1:10" ht="16" customHeight="1">
+    <row r="67" spans="1:10" ht="16.05" customHeight="1">
       <c r="A67" s="2" t="s">
         <v>56</v>
       </c>
@@ -3647,7 +4160,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="68" spans="1:10" ht="16" customHeight="1">
+    <row r="68" spans="1:10" ht="16.05" customHeight="1">
       <c r="A68" s="2" t="s">
         <v>57</v>
       </c>
@@ -3679,7 +4192,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="69" spans="1:10" ht="16" customHeight="1">
+    <row r="69" spans="1:10" ht="16.05" customHeight="1">
       <c r="A69" s="3" t="s">
         <v>130</v>
       </c>
@@ -3711,7 +4224,7 @@
         <v>32143</v>
       </c>
     </row>
-    <row r="70" spans="1:10" ht="16" customHeight="1">
+    <row r="70" spans="1:10" ht="16.05" customHeight="1">
       <c r="A70" s="2" t="s">
         <v>58</v>
       </c>
@@ -3753,584 +4266,1198 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A7EF705-CFED-174D-8EBB-657B7E248B5D}">
-  <dimension ref="A1:F77"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="13"/>
+  <dimension ref="A2:G79"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="13.15"/>
   <cols>
-    <col min="1" max="1" width="19.3984375" customWidth="1"/>
-    <col min="2" max="2" width="29.3984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.19921875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.42578125" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="11.5" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="14" customHeight="1">
-      <c r="A1" s="2" t="s">
+    <row r="2" spans="1:5">
+      <c r="A2" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="14" customHeight="1">
+      <c r="A3" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B3" s="8" t="s">
         <v>183</v>
       </c>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-    </row>
-    <row r="2" spans="1:4" ht="14" customHeight="1">
-      <c r="A2" s="2" t="s">
+      <c r="C3" s="8" t="s">
+        <v>356</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>355</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="14" customHeight="1">
+      <c r="A4" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B4" s="1" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="14" customHeight="1">
-      <c r="A3" s="2" t="s">
+      <c r="C4" s="8" t="s">
+        <v>264</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>263</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="14" customHeight="1">
+      <c r="A5" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B5" s="1" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="14" customHeight="1">
-      <c r="A4" s="2" t="s">
+      <c r="C5" s="8" t="s">
+        <v>262</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>261</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="14" customHeight="1">
+      <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B6" s="1" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="14" customHeight="1">
-      <c r="A5" s="2" t="s">
+      <c r="C6" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="14" customHeight="1">
+      <c r="A7" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B7" s="1" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" ht="14" customHeight="1">
-      <c r="A6" s="3" t="s">
+      <c r="C7" s="8" t="s">
+        <v>268</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>267</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="14" customHeight="1">
+      <c r="A8" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B8" s="1" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" ht="14" customHeight="1">
-      <c r="A7" s="2" t="s">
+      <c r="C8" s="8" t="s">
+        <v>274</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>273</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="14" customHeight="1">
+      <c r="A9" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B9" s="1" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" ht="14" customHeight="1">
-      <c r="A8" s="2" t="s">
+      <c r="C9" s="8" t="s">
+        <v>270</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>269</v>
+      </c>
+      <c r="E9" s="12" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="14" customHeight="1">
+      <c r="A10" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B10" s="1" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" ht="14" customHeight="1">
-      <c r="A9" s="2" t="s">
+      <c r="C10" s="8" t="s">
+        <v>272</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>271</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="14" customHeight="1">
+      <c r="A11" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B11" s="1" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" ht="14" customHeight="1">
-      <c r="A10" s="2" t="s">
+      <c r="C11" s="8" t="s">
+        <v>276</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>275</v>
+      </c>
+      <c r="E11" s="12" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="14" customHeight="1">
+      <c r="A12" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B12" s="1" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" ht="14" customHeight="1">
-      <c r="A11" s="2" t="s">
+      <c r="C12" s="8" t="s">
+        <v>278</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>277</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="14" customHeight="1">
+      <c r="A13" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B13" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" ht="14" customHeight="1">
-      <c r="A12" s="2" t="s">
+      <c r="C13" s="8" t="s">
+        <v>280</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>279</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="14" customHeight="1">
+      <c r="A14" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B14" s="1" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" ht="14" customHeight="1">
-      <c r="A13" s="2" t="s">
+      <c r="C14" s="8" t="s">
+        <v>282</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>281</v>
+      </c>
+      <c r="E14" s="12" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="14" customHeight="1">
+      <c r="A15" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B15" s="1" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" ht="14" customHeight="1">
-      <c r="A14" s="2" t="s">
+      <c r="C15" s="8" t="s">
+        <v>286</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="E15" s="12" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="14" customHeight="1">
+      <c r="A16" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B16" s="8" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" ht="14" customHeight="1">
-      <c r="A15" s="2" t="s">
+      <c r="C16" s="8" t="s">
+        <v>286</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="E16" s="12" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="14" customHeight="1">
+      <c r="A17" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B17" s="1" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" ht="14" customHeight="1">
-      <c r="A16" s="2" t="s">
+      <c r="C17" s="8" t="s">
+        <v>288</v>
+      </c>
+      <c r="D17" s="12" t="s">
+        <v>287</v>
+      </c>
+      <c r="E17" s="12" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="14" customHeight="1">
+      <c r="A18" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B18" s="1" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" ht="14" customHeight="1">
-      <c r="A17" s="2" t="s">
+      <c r="C18" s="8" t="s">
+        <v>290</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>289</v>
+      </c>
+      <c r="E18" s="12" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="14" customHeight="1">
+      <c r="A19" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B19" s="1" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" ht="14" customHeight="1">
-      <c r="A18" s="2" t="s">
+      <c r="C19" s="8" t="s">
+        <v>292</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>291</v>
+      </c>
+      <c r="E19" s="12" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="14" customHeight="1">
+      <c r="A20" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B20" s="1" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" ht="14" customHeight="1">
-      <c r="A19" s="2" t="s">
+      <c r="C20" s="8" t="s">
+        <v>294</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>293</v>
+      </c>
+      <c r="E20" s="12" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="14" customHeight="1">
+      <c r="A21" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B21" s="1" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" ht="14" customHeight="1">
-      <c r="A20" s="2" t="s">
+      <c r="C21" s="8" t="s">
+        <v>296</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>295</v>
+      </c>
+      <c r="E21" s="12" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="14" customHeight="1">
+      <c r="A22" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B22" s="1" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" ht="14" customHeight="1">
-      <c r="A21" s="2" t="s">
+      <c r="C22" s="8" t="s">
+        <v>300</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>299</v>
+      </c>
+      <c r="E22" s="12" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="14" customHeight="1">
+      <c r="A23" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B23" s="1" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" ht="14" customHeight="1">
-      <c r="A22" s="2" t="s">
+      <c r="C23" s="8" t="s">
+        <v>298</v>
+      </c>
+      <c r="D23" s="12" t="s">
+        <v>297</v>
+      </c>
+      <c r="E23" s="12" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="14" customHeight="1">
+      <c r="A24" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B24" s="1" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" ht="14" customHeight="1">
-      <c r="A23" s="3" t="s">
+      <c r="C24" s="8" t="s">
+        <v>298</v>
+      </c>
+      <c r="D24" s="12" t="s">
+        <v>297</v>
+      </c>
+      <c r="E24" s="12" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="14" customHeight="1">
+      <c r="A25" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B25" s="1" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" ht="14" customHeight="1">
-      <c r="A24" s="2" t="s">
+      <c r="C25" s="8" t="s">
+        <v>284</v>
+      </c>
+      <c r="D25" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="E25" s="12" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="14" customHeight="1">
+      <c r="A26" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B26" s="1" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" ht="14" customHeight="1">
-      <c r="A25" s="2" t="s">
+      <c r="C26" s="8" t="s">
+        <v>302</v>
+      </c>
+      <c r="D26" s="12" t="s">
+        <v>301</v>
+      </c>
+      <c r="E26" s="12" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="14" customHeight="1">
+      <c r="A27" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="B27" s="1" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" ht="14" customHeight="1">
-      <c r="A26" s="2" t="s">
+      <c r="C27" s="8" t="s">
+        <v>304</v>
+      </c>
+      <c r="D27" s="12" t="s">
+        <v>303</v>
+      </c>
+      <c r="E27" s="12" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="14" customHeight="1">
+      <c r="A28" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B28" s="1" t="s">
         <v>158</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" ht="14" customHeight="1">
-      <c r="A27" s="2" t="s">
+      <c r="C28" s="8" t="s">
+        <v>306</v>
+      </c>
+      <c r="D28" s="12" t="s">
+        <v>305</v>
+      </c>
+      <c r="E28" s="12" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="14" customHeight="1">
+      <c r="A29" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B27" s="8" t="s">
+      <c r="B29" s="8" t="s">
         <v>184</v>
       </c>
-      <c r="C27" s="9"/>
-      <c r="D27" s="9"/>
-    </row>
-    <row r="28" spans="1:4" ht="14" customHeight="1">
-      <c r="A28" s="2" t="s">
+      <c r="C29" s="8" t="s">
+        <v>358</v>
+      </c>
+      <c r="D29" s="12" t="s">
+        <v>357</v>
+      </c>
+      <c r="E29" s="12" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="14" customHeight="1">
+      <c r="A30" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B30" s="1" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" ht="14" customHeight="1">
-      <c r="A29" s="3" t="s">
+      <c r="C30" s="8" t="s">
+        <v>308</v>
+      </c>
+      <c r="D30" s="12" t="s">
+        <v>307</v>
+      </c>
+      <c r="E30" s="12" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="14" customHeight="1">
+      <c r="A31" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="B31" s="1" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" ht="14" customHeight="1">
-      <c r="A30" s="2" t="s">
+      <c r="C31" s="8" t="s">
+        <v>308</v>
+      </c>
+      <c r="D31" s="12" t="s">
+        <v>307</v>
+      </c>
+      <c r="E31" s="12" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="14" customHeight="1">
+      <c r="A32" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B30" s="1" t="s">
+      <c r="B32" s="1" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="31" spans="1:4" ht="14" customHeight="1">
-      <c r="A31" s="2" t="s">
+      <c r="C32" s="8" t="s">
+        <v>310</v>
+      </c>
+      <c r="D32" s="12" t="s">
+        <v>309</v>
+      </c>
+      <c r="E32" s="12" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="14" customHeight="1">
+      <c r="A33" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B31" s="8" t="s">
+      <c r="B33" s="8" t="s">
         <v>185</v>
       </c>
-      <c r="C31" s="9"/>
-      <c r="D31" s="9"/>
-    </row>
-    <row r="32" spans="1:4" ht="14" customHeight="1">
-      <c r="A32" s="2" t="s">
+      <c r="C33" s="8" t="s">
+        <v>360</v>
+      </c>
+      <c r="D33" s="12" t="s">
+        <v>359</v>
+      </c>
+      <c r="E33" s="12" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="14" customHeight="1">
+      <c r="A34" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B34" s="1" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="33" spans="1:4" ht="14" customHeight="1">
-      <c r="A33" s="2" t="s">
+      <c r="C34" s="8" t="s">
+        <v>312</v>
+      </c>
+      <c r="D34" s="12" t="s">
+        <v>311</v>
+      </c>
+      <c r="E34" s="12" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="14" customHeight="1">
+      <c r="A35" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="B35" s="1" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="34" spans="1:4" ht="14" customHeight="1">
-      <c r="A34" s="2" t="s">
+      <c r="C35" s="8" t="s">
+        <v>312</v>
+      </c>
+      <c r="D35" s="12" t="s">
+        <v>311</v>
+      </c>
+      <c r="E35" s="12" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="14" customHeight="1">
+      <c r="A36" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B36" s="1" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="35" spans="1:4" ht="14" customHeight="1">
-      <c r="A35" s="2" t="s">
+      <c r="C36" s="8" t="s">
+        <v>314</v>
+      </c>
+      <c r="D36" s="12" t="s">
+        <v>313</v>
+      </c>
+      <c r="E36" s="12" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="14" customHeight="1">
+      <c r="A37" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="B37" s="1" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="36" spans="1:4" ht="14" customHeight="1">
-      <c r="A36" s="2" t="s">
+      <c r="C37" s="8" t="s">
+        <v>314</v>
+      </c>
+      <c r="D37" s="12" t="s">
+        <v>313</v>
+      </c>
+      <c r="E37" s="12" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="14" customHeight="1">
+      <c r="A38" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B36" s="8" t="s">
+      <c r="B38" s="8" t="s">
         <v>186</v>
       </c>
-      <c r="C36" s="9"/>
-      <c r="D36" s="9"/>
-    </row>
-    <row r="37" spans="1:4" ht="14" customHeight="1">
-      <c r="A37" s="2" t="s">
+      <c r="C38" s="8" t="s">
+        <v>362</v>
+      </c>
+      <c r="D38" s="12" t="s">
+        <v>361</v>
+      </c>
+      <c r="E38" s="12" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="14" customHeight="1">
+      <c r="A39" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B37" s="1" t="s">
+      <c r="B39" s="1" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="38" spans="1:4" ht="14" customHeight="1">
-      <c r="A38" s="2" t="s">
+      <c r="C39" s="8" t="s">
+        <v>316</v>
+      </c>
+      <c r="D39" s="12" t="s">
+        <v>315</v>
+      </c>
+      <c r="E39" s="12" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="14" customHeight="1">
+      <c r="A40" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B38" s="1" t="s">
+      <c r="B40" s="1" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="39" spans="1:4" ht="14" customHeight="1">
-      <c r="A39" s="2" t="s">
+      <c r="C40" s="8" t="s">
+        <v>320</v>
+      </c>
+      <c r="D40" s="12" t="s">
+        <v>319</v>
+      </c>
+      <c r="E40" s="12" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="14" customHeight="1">
+      <c r="A41" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B39" s="1" t="s">
+      <c r="B41" s="1" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="40" spans="1:4" ht="14" customHeight="1">
-      <c r="A40" s="3" t="s">
+      <c r="C41" s="8" t="s">
+        <v>318</v>
+      </c>
+      <c r="D41" s="12" t="s">
+        <v>317</v>
+      </c>
+      <c r="E41" s="12" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="14" customHeight="1">
+      <c r="A42" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="B40" s="1" t="s">
+      <c r="B42" s="1" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="41" spans="1:4" ht="14" customHeight="1">
-      <c r="A41" s="2" t="s">
+      <c r="C42" s="8" t="s">
+        <v>318</v>
+      </c>
+      <c r="D42" s="12" t="s">
+        <v>317</v>
+      </c>
+      <c r="E42" s="12" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="14" customHeight="1">
+      <c r="A43" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B41" s="8" t="s">
+      <c r="B43" s="8" t="s">
         <v>187</v>
       </c>
-      <c r="C41" s="9"/>
-      <c r="D41" s="9"/>
-    </row>
-    <row r="42" spans="1:4" ht="14" customHeight="1">
-      <c r="A42" s="2" t="s">
+      <c r="C43" s="8" t="s">
+        <v>364</v>
+      </c>
+      <c r="D43" s="12" t="s">
+        <v>363</v>
+      </c>
+      <c r="E43" s="12" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="14" customHeight="1">
+      <c r="A44" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B42" s="1" t="s">
+      <c r="B44" s="1" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="43" spans="1:4" ht="14" customHeight="1">
-      <c r="A43" s="2" t="s">
+      <c r="C44" s="8" t="s">
+        <v>322</v>
+      </c>
+      <c r="D44" s="12" t="s">
+        <v>321</v>
+      </c>
+      <c r="E44" s="12" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="14" customHeight="1">
+      <c r="A45" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B43" s="1" t="s">
+      <c r="B45" s="1" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="44" spans="1:4" ht="14" customHeight="1">
-      <c r="A44" s="2" t="s">
+      <c r="C45" s="8" t="s">
+        <v>324</v>
+      </c>
+      <c r="D45" s="12" t="s">
+        <v>323</v>
+      </c>
+      <c r="E45" s="12" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="14" customHeight="1">
+      <c r="A46" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B44" s="1" t="s">
+      <c r="B46" s="1" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="45" spans="1:4" ht="14" customHeight="1">
-      <c r="A45" s="2" t="s">
+      <c r="C46" s="8" t="s">
+        <v>326</v>
+      </c>
+      <c r="D46" s="12" t="s">
+        <v>325</v>
+      </c>
+      <c r="E46" s="12" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="14" customHeight="1">
+      <c r="A47" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B45" s="1" t="s">
+      <c r="B47" s="1" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="46" spans="1:4" ht="14" customHeight="1">
-      <c r="A46" s="2" t="s">
+      <c r="C47" s="8" t="s">
+        <v>328</v>
+      </c>
+      <c r="D47" s="12" t="s">
+        <v>327</v>
+      </c>
+      <c r="E47" s="12" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="14" customHeight="1">
+      <c r="A48" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B46" s="1" t="s">
+      <c r="B48" s="1" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="47" spans="1:4" ht="14" customHeight="1">
-      <c r="A47" s="2" t="s">
+      <c r="C48" s="8" t="s">
+        <v>330</v>
+      </c>
+      <c r="D48" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="E48" s="12" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="14" customHeight="1">
+      <c r="A49" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B47" s="8" t="s">
+      <c r="B49" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="C47" s="9"/>
-      <c r="D47" s="9"/>
-    </row>
-    <row r="48" spans="1:4" ht="14" customHeight="1">
-      <c r="A48" s="2" t="s">
+      <c r="C49" s="8" t="s">
+        <v>366</v>
+      </c>
+      <c r="D49" s="12" t="s">
+        <v>365</v>
+      </c>
+      <c r="E49" s="12" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" ht="14" customHeight="1">
+      <c r="A50" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B48" s="1" t="s">
+      <c r="B50" s="1" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="49" spans="1:4" ht="14" customHeight="1">
-      <c r="A49" s="3" t="s">
+      <c r="C50" s="8" t="s">
+        <v>334</v>
+      </c>
+      <c r="D50" s="12" t="s">
+        <v>333</v>
+      </c>
+      <c r="E50" s="12" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" ht="14" customHeight="1">
+      <c r="A51" s="3" t="s">
         <v>59</v>
-      </c>
-      <c r="B49" s="1" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4">
-      <c r="A50" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="B50" s="1" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4">
-      <c r="A51" s="3" t="s">
-        <v>127</v>
       </c>
       <c r="B51" s="1" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="52" spans="1:4">
+      <c r="C51" s="8" t="s">
+        <v>336</v>
+      </c>
+      <c r="D51" s="12" t="s">
+        <v>335</v>
+      </c>
+      <c r="E51" s="12" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" ht="13.5">
       <c r="A52" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="C52" s="8" t="s">
+        <v>336</v>
+      </c>
+      <c r="D52" s="12" t="s">
+        <v>335</v>
+      </c>
+      <c r="E52" s="12" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" ht="13.5">
+      <c r="A53" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="C53" s="8" t="s">
+        <v>336</v>
+      </c>
+      <c r="D53" s="12" t="s">
+        <v>335</v>
+      </c>
+      <c r="E53" s="12" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" ht="13.5">
+      <c r="A54" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B52" s="1" t="s">
+      <c r="B54" s="1" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="53" spans="1:4" ht="20">
-      <c r="A53" s="3" t="s">
+      <c r="C54" s="8" t="s">
+        <v>332</v>
+      </c>
+      <c r="D54" s="12" t="s">
+        <v>331</v>
+      </c>
+      <c r="E54" s="12" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" ht="13.5">
+      <c r="A55" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="B53" s="1" t="s">
+      <c r="B55" s="1" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="54" spans="1:4">
-      <c r="A54" s="2" t="s">
+      <c r="C55" s="8" t="s">
+        <v>332</v>
+      </c>
+      <c r="D55" s="12" t="s">
+        <v>331</v>
+      </c>
+      <c r="E55" s="12" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" ht="13.5">
+      <c r="A56" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B54" s="1" t="s">
+      <c r="B56" s="1" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="55" spans="1:4" ht="14">
-      <c r="A55" s="2" t="s">
+      <c r="C56" s="8" t="s">
+        <v>338</v>
+      </c>
+      <c r="D56" s="12" t="s">
+        <v>337</v>
+      </c>
+      <c r="E56" s="12" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" ht="13.5">
+      <c r="A57" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B55" s="8" t="s">
+      <c r="B57" s="8" t="s">
         <v>189</v>
       </c>
-      <c r="C55" s="9"/>
-      <c r="D55" s="10"/>
-    </row>
-    <row r="56" spans="1:4">
-      <c r="A56" s="2" t="s">
+      <c r="C57" s="8" t="s">
+        <v>368</v>
+      </c>
+      <c r="D57" s="12" t="s">
+        <v>367</v>
+      </c>
+      <c r="E57" s="12" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" ht="13.5">
+      <c r="A58" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B56" s="1" t="s">
+      <c r="B58" s="1" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="57" spans="1:4">
-      <c r="A57" s="2" t="s">
+      <c r="C58" s="8" t="s">
+        <v>340</v>
+      </c>
+      <c r="D58" s="12" t="s">
+        <v>339</v>
+      </c>
+      <c r="E58" s="12" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" ht="13.5">
+      <c r="A59" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B57" s="1" t="s">
+      <c r="B59" s="1" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="58" spans="1:4">
-      <c r="A58" s="2" t="s">
+      <c r="C59" s="8" t="s">
+        <v>340</v>
+      </c>
+      <c r="D59" s="12" t="s">
+        <v>339</v>
+      </c>
+      <c r="E59" s="12" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" ht="13.5">
+      <c r="A60" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B58" s="1" t="s">
+      <c r="B60" s="1" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="59" spans="1:4">
-      <c r="A59" s="2" t="s">
+      <c r="C60" s="8" t="s">
+        <v>342</v>
+      </c>
+      <c r="D60" s="12" t="s">
+        <v>341</v>
+      </c>
+      <c r="E60" s="12" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" ht="13.5">
+      <c r="A61" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B59" s="1" t="s">
+      <c r="B61" s="1" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="60" spans="1:4">
-      <c r="A60" s="2" t="s">
+      <c r="C61" s="8" t="s">
+        <v>342</v>
+      </c>
+      <c r="D61" s="12" t="s">
+        <v>341</v>
+      </c>
+      <c r="E61" s="12" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" ht="13.5">
+      <c r="A62" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B60" s="1" t="s">
+      <c r="B62" s="1" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="61" spans="1:4" ht="14">
-      <c r="A61" s="7" t="s">
+      <c r="C62" s="8" t="s">
+        <v>344</v>
+      </c>
+      <c r="D62" s="12" t="s">
+        <v>343</v>
+      </c>
+      <c r="E62" s="12" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" ht="13.5">
+      <c r="A63" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="B61" s="1" t="s">
+      <c r="B63" s="1" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="62" spans="1:4">
-      <c r="A62" s="2" t="s">
+      <c r="C63" s="8" t="s">
+        <v>344</v>
+      </c>
+      <c r="D63" s="12" t="s">
+        <v>343</v>
+      </c>
+      <c r="E63" s="12" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" ht="13.5">
+      <c r="A64" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B62" s="1" t="s">
+      <c r="B64" s="1" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="63" spans="1:4">
-      <c r="A63" s="2" t="s">
+      <c r="C64" s="8" t="s">
+        <v>346</v>
+      </c>
+      <c r="D64" s="12" t="s">
+        <v>345</v>
+      </c>
+      <c r="E64" s="12" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" ht="13.5">
+      <c r="A65" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B63" s="1" t="s">
+      <c r="B65" s="1" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="64" spans="1:4">
-      <c r="A64" s="2" t="s">
+      <c r="C65" s="8" t="s">
+        <v>346</v>
+      </c>
+      <c r="D65" s="12" t="s">
+        <v>345</v>
+      </c>
+      <c r="E65" s="12" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" ht="13.5">
+      <c r="A66" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B64" s="1" t="s">
+      <c r="B66" s="1" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="65" spans="1:6">
-      <c r="A65" s="2" t="s">
+      <c r="C66" s="8" t="s">
+        <v>348</v>
+      </c>
+      <c r="D66" s="12" t="s">
+        <v>347</v>
+      </c>
+      <c r="E66" s="12" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" ht="13.5">
+      <c r="A67" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B65" s="1" t="s">
+      <c r="B67" s="1" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="66" spans="1:6">
-      <c r="A66" s="2" t="s">
+      <c r="C67" s="8" t="s">
+        <v>350</v>
+      </c>
+      <c r="D67" s="12" t="s">
+        <v>349</v>
+      </c>
+      <c r="E67" s="12" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" ht="13.5">
+      <c r="A68" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B66" s="1" t="s">
+      <c r="B68" s="1" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="67" spans="1:6">
-      <c r="A67" s="3" t="s">
+      <c r="C68" s="8" t="s">
+        <v>354</v>
+      </c>
+      <c r="D68" s="12" t="s">
+        <v>353</v>
+      </c>
+      <c r="E68" s="12" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" ht="13.5">
+      <c r="A69" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="B67" s="1" t="s">
+      <c r="B69" s="1" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="68" spans="1:6" ht="14">
-      <c r="A68" s="2" t="s">
+      <c r="C69" s="8" t="s">
+        <v>352</v>
+      </c>
+      <c r="D69" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="E69" s="12" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" ht="13.5">
+      <c r="A70" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B68" s="8" t="s">
+      <c r="B70" s="8" t="s">
         <v>190</v>
       </c>
-      <c r="C68" s="9"/>
-      <c r="D68" s="9"/>
-    </row>
-    <row r="77" spans="1:6" ht="14">
-      <c r="B77" s="10"/>
-      <c r="C77" s="10"/>
-      <c r="D77" s="10"/>
-      <c r="E77" s="10"/>
-      <c r="F77" s="10"/>
+      <c r="C70" s="8" t="s">
+        <v>370</v>
+      </c>
+      <c r="D70" s="12" t="s">
+        <v>369</v>
+      </c>
+      <c r="E70" s="12" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" ht="13.5">
+      <c r="B79" s="13"/>
+      <c r="C79" s="13"/>
+      <c r="D79" s="13"/>
+      <c r="E79" s="13"/>
+      <c r="F79" s="9"/>
+      <c r="G79" s="9"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A61" r:id="rId1" xr:uid="{484FCBF9-98EC-5A4C-87E4-AF76A89FDA61}"/>
+    <hyperlink ref="A63" r:id="rId1" xr:uid="{484FCBF9-98EC-5A4C-87E4-AF76A89FDA61}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
add misssing risk free rate data
</commit_message>
<xml_diff>
--- a/epsilon-phi-core/src/resources/templates/MSCI Index Construction.xlsx
+++ b/epsilon-phi-core/src/resources/templates/MSCI Index Construction.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11008"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fabar\repos\epsilon-phi\epsilon-phi-core\src\resources\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/francisbarker/Repositories/Python/epsilon-phi/epsilon-phi-core/src/resources/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A34E9905-6548-44B1-87C6-AC183A1F094D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2019E8AB-7844-644E-A92F-7F5F39E6D646}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13096" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="21800" windowHeight="13100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rules" sheetId="40" r:id="rId1"/>
@@ -926,9 +926,6 @@
     <t>Japan</t>
   </si>
   <si>
-    <t>Korea</t>
-  </si>
-  <si>
     <t>Kuwait</t>
   </si>
   <si>
@@ -989,9 +986,6 @@
     <t>Turkey</t>
   </si>
   <si>
-    <t>UAE</t>
-  </si>
-  <si>
     <t>UK</t>
   </si>
   <si>
@@ -1019,9 +1013,6 @@
     <t>Sri Lanka</t>
   </si>
   <si>
-    <t>Venuzuela</t>
-  </si>
-  <si>
     <t>MSACWF$</t>
   </si>
   <si>
@@ -1563,6 +1554,15 @@
   </si>
   <si>
     <t>Dollar</t>
+  </si>
+  <si>
+    <t>South Korea</t>
+  </si>
+  <si>
+    <t>United Arab Emirates</t>
+  </si>
+  <si>
+    <t>Venezuela</t>
   </si>
 </sst>
 </file>
@@ -2009,16 +2009,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{398A9000-FE9A-0D49-BC15-66DEE1B3B201}">
   <dimension ref="A1:J70"/>
-  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="13.15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.796875" defaultRowHeight="13"/>
   <cols>
-    <col min="1" max="1" width="31.78515625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="21.2109375" style="6" customWidth="1"/>
-    <col min="3" max="10" width="17.78515625" style="6" customWidth="1"/>
+    <col min="1" max="1" width="31.796875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="21.19921875" style="6" customWidth="1"/>
+    <col min="3" max="10" width="17.796875" style="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="11" customFormat="1" ht="19.05" customHeight="1">
+    <row r="1" spans="1:10" s="11" customFormat="1" ht="19" customHeight="1">
       <c r="A1" s="10" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>135</v>
@@ -2048,39 +2048,39 @@
         <v>122</v>
       </c>
     </row>
-    <row r="2" spans="1:10" s="11" customFormat="1" ht="19.05" customHeight="1">
+    <row r="2" spans="1:10" s="11" customFormat="1" ht="19" customHeight="1">
       <c r="A2" s="10" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B2" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="E2" s="4" t="s">
         <v>191</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="F2" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="G2" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="D2" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="E2" s="4" t="s">
+      <c r="H2" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="I2" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="J2" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="H2" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="16.05" customHeight="1">
+    </row>
+    <row r="3" spans="1:10" ht="16" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>0</v>
       </c>
@@ -2112,7 +2112,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="16.05" customHeight="1">
+    <row r="4" spans="1:10" ht="16" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>1</v>
       </c>
@@ -2144,7 +2144,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="16.05" customHeight="1">
+    <row r="5" spans="1:10" ht="16" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>2</v>
       </c>
@@ -2176,7 +2176,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="16.05" customHeight="1">
+    <row r="6" spans="1:10" ht="16" customHeight="1">
       <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
@@ -2208,7 +2208,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="16.05" customHeight="1">
+    <row r="7" spans="1:10" ht="16" customHeight="1">
       <c r="A7" s="2" t="s">
         <v>4</v>
       </c>
@@ -2240,7 +2240,7 @@
         <v>32143</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="16.05" customHeight="1">
+    <row r="8" spans="1:10" ht="16" customHeight="1">
       <c r="A8" s="3" t="s">
         <v>123</v>
       </c>
@@ -2272,7 +2272,7 @@
         <v>32143</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="16.05" customHeight="1">
+    <row r="9" spans="1:10" ht="16" customHeight="1">
       <c r="A9" s="2" t="s">
         <v>5</v>
       </c>
@@ -2304,7 +2304,7 @@
         <v>32143</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="16.05" customHeight="1">
+    <row r="10" spans="1:10" ht="16" customHeight="1">
       <c r="A10" s="2" t="s">
         <v>6</v>
       </c>
@@ -2336,7 +2336,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="16.05" customHeight="1">
+    <row r="11" spans="1:10" ht="16" customHeight="1">
       <c r="A11" s="2" t="s">
         <v>7</v>
       </c>
@@ -2368,7 +2368,7 @@
         <v>34367</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="16.05" customHeight="1">
+    <row r="12" spans="1:10" ht="16" customHeight="1">
       <c r="A12" s="2" t="s">
         <v>8</v>
       </c>
@@ -2400,7 +2400,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="16.05" customHeight="1">
+    <row r="13" spans="1:10" ht="16" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>9</v>
       </c>
@@ -2432,7 +2432,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="16.05" customHeight="1">
+    <row r="14" spans="1:10" ht="16" customHeight="1">
       <c r="A14" s="2" t="s">
         <v>10</v>
       </c>
@@ -2464,7 +2464,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="16.05" customHeight="1">
+    <row r="15" spans="1:10" ht="16" customHeight="1">
       <c r="A15" s="2" t="s">
         <v>11</v>
       </c>
@@ -2496,7 +2496,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="16.05" customHeight="1">
+    <row r="16" spans="1:10" ht="16" customHeight="1">
       <c r="A16" s="2" t="s">
         <v>12</v>
       </c>
@@ -2528,7 +2528,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="16.05" customHeight="1">
+    <row r="17" spans="1:10" ht="16" customHeight="1">
       <c r="A17" s="2" t="s">
         <v>13</v>
       </c>
@@ -2560,7 +2560,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="16.05" customHeight="1">
+    <row r="18" spans="1:10" ht="16" customHeight="1">
       <c r="A18" s="2" t="s">
         <v>14</v>
       </c>
@@ -2592,7 +2592,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="16.05" customHeight="1">
+    <row r="19" spans="1:10" ht="16" customHeight="1">
       <c r="A19" s="2" t="s">
         <v>15</v>
       </c>
@@ -2624,7 +2624,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="16.05" customHeight="1">
+    <row r="20" spans="1:10" ht="16" customHeight="1">
       <c r="A20" s="2" t="s">
         <v>16</v>
       </c>
@@ -2656,7 +2656,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="16.05" customHeight="1">
+    <row r="21" spans="1:10" ht="16" customHeight="1">
       <c r="A21" s="2" t="s">
         <v>17</v>
       </c>
@@ -2688,7 +2688,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="16.05" customHeight="1">
+    <row r="22" spans="1:10" ht="16" customHeight="1">
       <c r="A22" s="2" t="s">
         <v>18</v>
       </c>
@@ -2720,7 +2720,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="16.05" customHeight="1">
+    <row r="23" spans="1:10" ht="16" customHeight="1">
       <c r="A23" s="2" t="s">
         <v>19</v>
       </c>
@@ -2752,7 +2752,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="16.05" customHeight="1">
+    <row r="24" spans="1:10" ht="16" customHeight="1">
       <c r="A24" s="2" t="s">
         <v>20</v>
       </c>
@@ -2784,7 +2784,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="16.05" customHeight="1">
+    <row r="25" spans="1:10" ht="16" customHeight="1">
       <c r="A25" s="3" t="s">
         <v>124</v>
       </c>
@@ -2816,7 +2816,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="16.05" customHeight="1">
+    <row r="26" spans="1:10" ht="16" customHeight="1">
       <c r="A26" s="2" t="s">
         <v>21</v>
       </c>
@@ -2848,7 +2848,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="16.05" customHeight="1">
+    <row r="27" spans="1:10" ht="16" customHeight="1">
       <c r="A27" s="2" t="s">
         <v>22</v>
       </c>
@@ -2880,7 +2880,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="16.05" customHeight="1">
+    <row r="28" spans="1:10" ht="16" customHeight="1">
       <c r="A28" s="2" t="s">
         <v>23</v>
       </c>
@@ -2912,7 +2912,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="16.05" customHeight="1">
+    <row r="29" spans="1:10" ht="16" customHeight="1">
       <c r="A29" s="2" t="s">
         <v>24</v>
       </c>
@@ -2944,7 +2944,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="16.05" customHeight="1">
+    <row r="30" spans="1:10" ht="16" customHeight="1">
       <c r="A30" s="2" t="s">
         <v>25</v>
       </c>
@@ -2976,7 +2976,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="16.05" customHeight="1">
+    <row r="31" spans="1:10" ht="16" customHeight="1">
       <c r="A31" s="3" t="s">
         <v>125</v>
       </c>
@@ -3008,7 +3008,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="16.05" customHeight="1">
+    <row r="32" spans="1:10" ht="16" customHeight="1">
       <c r="A32" s="2" t="s">
         <v>26</v>
       </c>
@@ -3040,7 +3040,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ht="16.05" customHeight="1">
+    <row r="33" spans="1:10" ht="16" customHeight="1">
       <c r="A33" s="2" t="s">
         <v>27</v>
       </c>
@@ -3072,7 +3072,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="16.05" customHeight="1">
+    <row r="34" spans="1:10" ht="16" customHeight="1">
       <c r="A34" s="2" t="s">
         <v>28</v>
       </c>
@@ -3104,7 +3104,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="35" spans="1:10" ht="16.05" customHeight="1">
+    <row r="35" spans="1:10" ht="16" customHeight="1">
       <c r="A35" s="2" t="s">
         <v>29</v>
       </c>
@@ -3136,7 +3136,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="36" spans="1:10" ht="16.05" customHeight="1">
+    <row r="36" spans="1:10" ht="16" customHeight="1">
       <c r="A36" s="2" t="s">
         <v>30</v>
       </c>
@@ -3168,7 +3168,7 @@
         <v>32143</v>
       </c>
     </row>
-    <row r="37" spans="1:10" ht="16.05" customHeight="1">
+    <row r="37" spans="1:10" ht="16" customHeight="1">
       <c r="A37" s="2" t="s">
         <v>31</v>
       </c>
@@ -3200,7 +3200,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="38" spans="1:10" ht="16.05" customHeight="1">
+    <row r="38" spans="1:10" ht="16" customHeight="1">
       <c r="A38" s="2" t="s">
         <v>32</v>
       </c>
@@ -3232,7 +3232,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="39" spans="1:10" ht="16.05" customHeight="1">
+    <row r="39" spans="1:10" ht="16" customHeight="1">
       <c r="A39" s="2" t="s">
         <v>33</v>
       </c>
@@ -3264,7 +3264,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="40" spans="1:10" ht="16.05" customHeight="1">
+    <row r="40" spans="1:10" ht="16" customHeight="1">
       <c r="A40" s="2" t="s">
         <v>34</v>
       </c>
@@ -3296,7 +3296,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="41" spans="1:10" ht="16.05" customHeight="1">
+    <row r="41" spans="1:10" ht="16" customHeight="1">
       <c r="A41" s="2" t="s">
         <v>35</v>
       </c>
@@ -3328,7 +3328,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="42" spans="1:10" ht="16.05" customHeight="1">
+    <row r="42" spans="1:10" ht="16" customHeight="1">
       <c r="A42" s="3" t="s">
         <v>126</v>
       </c>
@@ -3360,7 +3360,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="43" spans="1:10" ht="16.05" customHeight="1">
+    <row r="43" spans="1:10" ht="16" customHeight="1">
       <c r="A43" s="2" t="s">
         <v>36</v>
       </c>
@@ -3392,7 +3392,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="44" spans="1:10" ht="16.05" customHeight="1">
+    <row r="44" spans="1:10" ht="16" customHeight="1">
       <c r="A44" s="2" t="s">
         <v>37</v>
       </c>
@@ -3424,7 +3424,7 @@
         <v>34367</v>
       </c>
     </row>
-    <row r="45" spans="1:10" ht="16.05" customHeight="1">
+    <row r="45" spans="1:10" ht="16" customHeight="1">
       <c r="A45" s="2" t="s">
         <v>38</v>
       </c>
@@ -3456,7 +3456,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="46" spans="1:10" ht="16.05" customHeight="1">
+    <row r="46" spans="1:10" ht="16" customHeight="1">
       <c r="A46" s="2" t="s">
         <v>39</v>
       </c>
@@ -3488,7 +3488,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="47" spans="1:10" ht="16.05" customHeight="1">
+    <row r="47" spans="1:10" ht="16" customHeight="1">
       <c r="A47" s="2" t="s">
         <v>40</v>
       </c>
@@ -3520,7 +3520,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="48" spans="1:10" ht="16.05" customHeight="1">
+    <row r="48" spans="1:10" ht="16" customHeight="1">
       <c r="A48" s="2" t="s">
         <v>41</v>
       </c>
@@ -3552,7 +3552,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="49" spans="1:10" ht="16.05" customHeight="1">
+    <row r="49" spans="1:10" ht="16" customHeight="1">
       <c r="A49" s="2" t="s">
         <v>42</v>
       </c>
@@ -3584,7 +3584,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="50" spans="1:10" ht="16.05" customHeight="1">
+    <row r="50" spans="1:10" ht="16" customHeight="1">
       <c r="A50" s="2" t="s">
         <v>43</v>
       </c>
@@ -3616,7 +3616,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="51" spans="1:10" ht="16.05" customHeight="1">
+    <row r="51" spans="1:10" ht="16" customHeight="1">
       <c r="A51" s="3" t="s">
         <v>59</v>
       </c>
@@ -3648,7 +3648,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="52" spans="1:10" ht="16.05" customHeight="1">
+    <row r="52" spans="1:10" ht="16" customHeight="1">
       <c r="A52" s="2" t="s">
         <v>44</v>
       </c>
@@ -3680,7 +3680,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="53" spans="1:10" ht="16.05" customHeight="1">
+    <row r="53" spans="1:10" ht="16" customHeight="1">
       <c r="A53" s="3" t="s">
         <v>127</v>
       </c>
@@ -3712,7 +3712,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="54" spans="1:10" ht="16.05" customHeight="1">
+    <row r="54" spans="1:10" ht="16" customHeight="1">
       <c r="A54" s="2" t="s">
         <v>45</v>
       </c>
@@ -3744,7 +3744,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="55" spans="1:10" ht="16.05" customHeight="1">
+    <row r="55" spans="1:10" ht="16" customHeight="1">
       <c r="A55" s="3" t="s">
         <v>128</v>
       </c>
@@ -3776,7 +3776,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="56" spans="1:10" ht="16.05" customHeight="1">
+    <row r="56" spans="1:10" ht="16" customHeight="1">
       <c r="A56" s="2" t="s">
         <v>46</v>
       </c>
@@ -3808,7 +3808,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="57" spans="1:10" ht="16.05" customHeight="1">
+    <row r="57" spans="1:10" ht="16" customHeight="1">
       <c r="A57" s="2" t="s">
         <v>47</v>
       </c>
@@ -3840,7 +3840,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="58" spans="1:10" ht="16.05" customHeight="1">
+    <row r="58" spans="1:10" ht="16" customHeight="1">
       <c r="A58" s="2" t="s">
         <v>48</v>
       </c>
@@ -3872,7 +3872,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="59" spans="1:10" ht="16.05" customHeight="1">
+    <row r="59" spans="1:10" ht="16" customHeight="1">
       <c r="A59" s="2" t="s">
         <v>49</v>
       </c>
@@ -3904,7 +3904,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="60" spans="1:10" ht="16.05" customHeight="1">
+    <row r="60" spans="1:10" ht="16" customHeight="1">
       <c r="A60" s="2" t="s">
         <v>50</v>
       </c>
@@ -3936,7 +3936,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="61" spans="1:10" ht="16.05" customHeight="1">
+    <row r="61" spans="1:10" ht="16" customHeight="1">
       <c r="A61" s="2" t="s">
         <v>51</v>
       </c>
@@ -3968,7 +3968,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="62" spans="1:10" ht="16.05" customHeight="1">
+    <row r="62" spans="1:10" ht="16" customHeight="1">
       <c r="A62" s="2" t="s">
         <v>52</v>
       </c>
@@ -4000,7 +4000,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="63" spans="1:10" ht="16.05" customHeight="1">
+    <row r="63" spans="1:10" ht="16" customHeight="1">
       <c r="A63" s="7" t="s">
         <v>129</v>
       </c>
@@ -4032,7 +4032,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="64" spans="1:10" ht="16.05" customHeight="1">
+    <row r="64" spans="1:10" ht="16" customHeight="1">
       <c r="A64" s="2" t="s">
         <v>53</v>
       </c>
@@ -4064,7 +4064,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="65" spans="1:10" ht="16.05" customHeight="1">
+    <row r="65" spans="1:10" ht="16" customHeight="1">
       <c r="A65" s="2" t="s">
         <v>54</v>
       </c>
@@ -4096,7 +4096,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="66" spans="1:10" ht="16.05" customHeight="1">
+    <row r="66" spans="1:10" ht="16" customHeight="1">
       <c r="A66" s="2" t="s">
         <v>55</v>
       </c>
@@ -4128,7 +4128,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="67" spans="1:10" ht="16.05" customHeight="1">
+    <row r="67" spans="1:10" ht="16" customHeight="1">
       <c r="A67" s="2" t="s">
         <v>56</v>
       </c>
@@ -4160,7 +4160,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="68" spans="1:10" ht="16.05" customHeight="1">
+    <row r="68" spans="1:10" ht="16" customHeight="1">
       <c r="A68" s="2" t="s">
         <v>57</v>
       </c>
@@ -4192,7 +4192,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="69" spans="1:10" ht="16.05" customHeight="1">
+    <row r="69" spans="1:10" ht="16" customHeight="1">
       <c r="A69" s="3" t="s">
         <v>130</v>
       </c>
@@ -4224,7 +4224,7 @@
         <v>32143</v>
       </c>
     </row>
-    <row r="70" spans="1:10" ht="16.05" customHeight="1">
+    <row r="70" spans="1:10" ht="16" customHeight="1">
       <c r="A70" s="2" t="s">
         <v>58</v>
       </c>
@@ -4267,28 +4267,28 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A7EF705-CFED-174D-8EBB-657B7E248B5D}">
   <dimension ref="A2:G79"/>
-  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="13.15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.796875" defaultRowHeight="13"/>
   <cols>
-    <col min="1" max="1" width="19.42578125" customWidth="1"/>
-    <col min="2" max="2" width="29.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="11.5" style="1" customWidth="1"/>
+    <col min="1" max="1" width="19.3984375" customWidth="1"/>
+    <col min="2" max="2" width="29.3984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="11.3984375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:5">
       <c r="A2" s="1" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="14" customHeight="1">
@@ -4296,16 +4296,16 @@
         <v>0</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="14" customHeight="1">
@@ -4316,13 +4316,13 @@
         <v>136</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="14" customHeight="1">
@@ -4333,13 +4333,13 @@
         <v>137</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="14" customHeight="1">
@@ -4350,13 +4350,13 @@
         <v>138</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="14" customHeight="1">
@@ -4367,13 +4367,13 @@
         <v>139</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="14" customHeight="1">
@@ -4384,13 +4384,13 @@
         <v>140</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="14" customHeight="1">
@@ -4401,13 +4401,13 @@
         <v>141</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="14" customHeight="1">
@@ -4418,13 +4418,13 @@
         <v>142</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="14" customHeight="1">
@@ -4435,13 +4435,13 @@
         <v>143</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="14" customHeight="1">
@@ -4452,13 +4452,13 @@
         <v>144</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="14" customHeight="1">
@@ -4469,13 +4469,13 @@
         <v>145</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="14" customHeight="1">
@@ -4486,13 +4486,13 @@
         <v>146</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="14" customHeight="1">
@@ -4503,13 +4503,13 @@
         <v>147</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="D15" s="12" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="14" customHeight="1">
@@ -4520,13 +4520,13 @@
         <v>147</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="14" customHeight="1">
@@ -4537,13 +4537,13 @@
         <v>148</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="14" customHeight="1">
@@ -4554,13 +4554,13 @@
         <v>149</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="14" customHeight="1">
@@ -4571,13 +4571,13 @@
         <v>150</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="E19" s="12" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="14" customHeight="1">
@@ -4588,13 +4588,13 @@
         <v>151</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="E20" s="12" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="14" customHeight="1">
@@ -4605,13 +4605,13 @@
         <v>152</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="E21" s="12" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="14" customHeight="1">
@@ -4622,13 +4622,13 @@
         <v>153</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="E22" s="12" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="14" customHeight="1">
@@ -4639,13 +4639,13 @@
         <v>154</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="D23" s="12" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="E23" s="12" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="14" customHeight="1">
@@ -4656,13 +4656,13 @@
         <v>154</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="E24" s="12" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="14" customHeight="1">
@@ -4673,13 +4673,13 @@
         <v>155</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="E25" s="12" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="14" customHeight="1">
@@ -4690,13 +4690,13 @@
         <v>156</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="E26" s="12" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="14" customHeight="1">
@@ -4707,13 +4707,13 @@
         <v>157</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="D27" s="12" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="E27" s="12" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="14" customHeight="1">
@@ -4724,13 +4724,13 @@
         <v>158</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="E28" s="12" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="14" customHeight="1">
@@ -4738,50 +4738,50 @@
         <v>24</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="E29" s="12" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="14" customHeight="1">
       <c r="A30" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B30" s="1" t="s">
-        <v>159</v>
+      <c r="B30" s="8" t="s">
+        <v>369</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="E30" s="12" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="14" customHeight="1">
       <c r="A31" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="B31" s="1" t="s">
-        <v>159</v>
+      <c r="B31" s="8" t="s">
+        <v>369</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="E31" s="12" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="14" customHeight="1">
@@ -4789,16 +4789,16 @@
         <v>26</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="D32" s="12" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="E32" s="12" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="14" customHeight="1">
@@ -4806,16 +4806,16 @@
         <v>27</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="E33" s="12" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="14" customHeight="1">
@@ -4823,16 +4823,16 @@
         <v>28</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="D34" s="12" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="E34" s="12" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="14" customHeight="1">
@@ -4840,16 +4840,16 @@
         <v>29</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="D35" s="12" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="E35" s="12" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="14" customHeight="1">
@@ -4857,16 +4857,16 @@
         <v>30</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="D36" s="12" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="E36" s="12" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="14" customHeight="1">
@@ -4874,16 +4874,16 @@
         <v>31</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="D37" s="12" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="E37" s="12" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="14" customHeight="1">
@@ -4891,16 +4891,16 @@
         <v>32</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="D38" s="12" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="E38" s="12" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="14" customHeight="1">
@@ -4908,16 +4908,16 @@
         <v>33</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="E39" s="12" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="14" customHeight="1">
@@ -4925,16 +4925,16 @@
         <v>34</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="D40" s="12" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="E40" s="12" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="14" customHeight="1">
@@ -4942,16 +4942,16 @@
         <v>35</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="D41" s="12" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="E41" s="12" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="14" customHeight="1">
@@ -4959,16 +4959,16 @@
         <v>126</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="D42" s="12" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="E42" s="12" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="14" customHeight="1">
@@ -4976,16 +4976,16 @@
         <v>36</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="E43" s="12" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="14" customHeight="1">
@@ -4993,16 +4993,16 @@
         <v>37</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C44" s="8" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="D44" s="12" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="E44" s="12" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="14" customHeight="1">
@@ -5010,16 +5010,16 @@
         <v>38</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C45" s="8" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="D45" s="12" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="E45" s="12" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="14" customHeight="1">
@@ -5027,16 +5027,16 @@
         <v>39</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C46" s="8" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="D46" s="12" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="E46" s="12" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="14" customHeight="1">
@@ -5044,16 +5044,16 @@
         <v>40</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C47" s="8" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="D47" s="12" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="E47" s="12" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
     </row>
     <row r="48" spans="1:5" ht="14" customHeight="1">
@@ -5061,16 +5061,16 @@
         <v>41</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C48" s="8" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="D48" s="12" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="E48" s="12" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
     </row>
     <row r="49" spans="1:5" ht="14" customHeight="1">
@@ -5078,16 +5078,16 @@
         <v>42</v>
       </c>
       <c r="B49" s="8" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C49" s="8" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="D49" s="12" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="E49" s="12" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
     </row>
     <row r="50" spans="1:5" ht="14" customHeight="1">
@@ -5095,16 +5095,16 @@
         <v>43</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C50" s="8" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="D50" s="12" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="E50" s="12" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
     </row>
     <row r="51" spans="1:5" ht="14" customHeight="1">
@@ -5112,342 +5112,342 @@
         <v>59</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C51" s="8" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="D51" s="12" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="E51" s="12" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" ht="13.5">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" ht="14">
       <c r="A52" s="2" t="s">
         <v>44</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C52" s="8" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="D52" s="12" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="E52" s="12" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" ht="13.5">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" ht="14">
       <c r="A53" s="3" t="s">
         <v>127</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C53" s="8" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="D53" s="12" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="E53" s="12" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" ht="13.5">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" ht="14">
       <c r="A54" s="2" t="s">
         <v>45</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C54" s="8" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="D54" s="12" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="E54" s="12" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" ht="13.5">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" ht="20">
       <c r="A55" s="3" t="s">
         <v>128</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C55" s="8" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="D55" s="12" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="E55" s="12" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" ht="13.5">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" ht="14">
       <c r="A56" s="2" t="s">
         <v>46</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C56" s="8" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="D56" s="12" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="E56" s="12" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" ht="13.5">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" ht="14">
       <c r="A57" s="2" t="s">
         <v>47</v>
       </c>
       <c r="B57" s="8" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C57" s="8" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="D57" s="12" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="E57" s="12" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" ht="13.5">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" ht="14">
       <c r="A58" s="2" t="s">
         <v>48</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C58" s="8" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="D58" s="12" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="E58" s="12" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" ht="13.5">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" ht="14">
       <c r="A59" s="2" t="s">
         <v>49</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C59" s="8" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="D59" s="12" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="E59" s="12" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" ht="13.5">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" ht="14">
       <c r="A60" s="2" t="s">
         <v>50</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C60" s="8" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="D60" s="12" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="E60" s="12" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" ht="13.5">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" ht="14">
       <c r="A61" s="2" t="s">
         <v>51</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C61" s="8" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="D61" s="12" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="E61" s="12" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" ht="13.5">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" ht="14">
       <c r="A62" s="2" t="s">
         <v>52</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C62" s="8" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="D62" s="12" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="E62" s="12" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" ht="13.5">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" ht="14">
       <c r="A63" s="7" t="s">
         <v>129</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C63" s="8" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="D63" s="12" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="E63" s="12" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" ht="13.5">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" ht="14">
       <c r="A64" s="2" t="s">
         <v>53</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C64" s="8" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="D64" s="12" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="E64" s="12" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="65" spans="1:7" ht="13.5">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" ht="14">
       <c r="A65" s="2" t="s">
         <v>54</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C65" s="8" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="D65" s="12" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="E65" s="12" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" ht="13.5">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" ht="14">
       <c r="A66" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C66" s="8" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="D66" s="12" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="E66" s="12" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7" ht="13.5">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" ht="14">
       <c r="A67" s="2" t="s">
         <v>56</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>180</v>
+        <v>370</v>
       </c>
       <c r="C67" s="8" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="D67" s="12" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="E67" s="12" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7" ht="13.5">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" ht="14">
       <c r="A68" s="2" t="s">
         <v>57</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C68" s="8" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="D68" s="12" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="E68" s="12" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7" ht="13.5">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" ht="14">
       <c r="A69" s="3" t="s">
         <v>130</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C69" s="8" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="D69" s="12" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="E69" s="12" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="70" spans="1:7" ht="13.5">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" ht="14">
       <c r="A70" s="2" t="s">
         <v>58</v>
       </c>
       <c r="B70" s="8" t="s">
-        <v>190</v>
+        <v>371</v>
       </c>
       <c r="C70" s="8" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="D70" s="12" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="E70" s="12" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="79" spans="1:7" ht="13.5">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" ht="14">
       <c r="B79" s="13"/>
       <c r="C79" s="13"/>
       <c r="D79" s="13"/>

</xml_diff>

<commit_message>
USD Risk Free Modelling (1 Month T Bills)
</commit_message>
<xml_diff>
--- a/epsilon-phi-core/src/resources/templates/MSCI Index Construction.xlsx
+++ b/epsilon-phi-core/src/resources/templates/MSCI Index Construction.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11008"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fabar\repos\epsilon-phi\epsilon-phi-core\src\resources\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/francisbarker/Repositories/Python/epsilon-phi/epsilon-phi-core/src/resources/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E348198-5A1D-40AB-AA33-037AC7E737C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46C1AFA0-D28B-6E49-A27D-D4C8E7F63DE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13096" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="21800" windowHeight="13100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rules" sheetId="40" r:id="rId1"/>
@@ -2009,14 +2009,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{398A9000-FE9A-0D49-BC15-66DEE1B3B201}">
   <dimension ref="A1:J70"/>
-  <sheetFormatPr defaultColWidth="10.78515625" defaultRowHeight="13.15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.796875" defaultRowHeight="13"/>
   <cols>
-    <col min="1" max="1" width="31.78515625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="21.2109375" style="6" customWidth="1"/>
-    <col min="3" max="10" width="17.78515625" style="6" customWidth="1"/>
+    <col min="1" max="1" width="31.796875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="21.19921875" style="6" customWidth="1"/>
+    <col min="3" max="10" width="17.796875" style="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="11" customFormat="1" ht="19.05" customHeight="1">
+    <row r="1" spans="1:10" s="11" customFormat="1" ht="19" customHeight="1">
       <c r="A1" s="10" t="s">
         <v>195</v>
       </c>
@@ -2048,7 +2048,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="2" spans="1:10" s="11" customFormat="1" ht="19.05" customHeight="1">
+    <row r="2" spans="1:10" s="11" customFormat="1" ht="19" customHeight="1">
       <c r="A2" s="10" t="s">
         <v>196</v>
       </c>
@@ -2080,7 +2080,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="16.05" customHeight="1">
+    <row r="3" spans="1:10" ht="16" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>0</v>
       </c>
@@ -2112,7 +2112,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="16.05" customHeight="1">
+    <row r="4" spans="1:10" ht="16" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>1</v>
       </c>
@@ -2144,7 +2144,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="16.05" customHeight="1">
+    <row r="5" spans="1:10" ht="16" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>2</v>
       </c>
@@ -2176,7 +2176,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="16.05" customHeight="1">
+    <row r="6" spans="1:10" ht="16" customHeight="1">
       <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
@@ -2208,7 +2208,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="16.05" customHeight="1">
+    <row r="7" spans="1:10" ht="16" customHeight="1">
       <c r="A7" s="2" t="s">
         <v>4</v>
       </c>
@@ -2240,7 +2240,7 @@
         <v>32143</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="16.05" customHeight="1">
+    <row r="8" spans="1:10" ht="16" customHeight="1">
       <c r="A8" s="3" t="s">
         <v>123</v>
       </c>
@@ -2272,7 +2272,7 @@
         <v>32143</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="16.05" customHeight="1">
+    <row r="9" spans="1:10" ht="16" customHeight="1">
       <c r="A9" s="2" t="s">
         <v>5</v>
       </c>
@@ -2304,7 +2304,7 @@
         <v>32143</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="16.05" customHeight="1">
+    <row r="10" spans="1:10" ht="16" customHeight="1">
       <c r="A10" s="2" t="s">
         <v>6</v>
       </c>
@@ -2336,7 +2336,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="16.05" customHeight="1">
+    <row r="11" spans="1:10" ht="16" customHeight="1">
       <c r="A11" s="2" t="s">
         <v>7</v>
       </c>
@@ -2368,7 +2368,7 @@
         <v>34367</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="16.05" customHeight="1">
+    <row r="12" spans="1:10" ht="16" customHeight="1">
       <c r="A12" s="2" t="s">
         <v>8</v>
       </c>
@@ -2400,7 +2400,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="16.05" customHeight="1">
+    <row r="13" spans="1:10" ht="16" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>9</v>
       </c>
@@ -2432,7 +2432,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="16.05" customHeight="1">
+    <row r="14" spans="1:10" ht="16" customHeight="1">
       <c r="A14" s="2" t="s">
         <v>10</v>
       </c>
@@ -2464,7 +2464,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="16.05" customHeight="1">
+    <row r="15" spans="1:10" ht="16" customHeight="1">
       <c r="A15" s="2" t="s">
         <v>11</v>
       </c>
@@ -2496,7 +2496,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="16.05" customHeight="1">
+    <row r="16" spans="1:10" ht="16" customHeight="1">
       <c r="A16" s="2" t="s">
         <v>12</v>
       </c>
@@ -2528,7 +2528,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="16.05" customHeight="1">
+    <row r="17" spans="1:10" ht="16" customHeight="1">
       <c r="A17" s="2" t="s">
         <v>13</v>
       </c>
@@ -2560,7 +2560,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="16.05" customHeight="1">
+    <row r="18" spans="1:10" ht="16" customHeight="1">
       <c r="A18" s="2" t="s">
         <v>14</v>
       </c>
@@ -2592,7 +2592,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="16.05" customHeight="1">
+    <row r="19" spans="1:10" ht="16" customHeight="1">
       <c r="A19" s="2" t="s">
         <v>15</v>
       </c>
@@ -2624,7 +2624,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="16.05" customHeight="1">
+    <row r="20" spans="1:10" ht="16" customHeight="1">
       <c r="A20" s="2" t="s">
         <v>16</v>
       </c>
@@ -2656,7 +2656,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="16.05" customHeight="1">
+    <row r="21" spans="1:10" ht="16" customHeight="1">
       <c r="A21" s="2" t="s">
         <v>17</v>
       </c>
@@ -2688,7 +2688,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="16.05" customHeight="1">
+    <row r="22" spans="1:10" ht="16" customHeight="1">
       <c r="A22" s="2" t="s">
         <v>18</v>
       </c>
@@ -2720,7 +2720,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="16.05" customHeight="1">
+    <row r="23" spans="1:10" ht="16" customHeight="1">
       <c r="A23" s="2" t="s">
         <v>19</v>
       </c>
@@ -2752,7 +2752,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="16.05" customHeight="1">
+    <row r="24" spans="1:10" ht="16" customHeight="1">
       <c r="A24" s="2" t="s">
         <v>20</v>
       </c>
@@ -2784,7 +2784,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="16.05" customHeight="1">
+    <row r="25" spans="1:10" ht="16" customHeight="1">
       <c r="A25" s="3" t="s">
         <v>124</v>
       </c>
@@ -2816,7 +2816,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="16.05" customHeight="1">
+    <row r="26" spans="1:10" ht="16" customHeight="1">
       <c r="A26" s="2" t="s">
         <v>21</v>
       </c>
@@ -2848,7 +2848,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="16.05" customHeight="1">
+    <row r="27" spans="1:10" ht="16" customHeight="1">
       <c r="A27" s="2" t="s">
         <v>22</v>
       </c>
@@ -2880,7 +2880,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="16.05" customHeight="1">
+    <row r="28" spans="1:10" ht="16" customHeight="1">
       <c r="A28" s="2" t="s">
         <v>23</v>
       </c>
@@ -2912,7 +2912,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="16.05" customHeight="1">
+    <row r="29" spans="1:10" ht="16" customHeight="1">
       <c r="A29" s="2" t="s">
         <v>24</v>
       </c>
@@ -2944,7 +2944,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="16.05" customHeight="1">
+    <row r="30" spans="1:10" ht="16" customHeight="1">
       <c r="A30" s="2" t="s">
         <v>25</v>
       </c>
@@ -2976,7 +2976,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="16.05" customHeight="1">
+    <row r="31" spans="1:10" ht="16" customHeight="1">
       <c r="A31" s="3" t="s">
         <v>125</v>
       </c>
@@ -3008,7 +3008,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="16.05" customHeight="1">
+    <row r="32" spans="1:10" ht="16" customHeight="1">
       <c r="A32" s="2" t="s">
         <v>26</v>
       </c>
@@ -3040,7 +3040,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ht="16.05" customHeight="1">
+    <row r="33" spans="1:10" ht="16" customHeight="1">
       <c r="A33" s="2" t="s">
         <v>27</v>
       </c>
@@ -3072,7 +3072,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="16.05" customHeight="1">
+    <row r="34" spans="1:10" ht="16" customHeight="1">
       <c r="A34" s="2" t="s">
         <v>28</v>
       </c>
@@ -3104,7 +3104,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="35" spans="1:10" ht="16.05" customHeight="1">
+    <row r="35" spans="1:10" ht="16" customHeight="1">
       <c r="A35" s="2" t="s">
         <v>29</v>
       </c>
@@ -3136,7 +3136,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="36" spans="1:10" ht="16.05" customHeight="1">
+    <row r="36" spans="1:10" ht="16" customHeight="1">
       <c r="A36" s="2" t="s">
         <v>30</v>
       </c>
@@ -3168,7 +3168,7 @@
         <v>32143</v>
       </c>
     </row>
-    <row r="37" spans="1:10" ht="16.05" customHeight="1">
+    <row r="37" spans="1:10" ht="16" customHeight="1">
       <c r="A37" s="2" t="s">
         <v>31</v>
       </c>
@@ -3200,7 +3200,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="38" spans="1:10" ht="16.05" customHeight="1">
+    <row r="38" spans="1:10" ht="16" customHeight="1">
       <c r="A38" s="2" t="s">
         <v>32</v>
       </c>
@@ -3232,7 +3232,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="39" spans="1:10" ht="16.05" customHeight="1">
+    <row r="39" spans="1:10" ht="16" customHeight="1">
       <c r="A39" s="2" t="s">
         <v>33</v>
       </c>
@@ -3264,7 +3264,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="40" spans="1:10" ht="16.05" customHeight="1">
+    <row r="40" spans="1:10" ht="16" customHeight="1">
       <c r="A40" s="2" t="s">
         <v>34</v>
       </c>
@@ -3296,7 +3296,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="41" spans="1:10" ht="16.05" customHeight="1">
+    <row r="41" spans="1:10" ht="16" customHeight="1">
       <c r="A41" s="2" t="s">
         <v>35</v>
       </c>
@@ -3328,7 +3328,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="42" spans="1:10" ht="16.05" customHeight="1">
+    <row r="42" spans="1:10" ht="16" customHeight="1">
       <c r="A42" s="3" t="s">
         <v>126</v>
       </c>
@@ -3360,7 +3360,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="43" spans="1:10" ht="16.05" customHeight="1">
+    <row r="43" spans="1:10" ht="16" customHeight="1">
       <c r="A43" s="2" t="s">
         <v>36</v>
       </c>
@@ -3392,7 +3392,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="44" spans="1:10" ht="16.05" customHeight="1">
+    <row r="44" spans="1:10" ht="16" customHeight="1">
       <c r="A44" s="2" t="s">
         <v>37</v>
       </c>
@@ -3424,7 +3424,7 @@
         <v>34367</v>
       </c>
     </row>
-    <row r="45" spans="1:10" ht="16.05" customHeight="1">
+    <row r="45" spans="1:10" ht="16" customHeight="1">
       <c r="A45" s="2" t="s">
         <v>38</v>
       </c>
@@ -3456,7 +3456,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="46" spans="1:10" ht="16.05" customHeight="1">
+    <row r="46" spans="1:10" ht="16" customHeight="1">
       <c r="A46" s="2" t="s">
         <v>39</v>
       </c>
@@ -3488,7 +3488,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="47" spans="1:10" ht="16.05" customHeight="1">
+    <row r="47" spans="1:10" ht="16" customHeight="1">
       <c r="A47" s="2" t="s">
         <v>40</v>
       </c>
@@ -3520,7 +3520,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="48" spans="1:10" ht="16.05" customHeight="1">
+    <row r="48" spans="1:10" ht="16" customHeight="1">
       <c r="A48" s="2" t="s">
         <v>41</v>
       </c>
@@ -3552,7 +3552,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="49" spans="1:10" ht="16.05" customHeight="1">
+    <row r="49" spans="1:10" ht="16" customHeight="1">
       <c r="A49" s="2" t="s">
         <v>42</v>
       </c>
@@ -3584,7 +3584,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="50" spans="1:10" ht="16.05" customHeight="1">
+    <row r="50" spans="1:10" ht="16" customHeight="1">
       <c r="A50" s="2" t="s">
         <v>43</v>
       </c>
@@ -3616,7 +3616,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="51" spans="1:10" ht="16.05" customHeight="1">
+    <row r="51" spans="1:10" ht="16" customHeight="1">
       <c r="A51" s="3" t="s">
         <v>59</v>
       </c>
@@ -3648,7 +3648,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="52" spans="1:10" ht="16.05" customHeight="1">
+    <row r="52" spans="1:10" ht="16" customHeight="1">
       <c r="A52" s="2" t="s">
         <v>44</v>
       </c>
@@ -3680,7 +3680,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="53" spans="1:10" ht="16.05" customHeight="1">
+    <row r="53" spans="1:10" ht="16" customHeight="1">
       <c r="A53" s="3" t="s">
         <v>127</v>
       </c>
@@ -3712,7 +3712,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="54" spans="1:10" ht="16.05" customHeight="1">
+    <row r="54" spans="1:10" ht="16" customHeight="1">
       <c r="A54" s="2" t="s">
         <v>45</v>
       </c>
@@ -3744,7 +3744,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="55" spans="1:10" ht="16.05" customHeight="1">
+    <row r="55" spans="1:10" ht="16" customHeight="1">
       <c r="A55" s="3" t="s">
         <v>128</v>
       </c>
@@ -3776,7 +3776,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="56" spans="1:10" ht="16.05" customHeight="1">
+    <row r="56" spans="1:10" ht="16" customHeight="1">
       <c r="A56" s="2" t="s">
         <v>46</v>
       </c>
@@ -3808,7 +3808,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="57" spans="1:10" ht="16.05" customHeight="1">
+    <row r="57" spans="1:10" ht="16" customHeight="1">
       <c r="A57" s="2" t="s">
         <v>47</v>
       </c>
@@ -3840,7 +3840,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="58" spans="1:10" ht="16.05" customHeight="1">
+    <row r="58" spans="1:10" ht="16" customHeight="1">
       <c r="A58" s="2" t="s">
         <v>48</v>
       </c>
@@ -3872,7 +3872,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="59" spans="1:10" ht="16.05" customHeight="1">
+    <row r="59" spans="1:10" ht="16" customHeight="1">
       <c r="A59" s="2" t="s">
         <v>49</v>
       </c>
@@ -3904,7 +3904,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="60" spans="1:10" ht="16.05" customHeight="1">
+    <row r="60" spans="1:10" ht="16" customHeight="1">
       <c r="A60" s="2" t="s">
         <v>50</v>
       </c>
@@ -3936,7 +3936,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="61" spans="1:10" ht="16.05" customHeight="1">
+    <row r="61" spans="1:10" ht="16" customHeight="1">
       <c r="A61" s="2" t="s">
         <v>51</v>
       </c>
@@ -3968,7 +3968,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="62" spans="1:10" ht="16.05" customHeight="1">
+    <row r="62" spans="1:10" ht="16" customHeight="1">
       <c r="A62" s="2" t="s">
         <v>52</v>
       </c>
@@ -4000,7 +4000,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="63" spans="1:10" ht="16.05" customHeight="1">
+    <row r="63" spans="1:10" ht="16" customHeight="1">
       <c r="A63" s="7" t="s">
         <v>129</v>
       </c>
@@ -4032,7 +4032,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="64" spans="1:10" ht="16.05" customHeight="1">
+    <row r="64" spans="1:10" ht="16" customHeight="1">
       <c r="A64" s="2" t="s">
         <v>53</v>
       </c>
@@ -4064,7 +4064,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="65" spans="1:10" ht="16.05" customHeight="1">
+    <row r="65" spans="1:10" ht="16" customHeight="1">
       <c r="A65" s="2" t="s">
         <v>54</v>
       </c>
@@ -4096,7 +4096,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="66" spans="1:10" ht="16.05" customHeight="1">
+    <row r="66" spans="1:10" ht="16" customHeight="1">
       <c r="A66" s="2" t="s">
         <v>55</v>
       </c>
@@ -4128,7 +4128,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="67" spans="1:10" ht="16.05" customHeight="1">
+    <row r="67" spans="1:10" ht="16" customHeight="1">
       <c r="A67" s="2" t="s">
         <v>56</v>
       </c>
@@ -4160,7 +4160,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="68" spans="1:10" ht="16.05" customHeight="1">
+    <row r="68" spans="1:10" ht="16" customHeight="1">
       <c r="A68" s="2" t="s">
         <v>57</v>
       </c>
@@ -4192,7 +4192,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="69" spans="1:10" ht="16.05" customHeight="1">
+    <row r="69" spans="1:10" ht="16" customHeight="1">
       <c r="A69" s="3" t="s">
         <v>130</v>
       </c>
@@ -4224,7 +4224,7 @@
         <v>32143</v>
       </c>
     </row>
-    <row r="70" spans="1:10" ht="16.05" customHeight="1">
+    <row r="70" spans="1:10" ht="16" customHeight="1">
       <c r="A70" s="2" t="s">
         <v>58</v>
       </c>
@@ -4267,11 +4267,11 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A7EF705-CFED-174D-8EBB-657B7E248B5D}">
   <dimension ref="A2:G79"/>
-  <sheetFormatPr defaultColWidth="10.78515625" defaultRowHeight="13.15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.796875" defaultRowHeight="13"/>
   <cols>
-    <col min="1" max="1" width="19.42578125" customWidth="1"/>
-    <col min="2" max="2" width="29.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="11.42578125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="19.3984375" customWidth="1"/>
+    <col min="2" max="2" width="29.3984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="11.3984375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:5">
@@ -5124,7 +5124,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="52" spans="1:5" ht="13.5">
+    <row r="52" spans="1:5" ht="14">
       <c r="A52" s="2" t="s">
         <v>44</v>
       </c>
@@ -5141,7 +5141,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="53" spans="1:5" ht="13.5">
+    <row r="53" spans="1:5" ht="14">
       <c r="A53" s="3" t="s">
         <v>127</v>
       </c>
@@ -5158,7 +5158,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="54" spans="1:5" ht="13.5">
+    <row r="54" spans="1:5" ht="14">
       <c r="A54" s="2" t="s">
         <v>45</v>
       </c>
@@ -5175,7 +5175,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="55" spans="1:5" ht="13.5">
+    <row r="55" spans="1:5" ht="20">
       <c r="A55" s="3" t="s">
         <v>128</v>
       </c>
@@ -5192,7 +5192,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="56" spans="1:5" ht="13.5">
+    <row r="56" spans="1:5" ht="14">
       <c r="A56" s="2" t="s">
         <v>46</v>
       </c>
@@ -5209,7 +5209,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="57" spans="1:5" ht="13.5">
+    <row r="57" spans="1:5" ht="14">
       <c r="A57" s="2" t="s">
         <v>47</v>
       </c>
@@ -5226,7 +5226,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="58" spans="1:5" ht="13.5">
+    <row r="58" spans="1:5" ht="14">
       <c r="A58" s="2" t="s">
         <v>48</v>
       </c>
@@ -5243,7 +5243,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="59" spans="1:5" ht="13.5">
+    <row r="59" spans="1:5" ht="14">
       <c r="A59" s="2" t="s">
         <v>49</v>
       </c>
@@ -5260,7 +5260,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="60" spans="1:5" ht="13.5">
+    <row r="60" spans="1:5" ht="14">
       <c r="A60" s="2" t="s">
         <v>50</v>
       </c>
@@ -5277,7 +5277,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="61" spans="1:5" ht="13.5">
+    <row r="61" spans="1:5" ht="14">
       <c r="A61" s="2" t="s">
         <v>51</v>
       </c>
@@ -5294,7 +5294,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="62" spans="1:5" ht="13.5">
+    <row r="62" spans="1:5" ht="14">
       <c r="A62" s="2" t="s">
         <v>52</v>
       </c>
@@ -5311,7 +5311,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="63" spans="1:5" ht="13.5">
+    <row r="63" spans="1:5" ht="14">
       <c r="A63" s="7" t="s">
         <v>129</v>
       </c>
@@ -5328,7 +5328,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="64" spans="1:5" ht="13.5">
+    <row r="64" spans="1:5" ht="14">
       <c r="A64" s="2" t="s">
         <v>53</v>
       </c>
@@ -5345,7 +5345,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="65" spans="1:7" ht="13.5">
+    <row r="65" spans="1:7" ht="14">
       <c r="A65" s="2" t="s">
         <v>54</v>
       </c>
@@ -5362,7 +5362,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="66" spans="1:7" ht="13.5">
+    <row r="66" spans="1:7" ht="14">
       <c r="A66" s="2" t="s">
         <v>55</v>
       </c>
@@ -5379,7 +5379,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="67" spans="1:7" ht="13.5">
+    <row r="67" spans="1:7" ht="14">
       <c r="A67" s="2" t="s">
         <v>56</v>
       </c>
@@ -5396,7 +5396,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="68" spans="1:7" ht="13.5">
+    <row r="68" spans="1:7" ht="14">
       <c r="A68" s="2" t="s">
         <v>57</v>
       </c>
@@ -5413,7 +5413,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="69" spans="1:7" ht="13.5">
+    <row r="69" spans="1:7" ht="14">
       <c r="A69" s="3" t="s">
         <v>130</v>
       </c>
@@ -5430,7 +5430,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="70" spans="1:7" ht="13.5">
+    <row r="70" spans="1:7" ht="14">
       <c r="A70" s="2" t="s">
         <v>58</v>
       </c>
@@ -5447,7 +5447,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="79" spans="1:7" ht="13.5">
+    <row r="79" spans="1:7" ht="14">
       <c r="B79" s="13"/>
       <c r="C79" s="13"/>
       <c r="D79" s="13"/>

</xml_diff>

<commit_message>
refactor risk free rate class
</commit_message>
<xml_diff>
--- a/epsilon-phi-core/src/resources/templates/MSCI Index Construction.xlsx
+++ b/epsilon-phi-core/src/resources/templates/MSCI Index Construction.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11008"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fabar\repos\epsilon-phi\epsilon-phi-core\src\resources\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/francisbarker/Repositories/Python/epsilon-phi/epsilon-phi-core/src/resources/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E30160FA-2E2C-4131-B1FA-B0357D69F005}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EA27D92-944D-A344-9F3D-E51DABEA4678}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13096" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57600" yWindow="-8500" windowWidth="67200" windowHeight="37300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rules" sheetId="40" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="689" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="719" uniqueCount="325">
   <si>
     <r>
       <rPr>
@@ -1351,6 +1351,35 @@
   </si>
   <si>
     <t>2-Dec-1974 to 1-Mar-1995</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color rgb="FF73787B"/>
+        <rFont val="Roboto"/>
+      </rPr>
+      <t>SOUTH AFRICA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <rFont val="Roboto"/>
+      </rPr>
+      <t xml:space="preserve"> GOLD MINES</t>
+    </r>
+  </si>
+  <si>
+    <t>MEXICO FORMER</t>
+  </si>
+  <si>
+    <t>1-Jan-1988 to 1-Mar-1995</t>
+  </si>
+  <si>
+    <t>IFGMMX$</t>
+  </si>
+  <si>
+    <t>GOLDSSA$</t>
   </si>
 </sst>
 </file>
@@ -1796,15 +1825,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{398A9000-FE9A-0D49-BC15-66DEE1B3B201}">
-  <dimension ref="A1:J58"/>
-  <sheetFormatPr defaultColWidth="10.78515625" defaultRowHeight="13.15"/>
+  <dimension ref="A1:J60"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.796875" defaultRowHeight="13"/>
   <cols>
-    <col min="1" max="1" width="31.78515625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="21.2109375" style="6" customWidth="1"/>
-    <col min="3" max="10" width="17.78515625" style="6" customWidth="1"/>
+    <col min="1" max="1" width="31.796875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="21.19921875" style="6" customWidth="1"/>
+    <col min="3" max="10" width="17.796875" style="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="11" customFormat="1" ht="19.05" customHeight="1">
+    <row r="1" spans="1:10" s="11" customFormat="1" ht="19" customHeight="1">
       <c r="A1" s="10" t="s">
         <v>122</v>
       </c>
@@ -1836,7 +1865,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="2" spans="1:10" s="11" customFormat="1" ht="19.05" customHeight="1">
+    <row r="2" spans="1:10" s="11" customFormat="1" ht="19" customHeight="1">
       <c r="A2" s="10" t="s">
         <v>123</v>
       </c>
@@ -1868,7 +1897,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="28.15">
+    <row r="3" spans="1:10" ht="30">
       <c r="A3" s="2" t="s">
         <v>0</v>
       </c>
@@ -1900,7 +1929,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="16.05" customHeight="1">
+    <row r="4" spans="1:10" ht="16" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>1</v>
       </c>
@@ -1932,7 +1961,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="16.05" customHeight="1">
+    <row r="5" spans="1:10" ht="16" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>2</v>
       </c>
@@ -1964,7 +1993,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="16.05" customHeight="1">
+    <row r="6" spans="1:10" ht="16" customHeight="1">
       <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
@@ -1996,7 +2025,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="16.05" customHeight="1">
+    <row r="7" spans="1:10" ht="16" customHeight="1">
       <c r="A7" s="2" t="s">
         <v>4</v>
       </c>
@@ -2028,7 +2057,7 @@
         <v>32143</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="16.05" customHeight="1">
+    <row r="8" spans="1:10" ht="16" customHeight="1">
       <c r="A8" s="3" t="s">
         <v>57</v>
       </c>
@@ -2060,7 +2089,7 @@
         <v>32143</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="16.05" customHeight="1">
+    <row r="9" spans="1:10" ht="16" customHeight="1">
       <c r="A9" s="2" t="s">
         <v>5</v>
       </c>
@@ -2092,7 +2121,7 @@
         <v>32143</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="16.05" customHeight="1">
+    <row r="10" spans="1:10" ht="16" customHeight="1">
       <c r="A10" s="2" t="s">
         <v>6</v>
       </c>
@@ -2124,7 +2153,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="16.05" customHeight="1">
+    <row r="11" spans="1:10" ht="16" customHeight="1">
       <c r="A11" s="2" t="s">
         <v>7</v>
       </c>
@@ -2156,7 +2185,7 @@
         <v>34367</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="16.05" customHeight="1">
+    <row r="12" spans="1:10" ht="16" customHeight="1">
       <c r="A12" s="2" t="s">
         <v>8</v>
       </c>
@@ -2188,7 +2217,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="16.05" customHeight="1">
+    <row r="13" spans="1:10" ht="16" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>9</v>
       </c>
@@ -2220,7 +2249,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="16.05" customHeight="1">
+    <row r="14" spans="1:10" ht="16" customHeight="1">
       <c r="A14" s="2" t="s">
         <v>10</v>
       </c>
@@ -2252,7 +2281,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="16.05" customHeight="1">
+    <row r="15" spans="1:10" ht="16" customHeight="1">
       <c r="A15" s="2" t="s">
         <v>11</v>
       </c>
@@ -2284,7 +2313,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="16.05" customHeight="1">
+    <row r="16" spans="1:10" ht="16" customHeight="1">
       <c r="A16" s="2" t="s">
         <v>12</v>
       </c>
@@ -2316,7 +2345,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="16.05" customHeight="1">
+    <row r="17" spans="1:10" ht="16" customHeight="1">
       <c r="A17" s="2" t="s">
         <v>13</v>
       </c>
@@ -2348,7 +2377,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="16.05" customHeight="1">
+    <row r="18" spans="1:10" ht="16" customHeight="1">
       <c r="A18" s="2" t="s">
         <v>14</v>
       </c>
@@ -2380,7 +2409,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="16.05" customHeight="1">
+    <row r="19" spans="1:10" ht="16" customHeight="1">
       <c r="A19" s="2" t="s">
         <v>15</v>
       </c>
@@ -2412,7 +2441,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="16.05" customHeight="1">
+    <row r="20" spans="1:10" ht="16" customHeight="1">
       <c r="A20" s="2" t="s">
         <v>16</v>
       </c>
@@ -2444,7 +2473,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="16.05" customHeight="1">
+    <row r="21" spans="1:10" ht="16" customHeight="1">
       <c r="A21" s="2" t="s">
         <v>17</v>
       </c>
@@ -2476,7 +2505,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="16.05" customHeight="1">
+    <row r="22" spans="1:10" ht="16" customHeight="1">
       <c r="A22" s="2" t="s">
         <v>18</v>
       </c>
@@ -2508,7 +2537,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="16.05" customHeight="1">
+    <row r="23" spans="1:10" ht="16" customHeight="1">
       <c r="A23" s="3" t="s">
         <v>58</v>
       </c>
@@ -2540,7 +2569,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="16.05" customHeight="1">
+    <row r="24" spans="1:10" ht="16" customHeight="1">
       <c r="A24" s="2" t="s">
         <v>19</v>
       </c>
@@ -2572,7 +2601,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="16.05" customHeight="1">
+    <row r="25" spans="1:10" ht="16" customHeight="1">
       <c r="A25" s="2" t="s">
         <v>20</v>
       </c>
@@ -2604,7 +2633,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="16.05" customHeight="1">
+    <row r="26" spans="1:10" ht="16" customHeight="1">
       <c r="A26" s="2" t="s">
         <v>21</v>
       </c>
@@ -2636,7 +2665,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="16.05" customHeight="1">
+    <row r="27" spans="1:10" ht="16" customHeight="1">
       <c r="A27" s="2" t="s">
         <v>22</v>
       </c>
@@ -2668,7 +2697,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="16.05" customHeight="1">
+    <row r="28" spans="1:10" ht="16" customHeight="1">
       <c r="A28" s="2" t="s">
         <v>23</v>
       </c>
@@ -2700,7 +2729,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="16.05" customHeight="1">
+    <row r="29" spans="1:10" ht="16" customHeight="1">
       <c r="A29" s="2" t="s">
         <v>24</v>
       </c>
@@ -2732,7 +2761,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="16.05" customHeight="1">
+    <row r="30" spans="1:10" ht="16" customHeight="1">
       <c r="A30" s="3" t="s">
         <v>300</v>
       </c>
@@ -2764,7 +2793,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="16.05" customHeight="1">
+    <row r="31" spans="1:10" ht="16" customHeight="1">
       <c r="A31" s="2" t="s">
         <v>26</v>
       </c>
@@ -2796,7 +2825,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="16.05" customHeight="1">
+    <row r="32" spans="1:10" ht="16" customHeight="1">
       <c r="A32" s="2" t="s">
         <v>27</v>
       </c>
@@ -2807,542 +2836,542 @@
         <v>32143</v>
       </c>
       <c r="D32" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F32" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G32" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H32" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I32" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J32" s="5">
+        <v>32143</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="16" customHeight="1">
+      <c r="A33" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D33" s="5" t="s">
         <v>308</v>
       </c>
-      <c r="E32" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F32" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="G32" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="H32" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="I32" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="J32" s="5">
-        <v>32143</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" ht="16.05" customHeight="1">
-      <c r="A33" s="2" t="s">
+      <c r="E33" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F33" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G33" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H33" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I33" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J33" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="16" customHeight="1">
+      <c r="A34" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B33" s="5" t="s">
+      <c r="B34" s="5" t="s">
         <v>303</v>
       </c>
-      <c r="C33" s="5" t="s">
+      <c r="C34" s="5" t="s">
         <v>303</v>
       </c>
-      <c r="D33" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="E33" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F33" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="G33" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="H33" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="I33" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="J33" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" ht="16.05" customHeight="1">
-      <c r="A34" s="2" t="s">
+      <c r="D34" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F34" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G34" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H34" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I34" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J34" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="16" customHeight="1">
+      <c r="A35" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B34" s="5">
-        <v>32143</v>
-      </c>
-      <c r="C34" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D34" s="5">
+      <c r="B35" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D35" s="5">
         <v>25569</v>
       </c>
-      <c r="E34" s="5">
+      <c r="E35" s="5">
         <v>25569</v>
       </c>
-      <c r="F34" s="5">
+      <c r="F35" s="5">
         <v>25569</v>
       </c>
-      <c r="G34" s="5">
-        <v>32143</v>
-      </c>
-      <c r="H34" s="5">
-        <v>32143</v>
-      </c>
-      <c r="I34" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="J34" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" ht="16.05" customHeight="1">
-      <c r="A35" s="2" t="s">
+      <c r="G35" s="5">
+        <v>32143</v>
+      </c>
+      <c r="H35" s="5">
+        <v>32143</v>
+      </c>
+      <c r="I35" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J35" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" ht="16" customHeight="1">
+      <c r="A36" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B35" s="5">
-        <v>32143</v>
-      </c>
-      <c r="C35" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D35" s="5">
-        <v>32143</v>
-      </c>
-      <c r="E35" s="5">
-        <v>32143</v>
-      </c>
-      <c r="F35" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="G35" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="H35" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="I35" s="5">
-        <v>32143</v>
-      </c>
-      <c r="J35" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" ht="16.05" customHeight="1">
-      <c r="A36" s="2" t="s">
+      <c r="B36" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D36" s="5">
+        <v>32143</v>
+      </c>
+      <c r="E36" s="5">
+        <v>32143</v>
+      </c>
+      <c r="F36" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G36" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H36" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I36" s="5">
+        <v>32143</v>
+      </c>
+      <c r="J36" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" ht="16" customHeight="1">
+      <c r="A37" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B36" s="5">
-        <v>32143</v>
-      </c>
-      <c r="C36" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D36" s="5">
+      <c r="B37" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D37" s="5">
         <v>25569</v>
       </c>
-      <c r="E36" s="5">
+      <c r="E37" s="5">
         <v>25569</v>
       </c>
-      <c r="F36" s="5">
+      <c r="F37" s="5">
         <v>25569</v>
       </c>
-      <c r="G36" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="H36" s="5">
-        <v>32143</v>
-      </c>
-      <c r="I36" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="J36" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" ht="16.05" customHeight="1">
-      <c r="A37" s="2" t="s">
+      <c r="G37" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H37" s="5">
+        <v>32143</v>
+      </c>
+      <c r="I37" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J37" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" ht="16" customHeight="1">
+      <c r="A38" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B37" s="5" t="s">
+      <c r="B38" s="5" t="s">
         <v>318</v>
       </c>
-      <c r="C37" s="5" t="s">
+      <c r="C38" s="5" t="s">
         <v>318</v>
       </c>
-      <c r="D37" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="E37" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F37" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="G37" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="H37" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="I37" s="5" t="s">
+      <c r="D38" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E38" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F38" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G38" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H38" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I38" s="5" t="s">
         <v>318</v>
       </c>
-      <c r="J37" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" ht="16.05" customHeight="1">
-      <c r="A38" s="2" t="s">
+      <c r="J38" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" ht="16" customHeight="1">
+      <c r="A39" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B38" s="5">
+      <c r="B39" s="5">
         <v>34367</v>
       </c>
-      <c r="C38" s="5">
+      <c r="C39" s="5">
         <v>34367</v>
       </c>
-      <c r="D38" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="E38" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F38" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="G38" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="H38" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="I38" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="J38" s="5">
+      <c r="D39" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E39" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F39" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G39" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H39" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I39" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J39" s="5">
         <v>34367</v>
       </c>
     </row>
-    <row r="39" spans="1:10" ht="16.05" customHeight="1">
-      <c r="A39" s="2" t="s">
+    <row r="40" spans="1:10" ht="16" customHeight="1">
+      <c r="A40" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B39" s="5">
-        <v>32143</v>
-      </c>
-      <c r="C39" s="5">
-        <v>32143</v>
-      </c>
-      <c r="D39" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="E39" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F39" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="G39" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="H39" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="I39" s="5">
-        <v>32143</v>
-      </c>
-      <c r="J39" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" ht="16.05" customHeight="1">
-      <c r="A40" s="2" t="s">
+      <c r="B40" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C40" s="5">
+        <v>32143</v>
+      </c>
+      <c r="D40" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E40" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F40" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G40" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H40" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I40" s="5">
+        <v>32143</v>
+      </c>
+      <c r="J40" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" ht="16" customHeight="1">
+      <c r="A41" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B40" s="5">
+      <c r="B41" s="5">
         <v>34760</v>
       </c>
-      <c r="C40" s="5">
+      <c r="C41" s="5">
         <v>34760</v>
       </c>
-      <c r="D40" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="E40" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F40" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="G40" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="H40" s="5">
+      <c r="D41" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E41" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F41" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G41" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H41" s="5">
         <v>34760</v>
       </c>
-      <c r="I40" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="J40" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" ht="16.05" customHeight="1">
-      <c r="A41" s="2" t="s">
+      <c r="I41" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J41" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" ht="16" customHeight="1">
+      <c r="A42" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B41" s="5">
-        <v>32143</v>
-      </c>
-      <c r="C41" s="5" t="s">
+      <c r="B42" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C42" s="5" t="s">
         <v>309</v>
       </c>
-      <c r="D41" s="5">
+      <c r="D42" s="5">
         <v>35765</v>
       </c>
-      <c r="E41" s="5">
+      <c r="E42" s="5">
         <v>35765</v>
       </c>
-      <c r="F41" s="5">
+      <c r="F42" s="5">
         <v>35765</v>
       </c>
-      <c r="G41" s="5">
+      <c r="G42" s="5">
         <v>35765</v>
       </c>
-      <c r="H41" s="5">
-        <v>32143</v>
-      </c>
-      <c r="I41" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="J41" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" ht="16.05" customHeight="1">
-      <c r="A42" s="2" t="s">
+      <c r="H42" s="5">
+        <v>32143</v>
+      </c>
+      <c r="I42" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J42" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" ht="16" customHeight="1">
+      <c r="A43" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B42" s="5">
+      <c r="B43" s="5">
         <v>41792</v>
       </c>
-      <c r="C42" s="5">
+      <c r="C43" s="5">
         <v>41792</v>
       </c>
-      <c r="D42" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="E42" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F42" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="G42" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="H42" s="5">
+      <c r="D43" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E43" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F43" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G43" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H43" s="5">
         <v>41792</v>
       </c>
-      <c r="I42" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="J42" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" ht="16.05" customHeight="1">
-      <c r="A43" s="2" t="s">
+      <c r="I43" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J43" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" ht="16" customHeight="1">
+      <c r="A44" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B43" s="5" t="s">
+      <c r="B44" s="5" t="s">
         <v>310</v>
       </c>
-      <c r="C43" s="5" t="s">
+      <c r="C44" s="5" t="s">
         <v>310</v>
       </c>
-      <c r="D43" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="E43" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F43" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="G43" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="H43" s="5" t="s">
+      <c r="D44" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E44" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F44" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G44" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H44" s="5" t="s">
         <v>310</v>
       </c>
-      <c r="I43" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="J43" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" ht="16.05" customHeight="1">
-      <c r="A44" s="2" t="s">
+      <c r="I44" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J44" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" ht="16" customHeight="1">
+      <c r="A45" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B44" s="5">
+      <c r="B45" s="5">
         <v>43614</v>
       </c>
-      <c r="C44" s="5">
+      <c r="C45" s="5">
         <v>43614</v>
       </c>
-      <c r="D44" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="E44" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F44" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="G44" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="H44" s="5">
+      <c r="D45" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E45" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F45" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G45" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H45" s="5">
         <v>43614</v>
       </c>
-      <c r="I44" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="J44" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10" ht="16.05" customHeight="1">
-      <c r="A45" s="3" t="s">
+      <c r="I45" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J45" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" ht="16" customHeight="1">
+      <c r="A46" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B45" s="5">
-        <v>32143</v>
-      </c>
-      <c r="C45" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D45" s="5">
+      <c r="B46" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C46" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D46" s="5">
         <v>26634</v>
       </c>
-      <c r="E45" s="5">
+      <c r="E46" s="5">
         <v>26634</v>
       </c>
-      <c r="F45" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="G45" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="H45" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="I45" s="5">
-        <v>32143</v>
-      </c>
-      <c r="J45" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10" ht="16.05" customHeight="1">
-      <c r="A46" s="2" t="s">
+      <c r="F46" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G46" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H46" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I46" s="5">
+        <v>32143</v>
+      </c>
+      <c r="J46" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" ht="16" customHeight="1">
+      <c r="A47" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B46" s="5">
-        <v>32143</v>
-      </c>
-      <c r="C46" s="5">
-        <v>32143</v>
-      </c>
-      <c r="D46" s="5" t="s">
+      <c r="B47" s="5">
+        <v>34760</v>
+      </c>
+      <c r="C47" s="5">
+        <v>34760</v>
+      </c>
+      <c r="D47" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E47" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F47" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G47" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H47" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I47" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J47" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" ht="16" customHeight="1">
+      <c r="A48" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>322</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D48" s="5" t="s">
         <v>319</v>
       </c>
-      <c r="E46" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F46" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="G46" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="H46" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="I46" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="J46" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10" ht="16.05" customHeight="1">
-      <c r="A47" s="2" t="s">
+      <c r="E48" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F48" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G48" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H48" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I48" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J48" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" ht="16" customHeight="1">
+      <c r="A49" s="2" t="s">
         <v>41</v>
-      </c>
-      <c r="B47" s="5">
-        <v>32143</v>
-      </c>
-      <c r="C47" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D47" s="5">
-        <v>25569</v>
-      </c>
-      <c r="E47" s="5">
-        <v>25569</v>
-      </c>
-      <c r="F47" s="5">
-        <v>25569</v>
-      </c>
-      <c r="G47" s="5">
-        <v>32143</v>
-      </c>
-      <c r="H47" s="5">
-        <v>32143</v>
-      </c>
-      <c r="I47" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="J47" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" ht="16.05" customHeight="1">
-      <c r="A48" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="B48" s="5" t="s">
-        <v>311</v>
-      </c>
-      <c r="C48" s="5" t="s">
-        <v>311</v>
-      </c>
-      <c r="D48" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="E48" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F48" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="G48" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="H48" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="I48" s="5" t="s">
-        <v>311</v>
-      </c>
-      <c r="J48" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10" ht="16.05" customHeight="1">
-      <c r="A49" s="2" t="s">
-        <v>43</v>
       </c>
       <c r="B49" s="5">
         <v>32143</v>
@@ -3359,8 +3388,8 @@
       <c r="F49" s="5">
         <v>25569</v>
       </c>
-      <c r="G49" s="5" t="s">
-        <v>52</v>
+      <c r="G49" s="5">
+        <v>32143</v>
       </c>
       <c r="H49" s="5">
         <v>32143</v>
@@ -3372,297 +3401,361 @@
         <v>52</v>
       </c>
     </row>
-    <row r="50" spans="1:10" ht="16.05" customHeight="1">
+    <row r="50" spans="1:10" ht="16" customHeight="1">
       <c r="A50" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B50" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="C50" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="D50" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E50" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F50" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G50" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H50" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I50" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="J50" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" ht="16" customHeight="1">
+      <c r="A51" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B51" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C51" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D51" s="5">
+        <v>25569</v>
+      </c>
+      <c r="E51" s="5">
+        <v>25569</v>
+      </c>
+      <c r="F51" s="5">
+        <v>25569</v>
+      </c>
+      <c r="G51" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H51" s="5">
+        <v>32143</v>
+      </c>
+      <c r="I51" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J51" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" ht="16" customHeight="1">
+      <c r="A52" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B50" s="5">
-        <v>32143</v>
-      </c>
-      <c r="C50" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D50" s="5">
+      <c r="B52" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C52" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D52" s="5">
         <v>25569</v>
       </c>
-      <c r="E50" s="5">
+      <c r="E52" s="5">
         <v>25569</v>
       </c>
-      <c r="F50" s="5">
+      <c r="F52" s="5">
         <v>25569</v>
       </c>
-      <c r="G50" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="H50" s="5">
-        <v>32143</v>
-      </c>
-      <c r="I50" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="J50" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10" ht="16.05" customHeight="1">
-      <c r="A51" s="2" t="s">
+      <c r="G52" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H52" s="5">
+        <v>32143</v>
+      </c>
+      <c r="I52" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J52" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" ht="16" customHeight="1">
+      <c r="A53" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B51" s="5">
+      <c r="B53" s="5">
         <v>37410</v>
       </c>
-      <c r="C51" s="5">
+      <c r="C53" s="5">
         <v>37410</v>
       </c>
-      <c r="D51" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="E51" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F51" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="G51" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="H51" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="I51" s="5">
+      <c r="D53" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E53" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F53" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G53" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H53" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I53" s="5">
         <v>37410</v>
       </c>
-      <c r="J51" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" ht="16.05" customHeight="1">
-      <c r="A52" s="7" t="s">
+      <c r="J53" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" ht="16" customHeight="1">
+      <c r="A54" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="B52" s="5" t="s">
+      <c r="B54" s="5" t="s">
         <v>312</v>
       </c>
-      <c r="C52" s="5" t="s">
+      <c r="C54" s="5" t="s">
         <v>312</v>
       </c>
-      <c r="D52" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="E52" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F52" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="G52" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="H52" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="I52" s="5" t="s">
+      <c r="D54" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E54" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F54" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G54" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H54" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I54" s="5" t="s">
         <v>312</v>
       </c>
-      <c r="J52" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10" ht="16.05" customHeight="1">
-      <c r="A53" s="2" t="s">
+      <c r="J54" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" ht="16" customHeight="1">
+      <c r="A55" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B53" s="5">
-        <v>32143</v>
-      </c>
-      <c r="C53" s="5">
-        <v>32143</v>
-      </c>
-      <c r="D53" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="E53" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F53" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="G53" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="H53" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="I53" s="5">
-        <v>32143</v>
-      </c>
-      <c r="J53" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" ht="16.05" customHeight="1">
-      <c r="A54" s="2" t="s">
+      <c r="B55" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C55" s="5">
+        <v>32143</v>
+      </c>
+      <c r="D55" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E55" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F55" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G55" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H55" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I55" s="5">
+        <v>32143</v>
+      </c>
+      <c r="J55" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" ht="16" customHeight="1">
+      <c r="A56" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B54" s="5">
+      <c r="B56" s="5">
         <v>32752</v>
       </c>
-      <c r="C54" s="5">
+      <c r="C56" s="5">
         <v>32752</v>
       </c>
-      <c r="D54" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="E54" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F54" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="G54" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="H54" s="5">
+      <c r="D56" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E56" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F56" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G56" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H56" s="5">
         <v>35339</v>
       </c>
-      <c r="I54" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="J54" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" ht="16.05" customHeight="1">
-      <c r="A55" s="2" t="s">
+      <c r="I56" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J56" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" ht="16" customHeight="1">
+      <c r="A57" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B55" s="5">
+      <c r="B57" s="5">
         <v>41792</v>
       </c>
-      <c r="C55" s="5">
+      <c r="C57" s="5">
         <v>41792</v>
       </c>
-      <c r="D55" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="E55" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F55" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="G55" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="H55" s="5">
+      <c r="D57" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E57" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F57" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G57" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H57" s="5">
         <v>41792</v>
       </c>
-      <c r="I55" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="J55" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="56" spans="1:10" ht="16.05" customHeight="1">
-      <c r="A56" s="2" t="s">
+      <c r="I57" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J57" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" ht="16" customHeight="1">
+      <c r="A58" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B56" s="5">
-        <v>32143</v>
-      </c>
-      <c r="C56" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D56" s="5">
+      <c r="B58" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C58" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D58" s="5">
         <v>25569</v>
       </c>
-      <c r="E56" s="5">
+      <c r="E58" s="5">
         <v>25569</v>
       </c>
-      <c r="F56" s="5">
+      <c r="F58" s="5">
         <v>25569</v>
       </c>
-      <c r="G56" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="H56" s="5">
-        <v>32143</v>
-      </c>
-      <c r="I56" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="J56" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10" ht="16.05" customHeight="1">
-      <c r="A57" s="3" t="s">
+      <c r="G58" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H58" s="5">
+        <v>32143</v>
+      </c>
+      <c r="I58" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J58" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" ht="16" customHeight="1">
+      <c r="A59" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="B57" s="5">
-        <v>32143</v>
-      </c>
-      <c r="C57" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D57" s="5">
+      <c r="B59" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C59" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D59" s="5">
         <v>25569</v>
       </c>
-      <c r="E57" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F57" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="G57" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="H57" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="I57" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="J57" s="5">
-        <v>32143</v>
-      </c>
-    </row>
-    <row r="58" spans="1:10" ht="16.05" customHeight="1">
-      <c r="A58" s="2" t="s">
+      <c r="E59" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F59" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G59" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H59" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I59" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J59" s="5">
+        <v>32143</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" ht="16" customHeight="1">
+      <c r="A60" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B58" s="5" t="s">
+      <c r="B60" s="5" t="s">
         <v>313</v>
       </c>
-      <c r="C58" s="5" t="s">
+      <c r="C60" s="5" t="s">
         <v>313</v>
       </c>
-      <c r="D58" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="E58" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F58" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="G58" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="H58" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="I58" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="J58" s="5" t="s">
+      <c r="D60" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E60" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F60" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G60" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H60" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I60" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J60" s="5" t="s">
         <v>313</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A52" r:id="rId1" xr:uid="{52D16EEC-E5ED-404C-86D1-39D51CBCCAC6}"/>
+    <hyperlink ref="A54" r:id="rId1" xr:uid="{52D16EEC-E5ED-404C-86D1-39D51CBCCAC6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
@@ -3671,12 +3764,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A7EF705-CFED-174D-8EBB-657B7E248B5D}">
-  <dimension ref="A2:G68"/>
-  <sheetFormatPr defaultColWidth="10.78515625" defaultRowHeight="13.15"/>
+  <dimension ref="A2:G70"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.796875" defaultRowHeight="13"/>
   <cols>
-    <col min="1" max="1" width="19.42578125" customWidth="1"/>
-    <col min="2" max="2" width="29.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="11.42578125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="19.3984375" customWidth="1"/>
+    <col min="2" max="2" width="29.3984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="11.3984375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:5">
@@ -4208,228 +4301,228 @@
     </row>
     <row r="33" spans="1:5" ht="14" customHeight="1">
       <c r="A33" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B33" s="8" t="s">
-        <v>109</v>
+        <v>321</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>88</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>284</v>
+        <v>236</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>283</v>
+        <v>323</v>
       </c>
       <c r="E33" s="12" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="14" customHeight="1">
       <c r="A34" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>89</v>
+        <v>28</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>109</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>238</v>
+        <v>284</v>
       </c>
       <c r="D34" s="12" t="s">
-        <v>237</v>
+        <v>283</v>
       </c>
       <c r="E34" s="12" t="s">
-        <v>179</v>
+        <v>153</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="14" customHeight="1">
       <c r="A35" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="D35" s="12" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="E35" s="12" t="s">
-        <v>154</v>
+        <v>179</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="14" customHeight="1">
       <c r="A36" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="D36" s="12" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="E36" s="12" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="14" customHeight="1">
       <c r="A37" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B37" s="8" t="s">
-        <v>110</v>
+        <v>31</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>91</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>286</v>
+        <v>240</v>
       </c>
       <c r="D37" s="12" t="s">
-        <v>285</v>
+        <v>239</v>
       </c>
       <c r="E37" s="12" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="14" customHeight="1">
       <c r="A38" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>92</v>
+        <v>32</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>110</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>244</v>
+        <v>286</v>
       </c>
       <c r="D38" s="12" t="s">
-        <v>243</v>
+        <v>285</v>
       </c>
       <c r="E38" s="12" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="14" customHeight="1">
       <c r="A39" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="E39" s="12" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="14" customHeight="1">
       <c r="A40" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="D40" s="12" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="E40" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="14" customHeight="1">
       <c r="A41" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="D41" s="12" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="E41" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="14" customHeight="1">
       <c r="A42" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="D42" s="12" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="E42" s="12" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="14" customHeight="1">
       <c r="A43" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B43" s="8" t="s">
-        <v>111</v>
+        <v>37</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>96</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>288</v>
+        <v>252</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>287</v>
+        <v>251</v>
       </c>
       <c r="E43" s="12" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="14" customHeight="1">
       <c r="A44" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B44" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="C44" s="8" t="s">
+        <v>288</v>
+      </c>
+      <c r="D44" s="12" t="s">
+        <v>287</v>
+      </c>
+      <c r="E44" s="12" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="14" customHeight="1">
+      <c r="A45" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B44" s="1" t="s">
+      <c r="B45" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="C44" s="8" t="s">
+      <c r="C45" s="8" t="s">
         <v>256</v>
       </c>
-      <c r="D44" s="12" t="s">
+      <c r="D45" s="12" t="s">
         <v>255</v>
       </c>
-      <c r="E44" s="12" t="s">
+      <c r="E45" s="12" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="45" spans="1:5" ht="14" customHeight="1">
-      <c r="A45" s="3" t="s">
+    <row r="46" spans="1:5" ht="14" customHeight="1">
+      <c r="A46" s="3" t="s">
         <v>51</v>
-      </c>
-      <c r="B45" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="C45" s="8" t="s">
-        <v>258</v>
-      </c>
-      <c r="D45" s="12" t="s">
-        <v>257</v>
-      </c>
-      <c r="E45" s="12" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" ht="13.5">
-      <c r="A46" s="3" t="s">
-        <v>59</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>98</v>
@@ -4444,238 +4537,272 @@
         <v>164</v>
       </c>
     </row>
-    <row r="47" spans="1:5" ht="13.5">
-      <c r="A47" s="2" t="s">
+    <row r="47" spans="1:5" ht="14">
+      <c r="A47" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C47" s="8" t="s">
+        <v>258</v>
+      </c>
+      <c r="D47" s="12" t="s">
+        <v>257</v>
+      </c>
+      <c r="E47" s="12" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="14">
+      <c r="A48" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B47" s="1" t="s">
+      <c r="B48" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="C47" s="8" t="s">
+      <c r="C48" s="8" t="s">
         <v>254</v>
       </c>
-      <c r="D47" s="12" t="s">
+      <c r="D48" s="12" t="s">
         <v>253</v>
       </c>
-      <c r="E47" s="12" t="s">
+      <c r="E48" s="12" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="48" spans="1:5" ht="13.5">
-      <c r="A48" s="2" t="s">
+    <row r="49" spans="1:5" ht="12" customHeight="1">
+      <c r="A49" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C49" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="D49" s="12" t="s">
+        <v>324</v>
+      </c>
+      <c r="E49" s="12" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" ht="14">
+      <c r="A50" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B48" s="1" t="s">
+      <c r="B50" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="C48" s="8" t="s">
+      <c r="C50" s="8" t="s">
         <v>260</v>
       </c>
-      <c r="D48" s="12" t="s">
+      <c r="D50" s="12" t="s">
         <v>259</v>
       </c>
-      <c r="E48" s="12" t="s">
+      <c r="E50" s="12" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="49" spans="1:5" ht="13.5">
-      <c r="A49" s="2" t="s">
+    <row r="51" spans="1:5" ht="14">
+      <c r="A51" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B49" s="8" t="s">
+      <c r="B51" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="C49" s="8" t="s">
+      <c r="C51" s="8" t="s">
         <v>290</v>
       </c>
-      <c r="D49" s="12" t="s">
+      <c r="D51" s="12" t="s">
         <v>289</v>
       </c>
-      <c r="E49" s="12" t="s">
+      <c r="E51" s="12" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="50" spans="1:5" ht="13.5">
-      <c r="A50" s="2" t="s">
+    <row r="52" spans="1:5" ht="14">
+      <c r="A52" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B50" s="1" t="s">
+      <c r="B52" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="C50" s="8" t="s">
+      <c r="C52" s="8" t="s">
         <v>262</v>
       </c>
-      <c r="D50" s="12" t="s">
+      <c r="D52" s="12" t="s">
         <v>261</v>
       </c>
-      <c r="E50" s="12" t="s">
+      <c r="E52" s="12" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="51" spans="1:5" ht="13.5">
-      <c r="A51" s="2" t="s">
+    <row r="53" spans="1:5" ht="14">
+      <c r="A53" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B51" s="1" t="s">
+      <c r="B53" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="C51" s="8" t="s">
+      <c r="C53" s="8" t="s">
         <v>264</v>
       </c>
-      <c r="D51" s="12" t="s">
+      <c r="D53" s="12" t="s">
         <v>263</v>
       </c>
-      <c r="E51" s="12" t="s">
+      <c r="E53" s="12" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="52" spans="1:5" ht="13.5">
-      <c r="A52" s="2" t="s">
+    <row r="54" spans="1:5" ht="14">
+      <c r="A54" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B52" s="1" t="s">
+      <c r="B54" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="C52" s="8" t="s">
+      <c r="C54" s="8" t="s">
         <v>266</v>
       </c>
-      <c r="D52" s="12" t="s">
+      <c r="D54" s="12" t="s">
         <v>265</v>
       </c>
-      <c r="E52" s="12" t="s">
+      <c r="E54" s="12" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="53" spans="1:5" ht="13.5">
-      <c r="A53" s="7" t="s">
+    <row r="55" spans="1:5" ht="14">
+      <c r="A55" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="B53" s="1" t="s">
+      <c r="B55" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="C53" s="8" t="s">
+      <c r="C55" s="8" t="s">
         <v>266</v>
       </c>
-      <c r="D53" s="12" t="s">
+      <c r="D55" s="12" t="s">
         <v>265</v>
       </c>
-      <c r="E53" s="12" t="s">
+      <c r="E55" s="12" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="54" spans="1:5" ht="13.5">
-      <c r="A54" s="2" t="s">
+    <row r="56" spans="1:5" ht="14">
+      <c r="A56" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B54" s="1" t="s">
+      <c r="B56" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="C54" s="8" t="s">
+      <c r="C56" s="8" t="s">
         <v>268</v>
       </c>
-      <c r="D54" s="12" t="s">
+      <c r="D56" s="12" t="s">
         <v>267</v>
       </c>
-      <c r="E54" s="12" t="s">
+      <c r="E56" s="12" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="55" spans="1:5" ht="13.5">
-      <c r="A55" s="2" t="s">
+    <row r="57" spans="1:5" ht="14">
+      <c r="A57" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B55" s="1" t="s">
+      <c r="B57" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="C55" s="8" t="s">
+      <c r="C57" s="8" t="s">
         <v>270</v>
       </c>
-      <c r="D55" s="12" t="s">
+      <c r="D57" s="12" t="s">
         <v>269</v>
       </c>
-      <c r="E55" s="12" t="s">
+      <c r="E57" s="12" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="56" spans="1:5" ht="13.5">
-      <c r="A56" s="2" t="s">
+    <row r="58" spans="1:5" ht="14">
+      <c r="A58" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B56" s="1" t="s">
+      <c r="B58" s="1" t="s">
         <v>295</v>
       </c>
-      <c r="C56" s="8" t="s">
+      <c r="C58" s="8" t="s">
         <v>272</v>
       </c>
-      <c r="D56" s="12" t="s">
+      <c r="D58" s="12" t="s">
         <v>271</v>
       </c>
-      <c r="E56" s="12" t="s">
+      <c r="E58" s="12" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="57" spans="1:5" ht="13.5">
-      <c r="A57" s="2" t="s">
+    <row r="59" spans="1:5" ht="14">
+      <c r="A59" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B57" s="1" t="s">
+      <c r="B59" s="1" t="s">
         <v>298</v>
       </c>
-      <c r="C57" s="8" t="s">
+      <c r="C59" s="8" t="s">
         <v>276</v>
       </c>
-      <c r="D57" s="12" t="s">
+      <c r="D59" s="12" t="s">
         <v>275</v>
       </c>
-      <c r="E57" s="12" t="s">
+      <c r="E59" s="12" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="58" spans="1:5" ht="13.5">
-      <c r="A58" s="3" t="s">
+    <row r="60" spans="1:5" ht="14">
+      <c r="A60" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="B58" s="1" t="s">
+      <c r="B60" s="1" t="s">
         <v>297</v>
       </c>
-      <c r="C58" s="8" t="s">
+      <c r="C60" s="8" t="s">
         <v>274</v>
       </c>
-      <c r="D58" s="12" t="s">
+      <c r="D60" s="12" t="s">
         <v>273</v>
       </c>
-      <c r="E58" s="12" t="s">
+      <c r="E60" s="12" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="59" spans="1:5" ht="13.5">
-      <c r="A59" s="2" t="s">
+    <row r="61" spans="1:5" ht="14">
+      <c r="A61" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B59" s="8" t="s">
+      <c r="B61" s="8" t="s">
         <v>296</v>
       </c>
-      <c r="C59" s="8" t="s">
+      <c r="C61" s="8" t="s">
         <v>292</v>
       </c>
-      <c r="D59" s="12" t="s">
+      <c r="D61" s="12" t="s">
         <v>291</v>
       </c>
-      <c r="E59" s="12" t="s">
+      <c r="E61" s="12" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="68" spans="2:7" ht="13.5">
-      <c r="B68" s="13"/>
-      <c r="C68" s="13"/>
-      <c r="D68" s="13"/>
-      <c r="E68" s="13"/>
-      <c r="F68" s="9"/>
-      <c r="G68" s="9"/>
+    <row r="70" spans="2:7" ht="14">
+      <c r="B70" s="13"/>
+      <c r="C70" s="13"/>
+      <c r="D70" s="13"/>
+      <c r="E70" s="13"/>
+      <c r="F70" s="9"/>
+      <c r="G70" s="9"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A53" r:id="rId1" xr:uid="{484FCBF9-98EC-5A4C-87E4-AF76A89FDA61}"/>
+    <hyperlink ref="A55" r:id="rId1" xr:uid="{484FCBF9-98EC-5A4C-87E4-AF76A89FDA61}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>

</xml_diff>

<commit_message>
Factor classes and managers
</commit_message>
<xml_diff>
--- a/epsilon-phi-core/src/resources/templates/MSCI Index Construction.xlsx
+++ b/epsilon-phi-core/src/resources/templates/MSCI Index Construction.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/francisbarker/Repositories/Python/epsilon-phi/epsilon-phi-core/src/resources/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EA27D92-944D-A344-9F3D-E51DABEA4678}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFB85C0E-BAD2-6D4A-8462-FE4C4E42E6DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57600" yWindow="-8500" windowWidth="67200" windowHeight="37300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57600" yWindow="-9000" windowWidth="67200" windowHeight="37800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rules" sheetId="40" r:id="rId1"/>
     <sheet name="Mapping" sheetId="41" r:id="rId2"/>
+    <sheet name="Rules (2)" sheetId="42" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="719" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1138" uniqueCount="325">
   <si>
     <r>
       <rPr>
@@ -558,9 +559,6 @@
     <t>EAFE</t>
   </si>
   <si>
-    <t>EUROPE</t>
-  </si>
-  <si>
     <t>EMU</t>
   </si>
   <si>
@@ -579,9 +577,6 @@
     <t>USA</t>
   </si>
   <si>
-    <t>ACWI</t>
-  </si>
-  <si>
     <t>Australia</t>
   </si>
   <si>
@@ -1290,18 +1285,9 @@
     <t>United Kingdom</t>
   </si>
   <si>
-    <t>WORLD</t>
-  </si>
-  <si>
     <t>LUXEMBOURG (2)</t>
   </si>
   <si>
-    <t>ACASIAPACIFIC</t>
-  </si>
-  <si>
-    <t>ACAMERICAS</t>
-  </si>
-  <si>
     <t>1-Jun-2001 to 26-Nov-2013</t>
   </si>
   <si>
@@ -1333,9 +1319,6 @@
   </si>
   <si>
     <t>2-Feb-1994 to 31-May-2006</t>
-  </si>
-  <si>
-    <t>ACEUROPE, MIDDLEEAST</t>
   </si>
   <si>
     <t>1-Jan-1988 to 29-May-2009, 29-May-2019 to 30-Nov-2021</t>
@@ -1380,6 +1363,24 @@
   </si>
   <si>
     <t>GOLDSSA$</t>
+  </si>
+  <si>
+    <t>World</t>
+  </si>
+  <si>
+    <t>Europe</t>
+  </si>
+  <si>
+    <t>AC World</t>
+  </si>
+  <si>
+    <t>AC Europe and Middle East</t>
+  </si>
+  <si>
+    <t>AC Asia Pacific</t>
+  </si>
+  <si>
+    <t>AC Americas</t>
   </si>
 </sst>
 </file>
@@ -1477,7 +1478,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -1520,6 +1521,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1829,72 +1831,72 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.796875" defaultRowHeight="13"/>
   <cols>
     <col min="1" max="1" width="31.796875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="21.19921875" style="6" customWidth="1"/>
+    <col min="2" max="2" width="32" style="6" customWidth="1"/>
     <col min="3" max="10" width="17.796875" style="6" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" s="11" customFormat="1" ht="19" customHeight="1">
       <c r="A1" s="10" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>62</v>
+        <v>321</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>53</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>299</v>
+        <v>319</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>54</v>
       </c>
       <c r="F1" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="G1" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="G1" s="4" t="s">
-        <v>56</v>
-      </c>
       <c r="H1" s="4" t="s">
-        <v>314</v>
+        <v>322</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>301</v>
+        <v>323</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>302</v>
+        <v>324</v>
       </c>
     </row>
     <row r="2" spans="1:10" s="11" customFormat="1" ht="19" customHeight="1">
       <c r="A2" s="10" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B2" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="D2" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="F2" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="D2" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="E2" s="4" t="s">
+      <c r="G2" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="H2" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="I2" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="J2" s="4" t="s">
         <v>119</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="30">
@@ -1902,10 +1904,10 @@
         <v>0</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>315</v>
+        <v>309</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>315</v>
+        <v>309</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>52</v>
@@ -1926,7 +1928,7 @@
         <v>52</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>315</v>
+        <v>309</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="16" customHeight="1">
@@ -2059,7 +2061,7 @@
     </row>
     <row r="8" spans="1:10" ht="16" customHeight="1">
       <c r="A8" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B8" s="5">
         <v>32143</v>
@@ -2385,19 +2387,19 @@
         <v>32143</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>316</v>
+        <v>310</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="H18" s="5">
         <v>32143</v>
@@ -2539,7 +2541,7 @@
     </row>
     <row r="23" spans="1:10" ht="16" customHeight="1">
       <c r="A23" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B23" s="5">
         <v>32143</v>
@@ -2577,7 +2579,7 @@
         <v>34367</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="D24" s="5">
         <v>40325</v>
@@ -2670,10 +2672,10 @@
         <v>22</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="D27" s="5" t="s">
         <v>52</v>
@@ -2688,7 +2690,7 @@
         <v>52</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="I27" s="5" t="s">
         <v>52</v>
@@ -2763,10 +2765,10 @@
     </row>
     <row r="30" spans="1:10" ht="16" customHeight="1">
       <c r="A30" s="3" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>52</v>
@@ -2784,7 +2786,7 @@
         <v>52</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="I30" s="5" t="s">
         <v>52</v>
@@ -2798,16 +2800,16 @@
         <v>26</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>317</v>
+        <v>311</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>317</v>
+        <v>311</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="F31" s="5" t="s">
         <v>52</v>
@@ -2819,7 +2821,7 @@
         <v>52</v>
       </c>
       <c r="I31" s="5" t="s">
-        <v>317</v>
+        <v>311</v>
       </c>
       <c r="J31" s="5" t="s">
         <v>52</v>
@@ -2859,7 +2861,7 @@
     </row>
     <row r="33" spans="1:10" ht="16" customHeight="1">
       <c r="A33" s="2" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>52</v>
@@ -2868,7 +2870,7 @@
         <v>52</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
       <c r="E33" s="5" t="s">
         <v>52</v>
@@ -2894,10 +2896,10 @@
         <v>28</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>52</v>
@@ -3022,10 +3024,10 @@
         <v>32</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>52</v>
@@ -3043,7 +3045,7 @@
         <v>52</v>
       </c>
       <c r="I38" s="5" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="J38" s="5" t="s">
         <v>52</v>
@@ -3153,7 +3155,7 @@
         <v>32143</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
       <c r="D42" s="5">
         <v>35765</v>
@@ -3214,10 +3216,10 @@
         <v>38</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>310</v>
+        <v>305</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>310</v>
+        <v>305</v>
       </c>
       <c r="D44" s="5" t="s">
         <v>52</v>
@@ -3232,7 +3234,7 @@
         <v>52</v>
       </c>
       <c r="H44" s="5" t="s">
-        <v>310</v>
+        <v>305</v>
       </c>
       <c r="I44" s="5" t="s">
         <v>52</v>
@@ -3339,16 +3341,16 @@
     </row>
     <row r="48" spans="1:10" ht="16" customHeight="1">
       <c r="A48" s="2" t="s">
-        <v>320</v>
+        <v>314</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>322</v>
+        <v>316</v>
       </c>
       <c r="C48" s="5" t="s">
         <v>52</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>319</v>
+        <v>313</v>
       </c>
       <c r="E48" s="5" t="s">
         <v>52</v>
@@ -3406,10 +3408,10 @@
         <v>42</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="D50" s="5" t="s">
         <v>52</v>
@@ -3427,7 +3429,7 @@
         <v>52</v>
       </c>
       <c r="I50" s="5" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="J50" s="5" t="s">
         <v>52</v>
@@ -3531,13 +3533,13 @@
     </row>
     <row r="54" spans="1:10" ht="16" customHeight="1">
       <c r="A54" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>312</v>
+        <v>307</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>312</v>
+        <v>307</v>
       </c>
       <c r="D54" s="5" t="s">
         <v>52</v>
@@ -3555,7 +3557,7 @@
         <v>52</v>
       </c>
       <c r="I54" s="5" t="s">
-        <v>312</v>
+        <v>307</v>
       </c>
       <c r="J54" s="5" t="s">
         <v>52</v>
@@ -3691,7 +3693,7 @@
     </row>
     <row r="59" spans="1:10" ht="16" customHeight="1">
       <c r="A59" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B59" s="5">
         <v>32143</v>
@@ -3726,10 +3728,10 @@
         <v>50</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="D60" s="5" t="s">
         <v>52</v>
@@ -3750,7 +3752,7 @@
         <v>52</v>
       </c>
       <c r="J60" s="5" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
     </row>
   </sheetData>
@@ -3774,19 +3776,19 @@
   <sheetData>
     <row r="2" spans="1:5">
       <c r="A2" s="1" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>124</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>293</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="14" customHeight="1">
@@ -3794,16 +3796,16 @@
         <v>0</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="14" customHeight="1">
@@ -3811,16 +3813,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="14" customHeight="1">
@@ -3828,16 +3830,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="14" customHeight="1">
@@ -3845,16 +3847,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="14" customHeight="1">
@@ -3862,33 +3864,33 @@
         <v>4</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="14" customHeight="1">
       <c r="A8" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="14" customHeight="1">
@@ -3896,16 +3898,16 @@
         <v>5</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="14" customHeight="1">
@@ -3913,16 +3915,16 @@
         <v>6</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="14" customHeight="1">
@@ -3930,16 +3932,16 @@
         <v>7</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="14" customHeight="1">
@@ -3947,16 +3949,16 @@
         <v>8</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="14" customHeight="1">
@@ -3964,16 +3966,16 @@
         <v>9</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="14" customHeight="1">
@@ -3981,16 +3983,16 @@
         <v>10</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="14" customHeight="1">
@@ -3998,16 +4000,16 @@
         <v>11</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="D15" s="12" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="14" customHeight="1">
@@ -4015,16 +4017,16 @@
         <v>12</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="14" customHeight="1">
@@ -4032,16 +4034,16 @@
         <v>13</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="14" customHeight="1">
@@ -4049,16 +4051,16 @@
         <v>14</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="14" customHeight="1">
@@ -4066,16 +4068,16 @@
         <v>15</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="E19" s="12" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="14" customHeight="1">
@@ -4083,16 +4085,16 @@
         <v>16</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E20" s="12" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="14" customHeight="1">
@@ -4100,16 +4102,16 @@
         <v>17</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="E21" s="12" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="14" customHeight="1">
@@ -4117,33 +4119,33 @@
         <v>18</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="E22" s="12" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="14" customHeight="1">
       <c r="A23" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="D23" s="12" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="E23" s="12" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="14" customHeight="1">
@@ -4151,16 +4153,16 @@
         <v>19</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="E24" s="12" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="14" customHeight="1">
@@ -4168,16 +4170,16 @@
         <v>20</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="E25" s="12" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="14" customHeight="1">
@@ -4185,16 +4187,16 @@
         <v>21</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="E26" s="12" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="14" customHeight="1">
@@ -4202,16 +4204,16 @@
         <v>22</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="D27" s="12" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="E27" s="12" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="14" customHeight="1">
@@ -4219,16 +4221,16 @@
         <v>23</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="E28" s="12" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="14" customHeight="1">
@@ -4236,16 +4238,16 @@
         <v>24</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="E29" s="12" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="14" customHeight="1">
@@ -4253,16 +4255,16 @@
         <v>25</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="E30" s="12" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="14" customHeight="1">
@@ -4270,16 +4272,16 @@
         <v>26</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E31" s="12" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="14" customHeight="1">
@@ -4287,33 +4289,33 @@
         <v>27</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="D32" s="12" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="E32" s="12" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="14" customHeight="1">
       <c r="A33" s="2" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>323</v>
+        <v>317</v>
       </c>
       <c r="E33" s="12" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="14" customHeight="1">
@@ -4321,16 +4323,16 @@
         <v>28</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="D34" s="12" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="E34" s="12" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="14" customHeight="1">
@@ -4338,16 +4340,16 @@
         <v>29</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="D35" s="12" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="E35" s="12" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="14" customHeight="1">
@@ -4355,16 +4357,16 @@
         <v>30</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="D36" s="12" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="E36" s="12" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="14" customHeight="1">
@@ -4372,16 +4374,16 @@
         <v>31</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="D37" s="12" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="E37" s="12" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="14" customHeight="1">
@@ -4389,16 +4391,16 @@
         <v>32</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D38" s="12" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="E38" s="12" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="14" customHeight="1">
@@ -4406,16 +4408,16 @@
         <v>33</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="E39" s="12" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="14" customHeight="1">
@@ -4423,16 +4425,16 @@
         <v>34</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="D40" s="12" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="E40" s="12" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="14" customHeight="1">
@@ -4440,16 +4442,16 @@
         <v>35</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="D41" s="12" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="E41" s="12" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="14" customHeight="1">
@@ -4457,16 +4459,16 @@
         <v>36</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="D42" s="12" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="E42" s="12" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="14" customHeight="1">
@@ -4474,16 +4476,16 @@
         <v>37</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="E43" s="12" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="14" customHeight="1">
@@ -4491,16 +4493,16 @@
         <v>38</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C44" s="8" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="D44" s="12" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="E44" s="12" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="14" customHeight="1">
@@ -4508,16 +4510,16 @@
         <v>39</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C45" s="8" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="D45" s="12" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="E45" s="12" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="14" customHeight="1">
@@ -4525,33 +4527,33 @@
         <v>51</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C46" s="8" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="D46" s="12" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="E46" s="12" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="14">
       <c r="A47" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C47" s="8" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="D47" s="12" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="E47" s="12" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="48" spans="1:5" ht="14">
@@ -4559,33 +4561,33 @@
         <v>40</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C48" s="8" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="D48" s="12" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="E48" s="12" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="49" spans="1:5" ht="12" customHeight="1">
       <c r="A49" s="2" t="s">
-        <v>320</v>
+        <v>314</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C49" s="8" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="D49" s="12" t="s">
-        <v>324</v>
+        <v>318</v>
       </c>
       <c r="E49" s="12" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="50" spans="1:5" ht="14">
@@ -4593,16 +4595,16 @@
         <v>41</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C50" s="8" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="D50" s="12" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="E50" s="12" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="51" spans="1:5" ht="14">
@@ -4610,16 +4612,16 @@
         <v>42</v>
       </c>
       <c r="B51" s="8" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C51" s="8" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="D51" s="12" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="E51" s="12" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="52" spans="1:5" ht="14">
@@ -4627,16 +4629,16 @@
         <v>43</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C52" s="8" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="D52" s="12" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="E52" s="12" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
     </row>
     <row r="53" spans="1:5" ht="14">
@@ -4644,16 +4646,16 @@
         <v>44</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C53" s="8" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="D53" s="12" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="E53" s="12" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="14">
@@ -4661,33 +4663,33 @@
         <v>45</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C54" s="8" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="D54" s="12" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="E54" s="12" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="55" spans="1:5" ht="14">
       <c r="A55" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C55" s="8" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="D55" s="12" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="E55" s="12" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="56" spans="1:5" ht="14">
@@ -4695,16 +4697,16 @@
         <v>46</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C56" s="8" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="D56" s="12" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="E56" s="12" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="14">
@@ -4712,16 +4714,16 @@
         <v>47</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C57" s="8" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="D57" s="12" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="E57" s="12" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="58" spans="1:5" ht="14">
@@ -4729,16 +4731,16 @@
         <v>48</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C58" s="8" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="D58" s="12" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="E58" s="12" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="14">
@@ -4746,33 +4748,33 @@
         <v>49</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="C59" s="8" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="D59" s="12" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="E59" s="12" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="14">
       <c r="A60" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C60" s="8" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="D60" s="12" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="E60" s="12" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="14">
@@ -4780,16 +4782,16 @@
         <v>50</v>
       </c>
       <c r="B61" s="8" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="C61" s="8" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="D61" s="12" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="E61" s="12" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="70" spans="2:7" ht="14">
@@ -4807,4 +4809,1969 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E9BB519-30E4-0A4A-85E9-3AFB839C193C}">
+  <dimension ref="A1:N60"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.796875" defaultRowHeight="13"/>
+  <cols>
+    <col min="1" max="1" width="31.796875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="32" style="6" customWidth="1"/>
+    <col min="3" max="7" width="17.796875" style="6" customWidth="1"/>
+    <col min="8" max="8" width="19" style="6" customWidth="1"/>
+    <col min="9" max="10" width="17.796875" style="6" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" s="11" customFormat="1" ht="19" customHeight="1">
+      <c r="A1" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>321</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>322</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>323</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" s="11" customFormat="1" ht="19" customHeight="1">
+      <c r="A2" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" ht="30">
+      <c r="A3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>309</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>309</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" ht="16" customHeight="1">
+      <c r="A4" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D4" s="5">
+        <v>25569</v>
+      </c>
+      <c r="E4" s="5">
+        <v>25569</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I4" s="5">
+        <v>32143</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N4" s="14"/>
+    </row>
+    <row r="5" spans="1:14" ht="16" customHeight="1">
+      <c r="A5" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D5" s="5">
+        <v>25569</v>
+      </c>
+      <c r="E5" s="5">
+        <v>25569</v>
+      </c>
+      <c r="F5" s="5">
+        <v>25569</v>
+      </c>
+      <c r="G5" s="5">
+        <v>32143</v>
+      </c>
+      <c r="H5" s="5">
+        <v>32143</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N5" s="14"/>
+    </row>
+    <row r="6" spans="1:14" ht="16" customHeight="1">
+      <c r="A6" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D6" s="5">
+        <v>25569</v>
+      </c>
+      <c r="E6" s="5">
+        <v>25569</v>
+      </c>
+      <c r="F6" s="5">
+        <v>25569</v>
+      </c>
+      <c r="G6" s="5">
+        <v>32143</v>
+      </c>
+      <c r="H6" s="5">
+        <v>32143</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N6" s="14"/>
+    </row>
+    <row r="7" spans="1:14" ht="16" customHeight="1">
+      <c r="A7" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C7" s="5">
+        <v>32143</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J7" s="5">
+        <v>32143</v>
+      </c>
+      <c r="N7" s="14"/>
+    </row>
+    <row r="8" spans="1:14" ht="16" customHeight="1">
+      <c r="A8" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B8" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D8" s="5">
+        <v>25569</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J8" s="5">
+        <v>32143</v>
+      </c>
+      <c r="N8" s="14"/>
+    </row>
+    <row r="9" spans="1:14" ht="16" customHeight="1">
+      <c r="A9" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C9" s="5">
+        <v>32143</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J9" s="5">
+        <v>32143</v>
+      </c>
+      <c r="N9" s="14"/>
+    </row>
+    <row r="10" spans="1:14" ht="16" customHeight="1">
+      <c r="A10" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" s="5">
+        <v>35311</v>
+      </c>
+      <c r="C10" s="5">
+        <v>35311</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I10" s="5">
+        <v>35311</v>
+      </c>
+      <c r="J10" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N10" s="14"/>
+    </row>
+    <row r="11" spans="1:14" ht="16" customHeight="1">
+      <c r="A11" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11" s="5">
+        <v>34367</v>
+      </c>
+      <c r="C11" s="5">
+        <v>34367</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J11" s="5">
+        <v>34367</v>
+      </c>
+      <c r="N11" s="14"/>
+    </row>
+    <row r="12" spans="1:14" ht="16" customHeight="1">
+      <c r="A12" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" s="5">
+        <v>35311</v>
+      </c>
+      <c r="C12" s="5">
+        <v>35311</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H12" s="5">
+        <v>35311</v>
+      </c>
+      <c r="I12" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J12" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N12" s="14"/>
+    </row>
+    <row r="13" spans="1:14" ht="16" customHeight="1">
+      <c r="A13" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D13" s="5">
+        <v>25569</v>
+      </c>
+      <c r="E13" s="5">
+        <v>25569</v>
+      </c>
+      <c r="F13" s="5">
+        <v>25569</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H13" s="5">
+        <v>32143</v>
+      </c>
+      <c r="I13" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J13" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N13" s="14"/>
+    </row>
+    <row r="14" spans="1:14" ht="16" customHeight="1">
+      <c r="A14" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" s="5">
+        <v>37043</v>
+      </c>
+      <c r="C14" s="5">
+        <v>37043</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H14" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I14" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J14" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N14" s="14"/>
+    </row>
+    <row r="15" spans="1:14" ht="16" customHeight="1">
+      <c r="A15" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B15" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D15" s="5">
+        <v>32143</v>
+      </c>
+      <c r="E15" s="5">
+        <v>32143</v>
+      </c>
+      <c r="F15" s="5">
+        <v>32143</v>
+      </c>
+      <c r="G15" s="5">
+        <v>32143</v>
+      </c>
+      <c r="H15" s="5">
+        <v>32143</v>
+      </c>
+      <c r="I15" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J15" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N15" s="14"/>
+    </row>
+    <row r="16" spans="1:14" ht="16" customHeight="1">
+      <c r="A16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B16" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D16" s="5">
+        <v>25569</v>
+      </c>
+      <c r="E16" s="5">
+        <v>25569</v>
+      </c>
+      <c r="F16" s="5">
+        <v>25569</v>
+      </c>
+      <c r="G16" s="5">
+        <v>32143</v>
+      </c>
+      <c r="H16" s="5">
+        <v>32143</v>
+      </c>
+      <c r="I16" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J16" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N16" s="14"/>
+    </row>
+    <row r="17" spans="1:14" ht="16" customHeight="1">
+      <c r="A17" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B17" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D17" s="5">
+        <v>25569</v>
+      </c>
+      <c r="E17" s="5">
+        <v>25569</v>
+      </c>
+      <c r="F17" s="5">
+        <v>25569</v>
+      </c>
+      <c r="G17" s="5">
+        <v>32143</v>
+      </c>
+      <c r="H17" s="5">
+        <v>32143</v>
+      </c>
+      <c r="I17" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J17" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N17" s="14"/>
+    </row>
+    <row r="18" spans="1:14" ht="16" customHeight="1">
+      <c r="A18" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B18" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>310</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>298</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>298</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>298</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>298</v>
+      </c>
+      <c r="H18" s="5">
+        <v>32143</v>
+      </c>
+      <c r="I18" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J18" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N18" s="14"/>
+    </row>
+    <row r="19" spans="1:14" ht="16" customHeight="1">
+      <c r="A19" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B19" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D19" s="5">
+        <v>26634</v>
+      </c>
+      <c r="E19" s="5">
+        <v>26634</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G19" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H19" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I19" s="5">
+        <v>32143</v>
+      </c>
+      <c r="J19" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N19" s="14"/>
+    </row>
+    <row r="20" spans="1:14" ht="16" customHeight="1">
+      <c r="A20" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B20" s="5">
+        <v>35311</v>
+      </c>
+      <c r="C20" s="5">
+        <v>35311</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G20" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H20" s="5">
+        <v>35311</v>
+      </c>
+      <c r="I20" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J20" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N20" s="14"/>
+    </row>
+    <row r="21" spans="1:14" ht="16" customHeight="1">
+      <c r="A21" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B21" s="5">
+        <v>34367</v>
+      </c>
+      <c r="C21" s="5">
+        <v>34367</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G21" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H21" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I21" s="5">
+        <v>34367</v>
+      </c>
+      <c r="J21" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N21" s="14"/>
+    </row>
+    <row r="22" spans="1:14" ht="16" customHeight="1">
+      <c r="A22" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B22" s="5">
+        <v>32752</v>
+      </c>
+      <c r="C22" s="5">
+        <v>32752</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F22" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G22" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H22" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I22" s="5">
+        <v>32752</v>
+      </c>
+      <c r="J22" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N22" s="14"/>
+    </row>
+    <row r="23" spans="1:14" ht="16" customHeight="1">
+      <c r="A23" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B23" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D23" s="5">
+        <v>34092</v>
+      </c>
+      <c r="E23" s="5">
+        <v>34092</v>
+      </c>
+      <c r="F23" s="5">
+        <v>34092</v>
+      </c>
+      <c r="G23" s="5">
+        <v>34092</v>
+      </c>
+      <c r="H23" s="5">
+        <v>32143</v>
+      </c>
+      <c r="I23" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J23" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N23" s="14"/>
+    </row>
+    <row r="24" spans="1:14" ht="16" customHeight="1">
+      <c r="A24" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B24" s="5">
+        <v>34367</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>299</v>
+      </c>
+      <c r="D24" s="5">
+        <v>40325</v>
+      </c>
+      <c r="E24" s="5">
+        <v>40325</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G24" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H24" s="5">
+        <v>34760</v>
+      </c>
+      <c r="I24" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J24" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N24" s="14"/>
+    </row>
+    <row r="25" spans="1:14" ht="16" customHeight="1">
+      <c r="A25" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B25" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D25" s="5">
+        <v>25569</v>
+      </c>
+      <c r="E25" s="5">
+        <v>25569</v>
+      </c>
+      <c r="F25" s="5">
+        <v>25569</v>
+      </c>
+      <c r="G25" s="5">
+        <v>32143</v>
+      </c>
+      <c r="H25" s="5">
+        <v>32143</v>
+      </c>
+      <c r="I25" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J25" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N25" s="14"/>
+    </row>
+    <row r="26" spans="1:14" ht="16" customHeight="1">
+      <c r="A26" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B26" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D26" s="5">
+        <v>25569</v>
+      </c>
+      <c r="E26" s="5">
+        <v>25569</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G26" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H26" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I26" s="5">
+        <v>32143</v>
+      </c>
+      <c r="J26" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N26" s="14"/>
+    </row>
+    <row r="27" spans="1:14" ht="16" customHeight="1">
+      <c r="A27" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>300</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>300</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G27" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H27" s="5" t="s">
+        <v>300</v>
+      </c>
+      <c r="I27" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J27" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N27" s="14"/>
+    </row>
+    <row r="28" spans="1:14" ht="16" customHeight="1">
+      <c r="A28" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B28" s="5">
+        <v>33610</v>
+      </c>
+      <c r="C28" s="5">
+        <v>33610</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G28" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H28" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I28" s="5">
+        <v>33610</v>
+      </c>
+      <c r="J28" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" ht="16" customHeight="1">
+      <c r="A29" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B29" s="5">
+        <v>44166</v>
+      </c>
+      <c r="C29" s="5">
+        <v>44166</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G29" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H29" s="5">
+        <v>44166</v>
+      </c>
+      <c r="I29" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J29" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" ht="16" customHeight="1">
+      <c r="A30" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>301</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F30" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G30" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H30" s="5" t="s">
+        <v>301</v>
+      </c>
+      <c r="I30" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J30" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" ht="16" customHeight="1">
+      <c r="A31" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>302</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>302</v>
+      </c>
+      <c r="F31" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G31" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H31" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I31" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="J31" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" ht="16" customHeight="1">
+      <c r="A32" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B32" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C32" s="5">
+        <v>32143</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F32" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G32" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H32" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I32" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J32" s="5">
+        <v>32143</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="16" customHeight="1">
+      <c r="A33" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>303</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F33" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G33" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H33" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I33" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J33" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="16" customHeight="1">
+      <c r="A34" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>298</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>298</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F34" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G34" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H34" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I34" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J34" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="16" customHeight="1">
+      <c r="A35" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B35" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D35" s="5">
+        <v>25569</v>
+      </c>
+      <c r="E35" s="5">
+        <v>25569</v>
+      </c>
+      <c r="F35" s="5">
+        <v>25569</v>
+      </c>
+      <c r="G35" s="5">
+        <v>32143</v>
+      </c>
+      <c r="H35" s="5">
+        <v>32143</v>
+      </c>
+      <c r="I35" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J35" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" ht="16" customHeight="1">
+      <c r="A36" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B36" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D36" s="5">
+        <v>32143</v>
+      </c>
+      <c r="E36" s="5">
+        <v>32143</v>
+      </c>
+      <c r="F36" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G36" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H36" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I36" s="5">
+        <v>32143</v>
+      </c>
+      <c r="J36" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" ht="16" customHeight="1">
+      <c r="A37" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B37" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D37" s="5">
+        <v>25569</v>
+      </c>
+      <c r="E37" s="5">
+        <v>25569</v>
+      </c>
+      <c r="F37" s="5">
+        <v>25569</v>
+      </c>
+      <c r="G37" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H37" s="5">
+        <v>32143</v>
+      </c>
+      <c r="I37" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J37" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" ht="16" customHeight="1">
+      <c r="A38" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="D38" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E38" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F38" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G38" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H38" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I38" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="J38" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" ht="16" customHeight="1">
+      <c r="A39" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B39" s="5">
+        <v>34367</v>
+      </c>
+      <c r="C39" s="5">
+        <v>34367</v>
+      </c>
+      <c r="D39" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E39" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F39" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G39" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H39" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I39" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J39" s="5">
+        <v>34367</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" ht="16" customHeight="1">
+      <c r="A40" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B40" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C40" s="5">
+        <v>32143</v>
+      </c>
+      <c r="D40" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E40" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F40" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G40" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H40" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I40" s="5">
+        <v>32143</v>
+      </c>
+      <c r="J40" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" ht="16" customHeight="1">
+      <c r="A41" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B41" s="5">
+        <v>34760</v>
+      </c>
+      <c r="C41" s="5">
+        <v>34760</v>
+      </c>
+      <c r="D41" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E41" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F41" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G41" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H41" s="5">
+        <v>34760</v>
+      </c>
+      <c r="I41" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J41" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" ht="16" customHeight="1">
+      <c r="A42" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B42" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>304</v>
+      </c>
+      <c r="D42" s="5">
+        <v>35765</v>
+      </c>
+      <c r="E42" s="5">
+        <v>35765</v>
+      </c>
+      <c r="F42" s="5">
+        <v>35765</v>
+      </c>
+      <c r="G42" s="5">
+        <v>35765</v>
+      </c>
+      <c r="H42" s="5">
+        <v>32143</v>
+      </c>
+      <c r="I42" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J42" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" ht="16" customHeight="1">
+      <c r="A43" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B43" s="5">
+        <v>41792</v>
+      </c>
+      <c r="C43" s="5">
+        <v>41792</v>
+      </c>
+      <c r="D43" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E43" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F43" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G43" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H43" s="5">
+        <v>41792</v>
+      </c>
+      <c r="I43" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J43" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" ht="16" customHeight="1">
+      <c r="A44" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B44" s="5" t="s">
+        <v>305</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>305</v>
+      </c>
+      <c r="D44" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E44" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F44" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G44" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H44" s="5" t="s">
+        <v>305</v>
+      </c>
+      <c r="I44" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J44" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" ht="16" customHeight="1">
+      <c r="A45" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B45" s="5">
+        <v>43614</v>
+      </c>
+      <c r="C45" s="5">
+        <v>43614</v>
+      </c>
+      <c r="D45" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E45" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F45" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G45" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H45" s="5">
+        <v>43614</v>
+      </c>
+      <c r="I45" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J45" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" ht="16" customHeight="1">
+      <c r="A46" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B46" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C46" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D46" s="5">
+        <v>26634</v>
+      </c>
+      <c r="E46" s="5">
+        <v>26634</v>
+      </c>
+      <c r="F46" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G46" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H46" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I46" s="5">
+        <v>32143</v>
+      </c>
+      <c r="J46" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" ht="16" customHeight="1">
+      <c r="A47" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B47" s="5">
+        <v>34760</v>
+      </c>
+      <c r="C47" s="5">
+        <v>34760</v>
+      </c>
+      <c r="D47" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E47" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F47" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G47" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H47" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I47" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J47" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" ht="16" customHeight="1">
+      <c r="A48" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D48" s="5" t="s">
+        <v>313</v>
+      </c>
+      <c r="E48" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F48" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G48" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H48" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I48" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J48" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" ht="16" customHeight="1">
+      <c r="A49" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B49" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C49" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D49" s="5">
+        <v>25569</v>
+      </c>
+      <c r="E49" s="5">
+        <v>25569</v>
+      </c>
+      <c r="F49" s="5">
+        <v>25569</v>
+      </c>
+      <c r="G49" s="5">
+        <v>32143</v>
+      </c>
+      <c r="H49" s="5">
+        <v>32143</v>
+      </c>
+      <c r="I49" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J49" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" ht="16" customHeight="1">
+      <c r="A50" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B50" s="5" t="s">
+        <v>306</v>
+      </c>
+      <c r="C50" s="5" t="s">
+        <v>306</v>
+      </c>
+      <c r="D50" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E50" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F50" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G50" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H50" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I50" s="5" t="s">
+        <v>306</v>
+      </c>
+      <c r="J50" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" ht="16" customHeight="1">
+      <c r="A51" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B51" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C51" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D51" s="5">
+        <v>25569</v>
+      </c>
+      <c r="E51" s="5">
+        <v>25569</v>
+      </c>
+      <c r="F51" s="5">
+        <v>25569</v>
+      </c>
+      <c r="G51" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H51" s="5">
+        <v>32143</v>
+      </c>
+      <c r="I51" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J51" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" ht="16" customHeight="1">
+      <c r="A52" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B52" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C52" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D52" s="5">
+        <v>25569</v>
+      </c>
+      <c r="E52" s="5">
+        <v>25569</v>
+      </c>
+      <c r="F52" s="5">
+        <v>25569</v>
+      </c>
+      <c r="G52" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H52" s="5">
+        <v>32143</v>
+      </c>
+      <c r="I52" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J52" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" ht="16" customHeight="1">
+      <c r="A53" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B53" s="5">
+        <v>37410</v>
+      </c>
+      <c r="C53" s="5">
+        <v>37410</v>
+      </c>
+      <c r="D53" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E53" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F53" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G53" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H53" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I53" s="5">
+        <v>37410</v>
+      </c>
+      <c r="J53" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" ht="16" customHeight="1">
+      <c r="A54" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="B54" s="5" t="s">
+        <v>307</v>
+      </c>
+      <c r="C54" s="5" t="s">
+        <v>307</v>
+      </c>
+      <c r="D54" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E54" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F54" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G54" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H54" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I54" s="5" t="s">
+        <v>307</v>
+      </c>
+      <c r="J54" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" ht="16" customHeight="1">
+      <c r="A55" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B55" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C55" s="5">
+        <v>32143</v>
+      </c>
+      <c r="D55" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E55" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F55" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G55" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H55" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I55" s="5">
+        <v>32143</v>
+      </c>
+      <c r="J55" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" ht="16" customHeight="1">
+      <c r="A56" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B56" s="5">
+        <v>32752</v>
+      </c>
+      <c r="C56" s="5">
+        <v>32752</v>
+      </c>
+      <c r="D56" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E56" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F56" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G56" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H56" s="5">
+        <v>35339</v>
+      </c>
+      <c r="I56" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J56" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" ht="16" customHeight="1">
+      <c r="A57" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B57" s="5">
+        <v>41792</v>
+      </c>
+      <c r="C57" s="5">
+        <v>41792</v>
+      </c>
+      <c r="D57" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E57" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F57" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G57" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H57" s="5">
+        <v>41792</v>
+      </c>
+      <c r="I57" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J57" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" ht="16" customHeight="1">
+      <c r="A58" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B58" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C58" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D58" s="5">
+        <v>25569</v>
+      </c>
+      <c r="E58" s="5">
+        <v>25569</v>
+      </c>
+      <c r="F58" s="5">
+        <v>25569</v>
+      </c>
+      <c r="G58" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H58" s="5">
+        <v>32143</v>
+      </c>
+      <c r="I58" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J58" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" ht="16" customHeight="1">
+      <c r="A59" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B59" s="5">
+        <v>32143</v>
+      </c>
+      <c r="C59" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D59" s="5">
+        <v>25569</v>
+      </c>
+      <c r="E59" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F59" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G59" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H59" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I59" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J59" s="5">
+        <v>32143</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" ht="16" customHeight="1">
+      <c r="A60" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B60" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="C60" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="D60" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E60" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F60" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G60" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H60" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I60" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J60" s="5" t="s">
+        <v>308</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A54" r:id="rId1" xr:uid="{D35FBA93-2E12-9A49-B1F7-6AB790D3B523}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
extend factor manager for constructed and database related factor series
</commit_message>
<xml_diff>
--- a/epsilon-phi-core/src/resources/templates/MSCI Index Construction.xlsx
+++ b/epsilon-phi-core/src/resources/templates/MSCI Index Construction.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11008"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11028"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/francisbarker/Repositories/Python/epsilon-phi/epsilon-phi-core/src/resources/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFB85C0E-BAD2-6D4A-8462-FE4C4E42E6DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FC6A07D-DF23-9147-BF18-0A936BA28C8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57600" yWindow="-9000" windowWidth="67200" windowHeight="37800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="57600" windowHeight="30000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rules" sheetId="40" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1138" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1492" uniqueCount="341">
   <si>
     <r>
       <rPr>
@@ -1382,6 +1382,54 @@
   <si>
     <t>AC Americas</t>
   </si>
+  <si>
+    <t>Pacific</t>
+  </si>
+  <si>
+    <t>Pacific ex-Japan</t>
+  </si>
+  <si>
+    <t>Europe ex-UK</t>
+  </si>
+  <si>
+    <t>EM Europe and Middle East</t>
+  </si>
+  <si>
+    <t>EM Europe</t>
+  </si>
+  <si>
+    <t>Emerging Markets</t>
+  </si>
+  <si>
+    <t>EM Latin America</t>
+  </si>
+  <si>
+    <t>MSGEUX$</t>
+  </si>
+  <si>
+    <t>MSEMFA$</t>
+  </si>
+  <si>
+    <t>EM Asia</t>
+  </si>
+  <si>
+    <t>MSEEUR$</t>
+  </si>
+  <si>
+    <t>MSEMEA$</t>
+  </si>
+  <si>
+    <t>MSEMUI$</t>
+  </si>
+  <si>
+    <t>MSPXJP$</t>
+  </si>
+  <si>
+    <t>MSPACF$</t>
+  </si>
+  <si>
+    <t>MSEFLA$</t>
+  </si>
 </sst>
 </file>
 
@@ -1390,7 +1438,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-809]dd\ mmmm\ yyyy;@"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1435,6 +1483,11 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Inherit"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -1827,15 +1880,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{398A9000-FE9A-0D49-BC15-66DEE1B3B201}">
-  <dimension ref="A1:J60"/>
+  <dimension ref="A1:Q60"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.796875" defaultRowHeight="13"/>
   <cols>
     <col min="1" max="1" width="31.796875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="32" style="6" customWidth="1"/>
-    <col min="3" max="10" width="17.796875" style="6" customWidth="1"/>
+    <col min="2" max="17" width="14.59765625" style="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="11" customFormat="1" ht="19" customHeight="1">
+    <row r="1" spans="1:17" s="11" customFormat="1" ht="20">
       <c r="A1" s="10" t="s">
         <v>120</v>
       </c>
@@ -1843,7 +1895,7 @@
         <v>321</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>53</v>
+        <v>330</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>319</v>
@@ -1855,19 +1907,40 @@
         <v>320</v>
       </c>
       <c r="G1" s="4" t="s">
+        <v>327</v>
+      </c>
+      <c r="H1" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>322</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="J1" s="4" t="s">
+        <v>328</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>329</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>334</v>
+      </c>
+      <c r="M1" s="4" t="s">
         <v>323</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="N1" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="O1" s="4" t="s">
+        <v>326</v>
+      </c>
+      <c r="P1" s="4" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" s="11" customFormat="1" ht="19" customHeight="1">
+      <c r="Q1" s="4" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" s="11" customFormat="1" ht="19" customHeight="1">
       <c r="A2" s="10" t="s">
         <v>121</v>
       </c>
@@ -1887,19 +1960,40 @@
         <v>115</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>116</v>
+        <v>332</v>
       </c>
       <c r="H2" s="4" t="s">
+        <v>337</v>
+      </c>
+      <c r="I2" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="J2" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>335</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="M2" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="N2" s="4" t="s">
+        <v>339</v>
+      </c>
+      <c r="O2" s="4" t="s">
+        <v>338</v>
+      </c>
+      <c r="P2" s="4" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" ht="30">
+      <c r="Q2" s="4" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" ht="30">
       <c r="A3" s="2" t="s">
         <v>0</v>
       </c>
@@ -1928,10 +2022,31 @@
         <v>52</v>
       </c>
       <c r="J3" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O3" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P3" s="5" t="s">
         <v>309</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" ht="16" customHeight="1">
+      <c r="Q3" s="5" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" ht="16" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>1</v>
       </c>
@@ -1956,14 +2071,35 @@
       <c r="H4" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="I4" s="5">
-        <v>32143</v>
+      <c r="I4" s="5" t="s">
+        <v>52</v>
       </c>
       <c r="J4" s="5" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" ht="16" customHeight="1">
+      <c r="K4" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M4" s="5">
+        <v>32143</v>
+      </c>
+      <c r="N4" s="5">
+        <v>32143</v>
+      </c>
+      <c r="O4" s="5">
+        <v>32143</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q4" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" ht="16" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>2</v>
       </c>
@@ -1983,19 +2119,40 @@
         <v>25569</v>
       </c>
       <c r="G5" s="5">
-        <v>32143</v>
+        <v>25569</v>
       </c>
       <c r="H5" s="5">
         <v>32143</v>
       </c>
-      <c r="I5" s="5" t="s">
-        <v>52</v>
+      <c r="I5" s="5">
+        <v>32143</v>
       </c>
       <c r="J5" s="5" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" ht="16" customHeight="1">
+      <c r="K5" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O5" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P5" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q5" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" ht="16" customHeight="1">
       <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
@@ -2015,19 +2172,40 @@
         <v>25569</v>
       </c>
       <c r="G6" s="5">
-        <v>32143</v>
+        <v>25569</v>
       </c>
       <c r="H6" s="5">
         <v>32143</v>
       </c>
-      <c r="I6" s="5" t="s">
-        <v>52</v>
+      <c r="I6" s="5">
+        <v>32143</v>
       </c>
       <c r="J6" s="5" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" ht="16" customHeight="1">
+      <c r="K6" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N6" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O6" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P6" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q6" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" ht="16" customHeight="1">
       <c r="A7" s="2" t="s">
         <v>4</v>
       </c>
@@ -2055,11 +2233,32 @@
       <c r="I7" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="J7" s="5">
-        <v>32143</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="16" customHeight="1">
+      <c r="J7" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L7" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M7" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N7" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O7" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P7" s="5">
+        <v>32143</v>
+      </c>
+      <c r="Q7" s="5">
+        <v>32143</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" ht="16" customHeight="1">
       <c r="A8" s="3" t="s">
         <v>56</v>
       </c>
@@ -2087,11 +2286,32 @@
       <c r="I8" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="J8" s="5">
-        <v>32143</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="16" customHeight="1">
+      <c r="J8" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L8" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M8" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N8" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O8" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P8" s="5">
+        <v>32143</v>
+      </c>
+      <c r="Q8" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" ht="16" customHeight="1">
       <c r="A9" s="2" t="s">
         <v>5</v>
       </c>
@@ -2119,11 +2339,32 @@
       <c r="I9" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="J9" s="5">
-        <v>32143</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="16" customHeight="1">
+      <c r="J9" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L9" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M9" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N9" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O9" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P9" s="5">
+        <v>32143</v>
+      </c>
+      <c r="Q9" s="5">
+        <v>32143</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" ht="16" customHeight="1">
       <c r="A10" s="2" t="s">
         <v>6</v>
       </c>
@@ -2148,14 +2389,35 @@
       <c r="H10" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="I10" s="5">
+      <c r="I10" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J10" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L10" s="5">
         <v>35311</v>
       </c>
-      <c r="J10" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="16" customHeight="1">
+      <c r="M10" s="5">
+        <v>35311</v>
+      </c>
+      <c r="N10" s="5">
+        <v>35311</v>
+      </c>
+      <c r="O10" s="5">
+        <v>35311</v>
+      </c>
+      <c r="P10" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q10" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" ht="16" customHeight="1">
       <c r="A11" s="2" t="s">
         <v>7</v>
       </c>
@@ -2183,11 +2445,32 @@
       <c r="I11" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="J11" s="5">
+      <c r="J11" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L11" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M11" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N11" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O11" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P11" s="5">
         <v>34367</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" ht="16" customHeight="1">
+      <c r="Q11" s="5">
+        <v>34367</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" ht="16" customHeight="1">
       <c r="A12" s="2" t="s">
         <v>8</v>
       </c>
@@ -2209,17 +2492,39 @@
       <c r="G12" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="H12" s="5">
+      <c r="H12" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I12" s="5">
         <v>35311</v>
       </c>
-      <c r="I12" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="J12" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="16" customHeight="1">
+      <c r="J12" s="5">
+        <v>35311</v>
+      </c>
+      <c r="K12" s="5">
+        <f>C12</f>
+        <v>35311</v>
+      </c>
+      <c r="L12" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M12" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N12" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O12" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P12" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q12" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" ht="16" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>9</v>
       </c>
@@ -2238,20 +2543,41 @@
       <c r="F13" s="5">
         <v>25569</v>
       </c>
-      <c r="G13" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="H13" s="5">
-        <v>32143</v>
-      </c>
-      <c r="I13" s="5" t="s">
-        <v>52</v>
+      <c r="G13" s="5">
+        <v>25569</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I13" s="5">
+        <v>32143</v>
       </c>
       <c r="J13" s="5" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="14" spans="1:10" ht="16" customHeight="1">
+      <c r="K13" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L13" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M13" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N13" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O13" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P13" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q13" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" ht="16" customHeight="1">
       <c r="A14" s="2" t="s">
         <v>10</v>
       </c>
@@ -2282,8 +2608,29 @@
       <c r="J14" s="5" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="15" spans="1:10" ht="16" customHeight="1">
+      <c r="K14" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L14" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M14" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N14" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O14" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P14" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q14" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" ht="16" customHeight="1">
       <c r="A15" s="2" t="s">
         <v>11</v>
       </c>
@@ -2308,14 +2655,35 @@
       <c r="H15" s="5">
         <v>32143</v>
       </c>
-      <c r="I15" s="5" t="s">
-        <v>52</v>
+      <c r="I15" s="5">
+        <v>32143</v>
       </c>
       <c r="J15" s="5" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" ht="16" customHeight="1">
+      <c r="K15" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L15" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M15" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N15" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O15" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P15" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q15" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" ht="16" customHeight="1">
       <c r="A16" s="2" t="s">
         <v>12</v>
       </c>
@@ -2335,19 +2703,40 @@
         <v>25569</v>
       </c>
       <c r="G16" s="5">
-        <v>32143</v>
+        <v>25569</v>
       </c>
       <c r="H16" s="5">
         <v>32143</v>
       </c>
-      <c r="I16" s="5" t="s">
-        <v>52</v>
+      <c r="I16" s="5">
+        <v>32143</v>
       </c>
       <c r="J16" s="5" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" ht="16" customHeight="1">
+      <c r="K16" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L16" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M16" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N16" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O16" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P16" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q16" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" ht="16" customHeight="1">
       <c r="A17" s="2" t="s">
         <v>13</v>
       </c>
@@ -2367,19 +2756,40 @@
         <v>25569</v>
       </c>
       <c r="G17" s="5">
-        <v>32143</v>
+        <v>25569</v>
       </c>
       <c r="H17" s="5">
         <v>32143</v>
       </c>
-      <c r="I17" s="5" t="s">
-        <v>52</v>
+      <c r="I17" s="5">
+        <v>32143</v>
       </c>
       <c r="J17" s="5" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" ht="16" customHeight="1">
+      <c r="K17" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L17" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M17" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N17" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O17" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P17" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q17" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" ht="16" customHeight="1">
       <c r="A18" s="2" t="s">
         <v>14</v>
       </c>
@@ -2401,17 +2811,39 @@
       <c r="G18" s="5" t="s">
         <v>298</v>
       </c>
-      <c r="H18" s="5">
-        <v>32143</v>
-      </c>
-      <c r="I18" s="5" t="s">
-        <v>52</v>
+      <c r="H18" s="5" t="s">
+        <v>298</v>
+      </c>
+      <c r="I18" s="5">
+        <v>32143</v>
       </c>
       <c r="J18" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" ht="16" customHeight="1">
+        <v>310</v>
+      </c>
+      <c r="K18" s="5" t="str">
+        <f>C18</f>
+        <v>1-Jan-1988 to 31-May-2001, 27-Nov-2013</v>
+      </c>
+      <c r="L18" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M18" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N18" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O18" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P18" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q18" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" ht="16" customHeight="1">
       <c r="A19" s="2" t="s">
         <v>15</v>
       </c>
@@ -2436,14 +2868,35 @@
       <c r="H19" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="I19" s="5">
-        <v>32143</v>
+      <c r="I19" s="5" t="s">
+        <v>52</v>
       </c>
       <c r="J19" s="5" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="20" spans="1:10" ht="16" customHeight="1">
+      <c r="K19" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L19" s="5">
+        <v>32143</v>
+      </c>
+      <c r="M19" s="5">
+        <v>32143</v>
+      </c>
+      <c r="N19" s="5">
+        <v>32143</v>
+      </c>
+      <c r="O19" s="5">
+        <v>32143</v>
+      </c>
+      <c r="P19" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q19" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" ht="16" customHeight="1">
       <c r="A20" s="2" t="s">
         <v>16</v>
       </c>
@@ -2465,17 +2918,39 @@
       <c r="G20" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="H20" s="5">
+      <c r="H20" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I20" s="5">
         <v>35311</v>
       </c>
-      <c r="I20" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="J20" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" ht="16" customHeight="1">
+      <c r="J20" s="5">
+        <v>35311</v>
+      </c>
+      <c r="K20" s="5">
+        <f>C20</f>
+        <v>35311</v>
+      </c>
+      <c r="L20" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M20" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N20" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O20" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P20" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q20" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" ht="16" customHeight="1">
       <c r="A21" s="2" t="s">
         <v>17</v>
       </c>
@@ -2500,14 +2975,35 @@
       <c r="H21" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="I21" s="5">
+      <c r="I21" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J21" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="K21" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L21" s="5">
         <v>34367</v>
       </c>
-      <c r="J21" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" ht="16" customHeight="1">
+      <c r="M21" s="5">
+        <v>34367</v>
+      </c>
+      <c r="N21" s="5">
+        <v>34367</v>
+      </c>
+      <c r="O21" s="5">
+        <v>34367</v>
+      </c>
+      <c r="P21" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q21" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" ht="16" customHeight="1">
       <c r="A22" s="2" t="s">
         <v>18</v>
       </c>
@@ -2532,14 +3028,35 @@
       <c r="H22" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="I22" s="5">
+      <c r="I22" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J22" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="K22" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L22" s="5">
         <v>32752</v>
       </c>
-      <c r="J22" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" ht="16" customHeight="1">
+      <c r="M22" s="5">
+        <v>32752</v>
+      </c>
+      <c r="N22" s="5">
+        <v>32752</v>
+      </c>
+      <c r="O22" s="5">
+        <v>32752</v>
+      </c>
+      <c r="P22" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q22" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" ht="16" customHeight="1">
       <c r="A23" s="3" t="s">
         <v>57</v>
       </c>
@@ -2562,16 +3079,37 @@
         <v>34092</v>
       </c>
       <c r="H23" s="5">
-        <v>32143</v>
-      </c>
-      <c r="I23" s="5" t="s">
-        <v>52</v>
+        <v>34092</v>
+      </c>
+      <c r="I23" s="5">
+        <v>32143</v>
       </c>
       <c r="J23" s="5" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="24" spans="1:10" ht="16" customHeight="1">
+      <c r="K23" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L23" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M23" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N23" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O23" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P23" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q23" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" ht="16" customHeight="1">
       <c r="A24" s="2" t="s">
         <v>19</v>
       </c>
@@ -2593,17 +3131,38 @@
       <c r="G24" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="H24" s="5">
+      <c r="H24" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I24" s="5">
         <v>34760</v>
       </c>
-      <c r="I24" s="5" t="s">
-        <v>52</v>
-      </c>
       <c r="J24" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" ht="16" customHeight="1">
+        <v>299</v>
+      </c>
+      <c r="K24" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L24" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M24" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N24" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O24" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P24" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q24" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" ht="16" customHeight="1">
       <c r="A25" s="2" t="s">
         <v>20</v>
       </c>
@@ -2623,19 +3182,40 @@
         <v>25569</v>
       </c>
       <c r="G25" s="5">
-        <v>32143</v>
+        <v>25569</v>
       </c>
       <c r="H25" s="5">
         <v>32143</v>
       </c>
-      <c r="I25" s="5" t="s">
-        <v>52</v>
+      <c r="I25" s="5">
+        <v>32143</v>
       </c>
       <c r="J25" s="5" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="26" spans="1:10" ht="16" customHeight="1">
+      <c r="K25" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L25" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M25" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N25" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O25" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P25" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q25" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" ht="16" customHeight="1">
       <c r="A26" s="2" t="s">
         <v>21</v>
       </c>
@@ -2660,14 +3240,35 @@
       <c r="H26" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="I26" s="5">
-        <v>32143</v>
+      <c r="I26" s="5" t="s">
+        <v>52</v>
       </c>
       <c r="J26" s="5" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="27" spans="1:10" ht="16" customHeight="1">
+      <c r="K26" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L26" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M26" s="5">
+        <v>32143</v>
+      </c>
+      <c r="N26" s="5">
+        <v>32143</v>
+      </c>
+      <c r="O26" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P26" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q26" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" ht="16" customHeight="1">
       <c r="A27" s="2" t="s">
         <v>22</v>
       </c>
@@ -2690,16 +3291,37 @@
         <v>52</v>
       </c>
       <c r="H27" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I27" s="5" t="s">
         <v>300</v>
       </c>
-      <c r="I27" s="5" t="s">
-        <v>52</v>
-      </c>
       <c r="J27" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" ht="16" customHeight="1">
+        <v>300</v>
+      </c>
+      <c r="K27" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L27" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M27" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N27" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O27" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P27" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q27" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" ht="16" customHeight="1">
       <c r="A28" s="2" t="s">
         <v>23</v>
       </c>
@@ -2724,14 +3346,35 @@
       <c r="H28" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="I28" s="5">
+      <c r="I28" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J28" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="K28" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L28" s="5">
         <v>33610</v>
       </c>
-      <c r="J28" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" ht="16" customHeight="1">
+      <c r="M28" s="5">
+        <v>33610</v>
+      </c>
+      <c r="N28" s="5">
+        <v>33610</v>
+      </c>
+      <c r="O28" s="5">
+        <v>33610</v>
+      </c>
+      <c r="P28" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q28" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17" ht="16" customHeight="1">
       <c r="A29" s="2" t="s">
         <v>24</v>
       </c>
@@ -2753,17 +3396,38 @@
       <c r="G29" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="H29" s="5">
+      <c r="H29" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I29" s="5">
         <v>44166</v>
       </c>
-      <c r="I29" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="J29" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" ht="16" customHeight="1">
+      <c r="J29" s="5">
+        <v>44166</v>
+      </c>
+      <c r="K29" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L29" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M29" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N29" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O29" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P29" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q29" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17" ht="16" customHeight="1">
       <c r="A30" s="3" t="s">
         <v>297</v>
       </c>
@@ -2786,7 +3450,7 @@
         <v>52</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>301</v>
+        <v>52</v>
       </c>
       <c r="I30" s="5" t="s">
         <v>52</v>
@@ -2794,8 +3458,29 @@
       <c r="J30" s="5" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="31" spans="1:10" ht="16" customHeight="1">
+      <c r="K30" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L30" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M30" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N30" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O30" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P30" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q30" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17" ht="16" customHeight="1">
       <c r="A31" s="2" t="s">
         <v>26</v>
       </c>
@@ -2821,13 +3506,32 @@
         <v>52</v>
       </c>
       <c r="I31" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J31" s="5"/>
+      <c r="K31" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L31" s="5" t="s">
         <v>311</v>
       </c>
-      <c r="J31" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" ht="16" customHeight="1">
+      <c r="M31" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="N31" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="O31" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="P31" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q31" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17" ht="16" customHeight="1">
       <c r="A32" s="2" t="s">
         <v>27</v>
       </c>
@@ -2855,11 +3559,32 @@
       <c r="I32" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="J32" s="5">
-        <v>32143</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" ht="16" customHeight="1">
+      <c r="J32" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="K32" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L32" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M32" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N32" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O32" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P32" s="5">
+        <v>32143</v>
+      </c>
+      <c r="Q32" s="5">
+        <v>32143</v>
+      </c>
+    </row>
+    <row r="33" spans="1:17" ht="16" customHeight="1">
       <c r="A33" s="2" t="s">
         <v>315</v>
       </c>
@@ -2890,8 +3615,29 @@
       <c r="J33" s="5" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="34" spans="1:10" ht="16" customHeight="1">
+      <c r="K33" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L33" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M33" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N33" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O33" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P33" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q33" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="34" spans="1:17" ht="16" customHeight="1">
       <c r="A34" s="2" t="s">
         <v>28</v>
       </c>
@@ -2922,8 +3668,29 @@
       <c r="J34" s="5" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="35" spans="1:10" ht="16" customHeight="1">
+      <c r="K34" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L34" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M34" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N34" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O34" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P34" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q34" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="35" spans="1:17" ht="16" customHeight="1">
       <c r="A35" s="2" t="s">
         <v>29</v>
       </c>
@@ -2943,19 +3710,40 @@
         <v>25569</v>
       </c>
       <c r="G35" s="5">
-        <v>32143</v>
+        <v>25569</v>
       </c>
       <c r="H35" s="5">
         <v>32143</v>
       </c>
-      <c r="I35" s="5" t="s">
-        <v>52</v>
+      <c r="I35" s="5">
+        <v>32143</v>
       </c>
       <c r="J35" s="5" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="36" spans="1:10" ht="16" customHeight="1">
+      <c r="K35" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L35" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M35" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N35" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O35" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P35" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q35" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="36" spans="1:17" ht="16" customHeight="1">
       <c r="A36" s="2" t="s">
         <v>30</v>
       </c>
@@ -2980,14 +3768,35 @@
       <c r="H36" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="I36" s="5">
-        <v>32143</v>
+      <c r="I36" s="5" t="s">
+        <v>52</v>
       </c>
       <c r="J36" s="5" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="37" spans="1:10" ht="16" customHeight="1">
+      <c r="K36" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L36" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M36" s="5">
+        <v>32143</v>
+      </c>
+      <c r="N36" s="5">
+        <v>32143</v>
+      </c>
+      <c r="O36" s="5">
+        <v>32143</v>
+      </c>
+      <c r="P36" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q36" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="37" spans="1:17" ht="16" customHeight="1">
       <c r="A37" s="2" t="s">
         <v>31</v>
       </c>
@@ -3006,20 +3815,41 @@
       <c r="F37" s="5">
         <v>25569</v>
       </c>
-      <c r="G37" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="H37" s="5">
-        <v>32143</v>
-      </c>
-      <c r="I37" s="5" t="s">
-        <v>52</v>
+      <c r="G37" s="5">
+        <v>25569</v>
+      </c>
+      <c r="H37" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I37" s="5">
+        <v>32143</v>
       </c>
       <c r="J37" s="5" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="38" spans="1:10" ht="16" customHeight="1">
+      <c r="K37" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L37" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M37" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N37" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O37" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P37" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q37" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="38" spans="1:17" ht="16" customHeight="1">
       <c r="A38" s="2" t="s">
         <v>32</v>
       </c>
@@ -3045,13 +3875,34 @@
         <v>52</v>
       </c>
       <c r="I38" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J38" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="K38" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L38" s="5" t="s">
         <v>312</v>
       </c>
-      <c r="J38" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" ht="16" customHeight="1">
+      <c r="M38" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="N38" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="O38" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="P38" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q38" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="39" spans="1:17" ht="16" customHeight="1">
       <c r="A39" s="2" t="s">
         <v>33</v>
       </c>
@@ -3079,11 +3930,32 @@
       <c r="I39" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="J39" s="5">
+      <c r="J39" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="K39" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L39" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M39" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N39" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O39" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P39" s="5">
         <v>34367</v>
       </c>
-    </row>
-    <row r="40" spans="1:10" ht="16" customHeight="1">
+      <c r="Q39" s="5">
+        <v>34367</v>
+      </c>
+    </row>
+    <row r="40" spans="1:17" ht="16" customHeight="1">
       <c r="A40" s="2" t="s">
         <v>34</v>
       </c>
@@ -3108,14 +3980,35 @@
       <c r="H40" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="I40" s="5">
-        <v>32143</v>
+      <c r="I40" s="5" t="s">
+        <v>52</v>
       </c>
       <c r="J40" s="5" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="41" spans="1:10" ht="16" customHeight="1">
+      <c r="K40" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L40" s="5">
+        <v>32143</v>
+      </c>
+      <c r="M40" s="5">
+        <v>32143</v>
+      </c>
+      <c r="N40" s="5">
+        <v>32143</v>
+      </c>
+      <c r="O40" s="5">
+        <v>32143</v>
+      </c>
+      <c r="P40" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q40" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="41" spans="1:17" ht="16" customHeight="1">
       <c r="A41" s="2" t="s">
         <v>35</v>
       </c>
@@ -3137,17 +4030,39 @@
       <c r="G41" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="H41" s="5">
+      <c r="H41" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I41" s="5">
         <v>34760</v>
       </c>
-      <c r="I41" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="J41" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" ht="16" customHeight="1">
+      <c r="J41" s="5">
+        <v>34760</v>
+      </c>
+      <c r="K41" s="5">
+        <f>B41</f>
+        <v>34760</v>
+      </c>
+      <c r="L41" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M41" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N41" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O41" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P41" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q41" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="42" spans="1:17" ht="16" customHeight="1">
       <c r="A42" s="2" t="s">
         <v>36</v>
       </c>
@@ -3170,16 +4085,38 @@
         <v>35765</v>
       </c>
       <c r="H42" s="5">
-        <v>32143</v>
-      </c>
-      <c r="I42" s="5" t="s">
-        <v>52</v>
+        <v>35765</v>
+      </c>
+      <c r="I42" s="5">
+        <v>32143</v>
       </c>
       <c r="J42" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" ht="16" customHeight="1">
+        <v>304</v>
+      </c>
+      <c r="K42" s="5" t="str">
+        <f>C42</f>
+        <v>1-Jan-1988 to 30-Nov-1997</v>
+      </c>
+      <c r="L42" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M42" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N42" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O42" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P42" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q42" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="43" spans="1:17" ht="16" customHeight="1">
       <c r="A43" s="2" t="s">
         <v>37</v>
       </c>
@@ -3201,17 +4138,38 @@
       <c r="G43" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="H43" s="5">
+      <c r="H43" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I43" s="5">
         <v>41792</v>
       </c>
-      <c r="I43" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="J43" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" ht="16" customHeight="1">
+      <c r="J43" s="5">
+        <v>41792</v>
+      </c>
+      <c r="K43" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L43" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M43" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N43" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O43" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P43" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q43" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="44" spans="1:17" ht="16" customHeight="1">
       <c r="A44" s="2" t="s">
         <v>38</v>
       </c>
@@ -3234,16 +4192,38 @@
         <v>52</v>
       </c>
       <c r="H44" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I44" s="5" t="s">
         <v>305</v>
       </c>
-      <c r="I44" s="5" t="s">
-        <v>52</v>
-      </c>
       <c r="J44" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10" ht="16" customHeight="1">
+        <v>305</v>
+      </c>
+      <c r="K44" s="5" t="str">
+        <f>C44</f>
+        <v>01-Dec-1997 to 9-Mar-2022</v>
+      </c>
+      <c r="L44" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M44" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N44" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O44" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P44" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q44" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="45" spans="1:17" ht="16" customHeight="1">
       <c r="A45" s="2" t="s">
         <v>39</v>
       </c>
@@ -3265,17 +4245,38 @@
       <c r="G45" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="H45" s="5">
+      <c r="H45" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I45" s="5">
         <v>43614</v>
       </c>
-      <c r="I45" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="J45" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10" ht="16" customHeight="1">
+      <c r="J45" s="5">
+        <v>43614</v>
+      </c>
+      <c r="K45" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L45" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M45" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N45" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O45" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P45" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q45" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="46" spans="1:17" ht="16" customHeight="1">
       <c r="A46" s="3" t="s">
         <v>51</v>
       </c>
@@ -3300,14 +4301,35 @@
       <c r="H46" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="I46" s="5">
-        <v>32143</v>
+      <c r="I46" s="5" t="s">
+        <v>52</v>
       </c>
       <c r="J46" s="5" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="47" spans="1:10" ht="16" customHeight="1">
+      <c r="K46" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L46" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M46" s="5">
+        <v>32143</v>
+      </c>
+      <c r="N46" s="5">
+        <v>32143</v>
+      </c>
+      <c r="O46" s="5">
+        <v>32143</v>
+      </c>
+      <c r="P46" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q46" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="47" spans="1:17" ht="16" customHeight="1">
       <c r="A47" s="2" t="s">
         <v>40</v>
       </c>
@@ -3338,8 +4360,29 @@
       <c r="J47" s="5" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="48" spans="1:10" ht="16" customHeight="1">
+      <c r="K47" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L47" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M47" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N47" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O47" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P47" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q47" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="48" spans="1:17" ht="16" customHeight="1">
       <c r="A48" s="2" t="s">
         <v>314</v>
       </c>
@@ -3370,8 +4413,29 @@
       <c r="J48" s="5" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="49" spans="1:10" ht="16" customHeight="1">
+      <c r="K48" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L48" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M48" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N48" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O48" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P48" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q48" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="49" spans="1:17" ht="16" customHeight="1">
       <c r="A49" s="2" t="s">
         <v>41</v>
       </c>
@@ -3391,19 +4455,40 @@
         <v>25569</v>
       </c>
       <c r="G49" s="5">
-        <v>32143</v>
+        <v>25569</v>
       </c>
       <c r="H49" s="5">
         <v>32143</v>
       </c>
-      <c r="I49" s="5" t="s">
-        <v>52</v>
+      <c r="I49" s="5">
+        <v>32143</v>
       </c>
       <c r="J49" s="5" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="50" spans="1:10" ht="16" customHeight="1">
+      <c r="K49" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L49" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M49" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N49" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O49" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P49" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q49" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="50" spans="1:17" ht="16" customHeight="1">
       <c r="A50" s="2" t="s">
         <v>42</v>
       </c>
@@ -3429,13 +4514,34 @@
         <v>52</v>
       </c>
       <c r="I50" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J50" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="K50" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L50" s="5" t="s">
         <v>306</v>
       </c>
-      <c r="J50" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10" ht="16" customHeight="1">
+      <c r="M50" s="5" t="s">
+        <v>306</v>
+      </c>
+      <c r="N50" s="5" t="s">
+        <v>306</v>
+      </c>
+      <c r="O50" s="5" t="s">
+        <v>306</v>
+      </c>
+      <c r="P50" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q50" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="51" spans="1:17" ht="16" customHeight="1">
       <c r="A51" s="2" t="s">
         <v>43</v>
       </c>
@@ -3454,20 +4560,41 @@
       <c r="F51" s="5">
         <v>25569</v>
       </c>
-      <c r="G51" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="H51" s="5">
-        <v>32143</v>
-      </c>
-      <c r="I51" s="5" t="s">
-        <v>52</v>
+      <c r="G51" s="5">
+        <v>25569</v>
+      </c>
+      <c r="H51" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I51" s="5">
+        <v>32143</v>
       </c>
       <c r="J51" s="5" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="52" spans="1:10" ht="16" customHeight="1">
+      <c r="K51" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L51" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M51" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N51" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O51" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P51" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q51" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="52" spans="1:17" ht="16" customHeight="1">
       <c r="A52" s="2" t="s">
         <v>44</v>
       </c>
@@ -3486,20 +4613,41 @@
       <c r="F52" s="5">
         <v>25569</v>
       </c>
-      <c r="G52" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="H52" s="5">
-        <v>32143</v>
-      </c>
-      <c r="I52" s="5" t="s">
-        <v>52</v>
+      <c r="G52" s="5">
+        <v>25569</v>
+      </c>
+      <c r="H52" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I52" s="5">
+        <v>32143</v>
       </c>
       <c r="J52" s="5" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="53" spans="1:10" ht="16" customHeight="1">
+      <c r="K52" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L52" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M52" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N52" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O52" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P52" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q52" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="53" spans="1:17" ht="16" customHeight="1">
       <c r="A53" s="2" t="s">
         <v>45</v>
       </c>
@@ -3524,14 +4672,35 @@
       <c r="H53" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="I53" s="5">
+      <c r="I53" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J53" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="K53" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L53" s="5">
         <v>37410</v>
       </c>
-      <c r="J53" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" ht="16" customHeight="1">
+      <c r="M53" s="5">
+        <v>37410</v>
+      </c>
+      <c r="N53" s="5">
+        <v>37410</v>
+      </c>
+      <c r="O53" s="5">
+        <v>37410</v>
+      </c>
+      <c r="P53" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q53" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="54" spans="1:17" ht="16" customHeight="1">
       <c r="A54" s="7" t="s">
         <v>59</v>
       </c>
@@ -3557,13 +4726,34 @@
         <v>52</v>
       </c>
       <c r="I54" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J54" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="K54" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L54" s="5" t="s">
         <v>307</v>
       </c>
-      <c r="J54" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" ht="16" customHeight="1">
+      <c r="M54" s="5" t="s">
+        <v>307</v>
+      </c>
+      <c r="N54" s="5" t="s">
+        <v>307</v>
+      </c>
+      <c r="O54" s="5" t="s">
+        <v>307</v>
+      </c>
+      <c r="P54" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q54" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="55" spans="1:17" ht="16" customHeight="1">
       <c r="A55" s="2" t="s">
         <v>46</v>
       </c>
@@ -3588,14 +4778,35 @@
       <c r="H55" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="I55" s="5">
-        <v>32143</v>
+      <c r="I55" s="5" t="s">
+        <v>52</v>
       </c>
       <c r="J55" s="5" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="56" spans="1:10" ht="16" customHeight="1">
+      <c r="K55" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L55" s="5">
+        <v>32143</v>
+      </c>
+      <c r="M55" s="5">
+        <v>32143</v>
+      </c>
+      <c r="N55" s="5">
+        <v>32143</v>
+      </c>
+      <c r="O55" s="5">
+        <v>32143</v>
+      </c>
+      <c r="P55" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q55" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="56" spans="1:17" ht="16" customHeight="1">
       <c r="A56" s="2" t="s">
         <v>47</v>
       </c>
@@ -3617,17 +4828,39 @@
       <c r="G56" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="H56" s="5">
+      <c r="H56" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I56" s="5">
         <v>35339</v>
       </c>
-      <c r="I56" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="J56" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10" ht="16" customHeight="1">
+      <c r="J56" s="5">
+        <v>32752</v>
+      </c>
+      <c r="K56" s="5">
+        <f>C56</f>
+        <v>32752</v>
+      </c>
+      <c r="L56" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M56" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N56" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O56" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P56" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q56" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="57" spans="1:17" ht="16" customHeight="1">
       <c r="A57" s="2" t="s">
         <v>48</v>
       </c>
@@ -3649,17 +4882,38 @@
       <c r="G57" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="H57" s="5">
+      <c r="H57" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I57" s="5">
         <v>41792</v>
       </c>
-      <c r="I57" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="J57" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="58" spans="1:10" ht="16" customHeight="1">
+      <c r="J57" s="5">
+        <v>41792</v>
+      </c>
+      <c r="K57" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L57" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M57" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N57" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O57" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P57" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q57" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="58" spans="1:17" ht="16" customHeight="1">
       <c r="A58" s="2" t="s">
         <v>49</v>
       </c>
@@ -3681,17 +4935,38 @@
       <c r="G58" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="H58" s="5">
-        <v>32143</v>
-      </c>
-      <c r="I58" s="5" t="s">
-        <v>52</v>
+      <c r="H58" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I58" s="5">
+        <v>32143</v>
       </c>
       <c r="J58" s="5" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="59" spans="1:10" ht="16" customHeight="1">
+      <c r="K58" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L58" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M58" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N58" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O58" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P58" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q58" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="59" spans="1:17" ht="16" customHeight="1">
       <c r="A59" s="3" t="s">
         <v>60</v>
       </c>
@@ -3719,11 +4994,32 @@
       <c r="I59" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="J59" s="5">
-        <v>32143</v>
-      </c>
-    </row>
-    <row r="60" spans="1:10" ht="16" customHeight="1">
+      <c r="J59" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="K59" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L59" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M59" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N59" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O59" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P59" s="5">
+        <v>32143</v>
+      </c>
+      <c r="Q59" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="60" spans="1:17" ht="16" customHeight="1">
       <c r="A60" s="2" t="s">
         <v>50</v>
       </c>
@@ -3752,10 +5048,32 @@
         <v>52</v>
       </c>
       <c r="J60" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="K60" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L60" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M60" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N60" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O60" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P60" s="5" t="s">
         <v>308</v>
       </c>
+      <c r="Q60" s="5" t="s">
+        <v>308</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="8" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="A54" r:id="rId1" xr:uid="{52D16EEC-E5ED-404C-86D1-39D51CBCCAC6}"/>
   </hyperlinks>

</xml_diff>

<commit_message>
build MSCI exchange rates
</commit_message>
<xml_diff>
--- a/epsilon-phi-core/src/resources/templates/MSCI Index Construction.xlsx
+++ b/epsilon-phi-core/src/resources/templates/MSCI Index Construction.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11028"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11116"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/francisbarker/Repositories/Python/epsilon-phi/epsilon-phi-core/src/resources/templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/francisbarker/repo/epsilon-psi/epsilon-phi-core/src/resources/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FC6A07D-DF23-9147-BF18-0A936BA28C8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{652D156E-8F40-0C4E-9D5B-50C712D6474D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="57600" windowHeight="30000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="19360" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rules" sheetId="40" r:id="rId1"/>
@@ -871,9 +871,6 @@
     <t>PTE</t>
   </si>
   <si>
-    <t>QAD</t>
-  </si>
-  <si>
     <t>RUB</t>
   </si>
   <si>
@@ -1429,6 +1426,9 @@
   </si>
   <si>
     <t>MSEFLA$</t>
+  </si>
+  <si>
+    <t>QAR</t>
   </si>
 </sst>
 </file>
@@ -1892,52 +1892,52 @@
         <v>120</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>54</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="H1" s="4" t="s">
         <v>55</v>
       </c>
       <c r="I1" s="4" t="s">
+        <v>321</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>327</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>328</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="M1" s="4" t="s">
         <v>322</v>
       </c>
-      <c r="J1" s="4" t="s">
-        <v>328</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>329</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>334</v>
-      </c>
-      <c r="M1" s="4" t="s">
+      <c r="N1" s="4" t="s">
+        <v>324</v>
+      </c>
+      <c r="O1" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="P1" s="4" t="s">
         <v>323</v>
       </c>
-      <c r="N1" s="4" t="s">
-        <v>325</v>
-      </c>
-      <c r="O1" s="4" t="s">
-        <v>326</v>
-      </c>
-      <c r="P1" s="4" t="s">
-        <v>324</v>
-      </c>
       <c r="Q1" s="4" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="2" spans="1:17" s="11" customFormat="1" ht="19" customHeight="1">
@@ -1960,37 +1960,37 @@
         <v>115</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="I2" s="4" t="s">
         <v>117</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="K2" s="4" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="L2" s="4" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="M2" s="4" t="s">
         <v>118</v>
       </c>
       <c r="N2" s="4" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="O2" s="4" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="P2" s="4" t="s">
         <v>119</v>
       </c>
       <c r="Q2" s="4" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="3" spans="1:17" ht="30">
@@ -1998,10 +1998,10 @@
         <v>0</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>52</v>
@@ -2040,10 +2040,10 @@
         <v>52</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="4" spans="1:17" ht="16" customHeight="1">
@@ -2797,28 +2797,28 @@
         <v>32143</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="I18" s="5">
         <v>32143</v>
       </c>
       <c r="J18" s="5" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="K18" s="5" t="str">
         <f>C18</f>
@@ -3117,7 +3117,7 @@
         <v>34367</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D24" s="5">
         <v>40325</v>
@@ -3138,7 +3138,7 @@
         <v>34760</v>
       </c>
       <c r="J24" s="5" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K24" s="5" t="s">
         <v>52</v>
@@ -3273,10 +3273,10 @@
         <v>22</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D27" s="5" t="s">
         <v>52</v>
@@ -3294,10 +3294,10 @@
         <v>52</v>
       </c>
       <c r="I27" s="5" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="J27" s="5" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="K27" s="5" t="s">
         <v>52</v>
@@ -3429,10 +3429,10 @@
     </row>
     <row r="30" spans="1:17" ht="16" customHeight="1">
       <c r="A30" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>52</v>
@@ -3485,16 +3485,16 @@
         <v>26</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="F31" s="5" t="s">
         <v>52</v>
@@ -3513,16 +3513,16 @@
         <v>52</v>
       </c>
       <c r="L31" s="5" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="M31" s="5" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="N31" s="5" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="O31" s="5" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="P31" s="5" t="s">
         <v>52</v>
@@ -3586,7 +3586,7 @@
     </row>
     <row r="33" spans="1:17" ht="16" customHeight="1">
       <c r="A33" s="2" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>52</v>
@@ -3595,7 +3595,7 @@
         <v>52</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="E33" s="5" t="s">
         <v>52</v>
@@ -3642,10 +3642,10 @@
         <v>28</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>52</v>
@@ -3854,10 +3854,10 @@
         <v>32</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>52</v>
@@ -3884,16 +3884,16 @@
         <v>52</v>
       </c>
       <c r="L38" s="5" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="M38" s="5" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="N38" s="5" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="O38" s="5" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="P38" s="5" t="s">
         <v>52</v>
@@ -4070,7 +4070,7 @@
         <v>32143</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D42" s="5">
         <v>35765</v>
@@ -4091,7 +4091,7 @@
         <v>32143</v>
       </c>
       <c r="J42" s="5" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="K42" s="5" t="str">
         <f>C42</f>
@@ -4174,10 +4174,10 @@
         <v>38</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="D44" s="5" t="s">
         <v>52</v>
@@ -4195,10 +4195,10 @@
         <v>52</v>
       </c>
       <c r="I44" s="5" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="J44" s="5" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="K44" s="5" t="str">
         <f>C44</f>
@@ -4384,16 +4384,16 @@
     </row>
     <row r="48" spans="1:17" ht="16" customHeight="1">
       <c r="A48" s="2" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C48" s="5" t="s">
         <v>52</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="E48" s="5" t="s">
         <v>52</v>
@@ -4493,10 +4493,10 @@
         <v>42</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="D50" s="5" t="s">
         <v>52</v>
@@ -4523,16 +4523,16 @@
         <v>52</v>
       </c>
       <c r="L50" s="5" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="M50" s="5" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="N50" s="5" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="O50" s="5" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="P50" s="5" t="s">
         <v>52</v>
@@ -4705,10 +4705,10 @@
         <v>59</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D54" s="5" t="s">
         <v>52</v>
@@ -4735,16 +4735,16 @@
         <v>52</v>
       </c>
       <c r="L54" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="M54" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="N54" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="O54" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="P54" s="5" t="s">
         <v>52</v>
@@ -5024,10 +5024,10 @@
         <v>50</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="D60" s="5" t="s">
         <v>52</v>
@@ -5066,10 +5066,10 @@
         <v>52</v>
       </c>
       <c r="P60" s="5" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="Q60" s="5" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
   </sheetData>
@@ -5100,10 +5100,10 @@
         <v>122</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>124</v>
@@ -5117,10 +5117,10 @@
         <v>104</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E3" s="12" t="s">
         <v>125</v>
@@ -5134,10 +5134,10 @@
         <v>61</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E4" s="12" t="s">
         <v>126</v>
@@ -5151,10 +5151,10 @@
         <v>62</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E5" s="12" t="s">
         <v>127</v>
@@ -5168,10 +5168,10 @@
         <v>63</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E6" s="12" t="s">
         <v>128</v>
@@ -5185,10 +5185,10 @@
         <v>64</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="E7" s="12" t="s">
         <v>129</v>
@@ -5202,10 +5202,10 @@
         <v>65</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E8" s="12" t="s">
         <v>130</v>
@@ -5219,13 +5219,13 @@
         <v>66</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="14" customHeight="1">
@@ -5236,10 +5236,10 @@
         <v>67</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E10" s="12" t="s">
         <v>131</v>
@@ -5253,10 +5253,10 @@
         <v>68</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E11" s="12" t="s">
         <v>132</v>
@@ -5270,10 +5270,10 @@
         <v>69</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E12" s="12" t="s">
         <v>133</v>
@@ -5287,10 +5287,10 @@
         <v>70</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E13" s="12" t="s">
         <v>134</v>
@@ -5304,13 +5304,13 @@
         <v>71</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="14" customHeight="1">
@@ -5321,10 +5321,10 @@
         <v>72</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D15" s="12" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E15" s="12" t="s">
         <v>135</v>
@@ -5338,10 +5338,10 @@
         <v>73</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E16" s="12" t="s">
         <v>136</v>
@@ -5355,10 +5355,10 @@
         <v>74</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E17" s="12" t="s">
         <v>137</v>
@@ -5372,10 +5372,10 @@
         <v>75</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="E18" s="12" t="s">
         <v>138</v>
@@ -5389,10 +5389,10 @@
         <v>76</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="E19" s="12" t="s">
         <v>139</v>
@@ -5406,10 +5406,10 @@
         <v>77</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E20" s="12" t="s">
         <v>140</v>
@@ -5423,10 +5423,10 @@
         <v>78</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="E21" s="12" t="s">
         <v>141</v>
@@ -5440,10 +5440,10 @@
         <v>79</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="E22" s="12" t="s">
         <v>142</v>
@@ -5457,13 +5457,13 @@
         <v>80</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D23" s="12" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E23" s="12" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="14" customHeight="1">
@@ -5474,10 +5474,10 @@
         <v>81</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E24" s="12" t="s">
         <v>143</v>
@@ -5491,10 +5491,10 @@
         <v>82</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E25" s="12" t="s">
         <v>144</v>
@@ -5508,10 +5508,10 @@
         <v>83</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E26" s="12" t="s">
         <v>145</v>
@@ -5525,10 +5525,10 @@
         <v>105</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D27" s="12" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E27" s="12" t="s">
         <v>146</v>
@@ -5539,13 +5539,13 @@
         <v>23</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E28" s="12" t="s">
         <v>147</v>
@@ -5559,13 +5559,13 @@
         <v>84</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E29" s="12" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="14" customHeight="1">
@@ -5576,10 +5576,10 @@
         <v>106</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E30" s="12" t="s">
         <v>148</v>
@@ -5593,10 +5593,10 @@
         <v>85</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E31" s="12" t="s">
         <v>149</v>
@@ -5610,10 +5610,10 @@
         <v>86</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D32" s="12" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E32" s="12" t="s">
         <v>150</v>
@@ -5621,16 +5621,16 @@
     </row>
     <row r="33" spans="1:5" ht="14" customHeight="1">
       <c r="A33" s="2" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>86</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="E33" s="12" t="s">
         <v>150</v>
@@ -5644,10 +5644,10 @@
         <v>107</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="D34" s="12" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E34" s="12" t="s">
         <v>151</v>
@@ -5661,13 +5661,13 @@
         <v>87</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="D35" s="12" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E35" s="12" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="14" customHeight="1">
@@ -5678,10 +5678,10 @@
         <v>88</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="D36" s="12" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E36" s="12" t="s">
         <v>152</v>
@@ -5695,10 +5695,10 @@
         <v>89</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="D37" s="12" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E37" s="12" t="s">
         <v>153</v>
@@ -5712,10 +5712,10 @@
         <v>108</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="D38" s="12" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="E38" s="12" t="s">
         <v>154</v>
@@ -5729,10 +5729,10 @@
         <v>90</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E39" s="12" t="s">
         <v>155</v>
@@ -5746,10 +5746,10 @@
         <v>91</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D40" s="12" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E40" s="12" t="s">
         <v>156</v>
@@ -5763,10 +5763,10 @@
         <v>92</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D41" s="12" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E41" s="12" t="s">
         <v>157</v>
@@ -5780,10 +5780,10 @@
         <v>93</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D42" s="12" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E42" s="12" t="s">
         <v>158</v>
@@ -5797,13 +5797,13 @@
         <v>94</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E43" s="12" t="s">
-        <v>159</v>
+        <v>340</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="14" customHeight="1">
@@ -5814,13 +5814,13 @@
         <v>109</v>
       </c>
       <c r="C44" s="8" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="D44" s="12" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="E44" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="14" customHeight="1">
@@ -5831,13 +5831,13 @@
         <v>95</v>
       </c>
       <c r="C45" s="8" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D45" s="12" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E45" s="12" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="14" customHeight="1">
@@ -5848,13 +5848,13 @@
         <v>96</v>
       </c>
       <c r="C46" s="8" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D46" s="12" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E46" s="12" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="14">
@@ -5865,13 +5865,13 @@
         <v>96</v>
       </c>
       <c r="C47" s="8" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D47" s="12" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E47" s="12" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="48" spans="1:5" ht="14">
@@ -5882,30 +5882,30 @@
         <v>97</v>
       </c>
       <c r="C48" s="8" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D48" s="12" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E48" s="12" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="49" spans="1:5" ht="12" customHeight="1">
       <c r="A49" s="2" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B49" s="1" t="s">
         <v>97</v>
       </c>
       <c r="C49" s="8" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D49" s="12" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="E49" s="12" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="50" spans="1:5" ht="14">
@@ -5916,13 +5916,13 @@
         <v>98</v>
       </c>
       <c r="C50" s="8" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D50" s="12" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E50" s="12" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="51" spans="1:5" ht="14">
@@ -5933,13 +5933,13 @@
         <v>110</v>
       </c>
       <c r="C51" s="8" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D51" s="12" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E51" s="12" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="52" spans="1:5" ht="14">
@@ -5950,13 +5950,13 @@
         <v>99</v>
       </c>
       <c r="C52" s="8" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="D52" s="12" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E52" s="12" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="53" spans="1:5" ht="14">
@@ -5967,13 +5967,13 @@
         <v>100</v>
       </c>
       <c r="C53" s="8" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D53" s="12" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="E53" s="12" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="14">
@@ -5984,13 +5984,13 @@
         <v>101</v>
       </c>
       <c r="C54" s="8" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D54" s="12" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E54" s="12" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="55" spans="1:5" ht="14">
@@ -6001,13 +6001,13 @@
         <v>101</v>
       </c>
       <c r="C55" s="8" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D55" s="12" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E55" s="12" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="56" spans="1:5" ht="14">
@@ -6018,13 +6018,13 @@
         <v>102</v>
       </c>
       <c r="C56" s="8" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D56" s="12" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E56" s="12" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="14">
@@ -6035,13 +6035,13 @@
         <v>103</v>
       </c>
       <c r="C57" s="8" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D57" s="12" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E57" s="12" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="58" spans="1:5" ht="14">
@@ -6049,16 +6049,16 @@
         <v>48</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="C58" s="8" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="D58" s="12" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="E58" s="12" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="14">
@@ -6066,16 +6066,16 @@
         <v>49</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C59" s="8" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D59" s="12" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="E59" s="12" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="14">
@@ -6083,16 +6083,16 @@
         <v>60</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C60" s="8" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D60" s="12" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E60" s="12" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="14">
@@ -6100,16 +6100,16 @@
         <v>50</v>
       </c>
       <c r="B61" s="8" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C61" s="8" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D61" s="12" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E61" s="12" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="70" spans="2:7" ht="14">
@@ -6146,31 +6146,31 @@
         <v>120</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>53</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>54</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>55</v>
       </c>
       <c r="H1" s="4" t="s">
+        <v>321</v>
+      </c>
+      <c r="I1" s="4" t="s">
         <v>322</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="J1" s="4" t="s">
         <v>323</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>324</v>
       </c>
     </row>
     <row r="2" spans="1:14" s="11" customFormat="1" ht="19" customHeight="1">
@@ -6210,10 +6210,10 @@
         <v>0</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>52</v>
@@ -6234,7 +6234,7 @@
         <v>52</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="16" customHeight="1">
@@ -6707,19 +6707,19 @@
         <v>32143</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="H18" s="5">
         <v>32143</v>
@@ -6905,7 +6905,7 @@
         <v>34367</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D24" s="5">
         <v>40325</v>
@@ -7001,10 +7001,10 @@
         <v>22</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D27" s="5" t="s">
         <v>52</v>
@@ -7019,7 +7019,7 @@
         <v>52</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="I27" s="5" t="s">
         <v>52</v>
@@ -7095,10 +7095,10 @@
     </row>
     <row r="30" spans="1:14" ht="16" customHeight="1">
       <c r="A30" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>52</v>
@@ -7116,7 +7116,7 @@
         <v>52</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="I30" s="5" t="s">
         <v>52</v>
@@ -7130,16 +7130,16 @@
         <v>26</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="F31" s="5" t="s">
         <v>52</v>
@@ -7151,7 +7151,7 @@
         <v>52</v>
       </c>
       <c r="I31" s="5" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="J31" s="5" t="s">
         <v>52</v>
@@ -7191,7 +7191,7 @@
     </row>
     <row r="33" spans="1:10" ht="16" customHeight="1">
       <c r="A33" s="2" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>52</v>
@@ -7200,7 +7200,7 @@
         <v>52</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="E33" s="5" t="s">
         <v>52</v>
@@ -7226,10 +7226,10 @@
         <v>28</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>52</v>
@@ -7354,10 +7354,10 @@
         <v>32</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>52</v>
@@ -7375,7 +7375,7 @@
         <v>52</v>
       </c>
       <c r="I38" s="5" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="J38" s="5" t="s">
         <v>52</v>
@@ -7485,7 +7485,7 @@
         <v>32143</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D42" s="5">
         <v>35765</v>
@@ -7546,10 +7546,10 @@
         <v>38</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="D44" s="5" t="s">
         <v>52</v>
@@ -7564,7 +7564,7 @@
         <v>52</v>
       </c>
       <c r="H44" s="5" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="I44" s="5" t="s">
         <v>52</v>
@@ -7671,16 +7671,16 @@
     </row>
     <row r="48" spans="1:10" ht="16" customHeight="1">
       <c r="A48" s="2" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C48" s="5" t="s">
         <v>52</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="E48" s="5" t="s">
         <v>52</v>
@@ -7738,10 +7738,10 @@
         <v>42</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="D50" s="5" t="s">
         <v>52</v>
@@ -7759,7 +7759,7 @@
         <v>52</v>
       </c>
       <c r="I50" s="5" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="J50" s="5" t="s">
         <v>52</v>
@@ -7866,10 +7866,10 @@
         <v>59</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D54" s="5" t="s">
         <v>52</v>
@@ -7887,7 +7887,7 @@
         <v>52</v>
       </c>
       <c r="I54" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J54" s="5" t="s">
         <v>52</v>
@@ -8058,10 +8058,10 @@
         <v>50</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="D60" s="5" t="s">
         <v>52</v>
@@ -8082,7 +8082,7 @@
         <v>52</v>
       </c>
       <c r="J60" s="5" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
custom asset modelling, cash and inflation modelling
</commit_message>
<xml_diff>
--- a/epsilon-phi-core/src/resources/templates/MSCI Index Construction.xlsx
+++ b/epsilon-phi-core/src/resources/templates/MSCI Index Construction.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11116"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10511"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/francisbarker/repo/epsilon-psi/epsilon-phi-core/src/resources/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{652D156E-8F40-0C4E-9D5B-50C712D6474D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{931F26C0-6090-6E47-A8ED-5D8F7361CCED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="19360" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="19120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rules" sheetId="40" r:id="rId1"/>
@@ -907,9 +907,6 @@
     <t>USD</t>
   </si>
   <si>
-    <t>VEF</t>
-  </si>
-  <si>
     <t>CLP</t>
   </si>
   <si>
@@ -1429,6 +1426,9 @@
   </si>
   <si>
     <t>QAR</t>
+  </si>
+  <si>
+    <t>VEB</t>
   </si>
 </sst>
 </file>
@@ -1892,52 +1892,52 @@
         <v>120</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>54</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="H1" s="4" t="s">
         <v>55</v>
       </c>
       <c r="I1" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>326</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>327</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>332</v>
+      </c>
+      <c r="M1" s="4" t="s">
         <v>321</v>
       </c>
-      <c r="J1" s="4" t="s">
-        <v>327</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>328</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>333</v>
-      </c>
-      <c r="M1" s="4" t="s">
+      <c r="N1" s="4" t="s">
+        <v>323</v>
+      </c>
+      <c r="O1" s="4" t="s">
+        <v>324</v>
+      </c>
+      <c r="P1" s="4" t="s">
         <v>322</v>
       </c>
-      <c r="N1" s="4" t="s">
-        <v>324</v>
-      </c>
-      <c r="O1" s="4" t="s">
-        <v>325</v>
-      </c>
-      <c r="P1" s="4" t="s">
-        <v>323</v>
-      </c>
       <c r="Q1" s="4" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="2" spans="1:17" s="11" customFormat="1" ht="19" customHeight="1">
@@ -1960,37 +1960,37 @@
         <v>115</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="I2" s="4" t="s">
         <v>117</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="K2" s="4" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="L2" s="4" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="M2" s="4" t="s">
         <v>118</v>
       </c>
       <c r="N2" s="4" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="O2" s="4" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="P2" s="4" t="s">
         <v>119</v>
       </c>
       <c r="Q2" s="4" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="3" spans="1:17" ht="30">
@@ -1998,10 +1998,10 @@
         <v>0</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>52</v>
@@ -2040,10 +2040,10 @@
         <v>52</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="4" spans="1:17" ht="16" customHeight="1">
@@ -2797,28 +2797,28 @@
         <v>32143</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="I18" s="5">
         <v>32143</v>
       </c>
       <c r="J18" s="5" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="K18" s="5" t="str">
         <f>C18</f>
@@ -3117,7 +3117,7 @@
         <v>34367</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D24" s="5">
         <v>40325</v>
@@ -3138,7 +3138,7 @@
         <v>34760</v>
       </c>
       <c r="J24" s="5" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K24" s="5" t="s">
         <v>52</v>
@@ -3273,10 +3273,10 @@
         <v>22</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D27" s="5" t="s">
         <v>52</v>
@@ -3294,10 +3294,10 @@
         <v>52</v>
       </c>
       <c r="I27" s="5" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="J27" s="5" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K27" s="5" t="s">
         <v>52</v>
@@ -3429,10 +3429,10 @@
     </row>
     <row r="30" spans="1:17" ht="16" customHeight="1">
       <c r="A30" s="3" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>52</v>
@@ -3485,16 +3485,16 @@
         <v>26</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="F31" s="5" t="s">
         <v>52</v>
@@ -3513,16 +3513,16 @@
         <v>52</v>
       </c>
       <c r="L31" s="5" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="M31" s="5" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="N31" s="5" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="O31" s="5" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="P31" s="5" t="s">
         <v>52</v>
@@ -3586,7 +3586,7 @@
     </row>
     <row r="33" spans="1:17" ht="16" customHeight="1">
       <c r="A33" s="2" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>52</v>
@@ -3595,7 +3595,7 @@
         <v>52</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="E33" s="5" t="s">
         <v>52</v>
@@ -3642,10 +3642,10 @@
         <v>28</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>52</v>
@@ -3854,10 +3854,10 @@
         <v>32</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>52</v>
@@ -3884,16 +3884,16 @@
         <v>52</v>
       </c>
       <c r="L38" s="5" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="M38" s="5" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="N38" s="5" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="O38" s="5" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="P38" s="5" t="s">
         <v>52</v>
@@ -4070,7 +4070,7 @@
         <v>32143</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D42" s="5">
         <v>35765</v>
@@ -4091,7 +4091,7 @@
         <v>32143</v>
       </c>
       <c r="J42" s="5" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="K42" s="5" t="str">
         <f>C42</f>
@@ -4174,10 +4174,10 @@
         <v>38</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D44" s="5" t="s">
         <v>52</v>
@@ -4195,10 +4195,10 @@
         <v>52</v>
       </c>
       <c r="I44" s="5" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="J44" s="5" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="K44" s="5" t="str">
         <f>C44</f>
@@ -4384,16 +4384,16 @@
     </row>
     <row r="48" spans="1:17" ht="16" customHeight="1">
       <c r="A48" s="2" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C48" s="5" t="s">
         <v>52</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E48" s="5" t="s">
         <v>52</v>
@@ -4493,10 +4493,10 @@
         <v>42</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="D50" s="5" t="s">
         <v>52</v>
@@ -4523,16 +4523,16 @@
         <v>52</v>
       </c>
       <c r="L50" s="5" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="M50" s="5" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="N50" s="5" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="O50" s="5" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="P50" s="5" t="s">
         <v>52</v>
@@ -4705,10 +4705,10 @@
         <v>59</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="D54" s="5" t="s">
         <v>52</v>
@@ -4735,16 +4735,16 @@
         <v>52</v>
       </c>
       <c r="L54" s="5" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="M54" s="5" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="N54" s="5" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="O54" s="5" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="P54" s="5" t="s">
         <v>52</v>
@@ -5024,10 +5024,10 @@
         <v>50</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D60" s="5" t="s">
         <v>52</v>
@@ -5066,10 +5066,10 @@
         <v>52</v>
       </c>
       <c r="P60" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="Q60" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
   </sheetData>
@@ -5100,10 +5100,10 @@
         <v>122</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>124</v>
@@ -5117,10 +5117,10 @@
         <v>104</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E3" s="12" t="s">
         <v>125</v>
@@ -5134,10 +5134,10 @@
         <v>61</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E4" s="12" t="s">
         <v>126</v>
@@ -5151,10 +5151,10 @@
         <v>62</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E5" s="12" t="s">
         <v>127</v>
@@ -5168,10 +5168,10 @@
         <v>63</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E6" s="12" t="s">
         <v>128</v>
@@ -5185,10 +5185,10 @@
         <v>64</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E7" s="12" t="s">
         <v>129</v>
@@ -5202,10 +5202,10 @@
         <v>65</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E8" s="12" t="s">
         <v>130</v>
@@ -5219,13 +5219,13 @@
         <v>66</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="14" customHeight="1">
@@ -5236,10 +5236,10 @@
         <v>67</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E10" s="12" t="s">
         <v>131</v>
@@ -5253,10 +5253,10 @@
         <v>68</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E11" s="12" t="s">
         <v>132</v>
@@ -5270,10 +5270,10 @@
         <v>69</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E12" s="12" t="s">
         <v>133</v>
@@ -5287,10 +5287,10 @@
         <v>70</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E13" s="12" t="s">
         <v>134</v>
@@ -5304,13 +5304,13 @@
         <v>71</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="14" customHeight="1">
@@ -5321,10 +5321,10 @@
         <v>72</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D15" s="12" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="E15" s="12" t="s">
         <v>135</v>
@@ -5338,10 +5338,10 @@
         <v>73</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E16" s="12" t="s">
         <v>136</v>
@@ -5355,10 +5355,10 @@
         <v>74</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E17" s="12" t="s">
         <v>137</v>
@@ -5372,10 +5372,10 @@
         <v>75</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E18" s="12" t="s">
         <v>138</v>
@@ -5389,10 +5389,10 @@
         <v>76</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="E19" s="12" t="s">
         <v>139</v>
@@ -5406,10 +5406,10 @@
         <v>77</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="E20" s="12" t="s">
         <v>140</v>
@@ -5423,10 +5423,10 @@
         <v>78</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="E21" s="12" t="s">
         <v>141</v>
@@ -5440,10 +5440,10 @@
         <v>79</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="E22" s="12" t="s">
         <v>142</v>
@@ -5457,13 +5457,13 @@
         <v>80</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D23" s="12" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E23" s="12" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="14" customHeight="1">
@@ -5474,10 +5474,10 @@
         <v>81</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E24" s="12" t="s">
         <v>143</v>
@@ -5491,10 +5491,10 @@
         <v>82</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E25" s="12" t="s">
         <v>144</v>
@@ -5508,10 +5508,10 @@
         <v>83</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E26" s="12" t="s">
         <v>145</v>
@@ -5525,10 +5525,10 @@
         <v>105</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="D27" s="12" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="E27" s="12" t="s">
         <v>146</v>
@@ -5539,13 +5539,13 @@
         <v>23</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E28" s="12" t="s">
         <v>147</v>
@@ -5559,13 +5559,13 @@
         <v>84</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E29" s="12" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="14" customHeight="1">
@@ -5576,10 +5576,10 @@
         <v>106</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="E30" s="12" t="s">
         <v>148</v>
@@ -5593,10 +5593,10 @@
         <v>85</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E31" s="12" t="s">
         <v>149</v>
@@ -5610,10 +5610,10 @@
         <v>86</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D32" s="12" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E32" s="12" t="s">
         <v>150</v>
@@ -5621,16 +5621,16 @@
     </row>
     <row r="33" spans="1:5" ht="14" customHeight="1">
       <c r="A33" s="2" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>86</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E33" s="12" t="s">
         <v>150</v>
@@ -5644,10 +5644,10 @@
         <v>107</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="D34" s="12" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="E34" s="12" t="s">
         <v>151</v>
@@ -5661,13 +5661,13 @@
         <v>87</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D35" s="12" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E35" s="12" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="14" customHeight="1">
@@ -5678,10 +5678,10 @@
         <v>88</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="D36" s="12" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E36" s="12" t="s">
         <v>152</v>
@@ -5695,10 +5695,10 @@
         <v>89</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="D37" s="12" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E37" s="12" t="s">
         <v>153</v>
@@ -5712,10 +5712,10 @@
         <v>108</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="D38" s="12" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="E38" s="12" t="s">
         <v>154</v>
@@ -5729,10 +5729,10 @@
         <v>90</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E39" s="12" t="s">
         <v>155</v>
@@ -5746,10 +5746,10 @@
         <v>91</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D40" s="12" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E40" s="12" t="s">
         <v>156</v>
@@ -5763,10 +5763,10 @@
         <v>92</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D41" s="12" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E41" s="12" t="s">
         <v>157</v>
@@ -5780,10 +5780,10 @@
         <v>93</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D42" s="12" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E42" s="12" t="s">
         <v>158</v>
@@ -5797,13 +5797,13 @@
         <v>94</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E43" s="12" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="14" customHeight="1">
@@ -5814,10 +5814,10 @@
         <v>109</v>
       </c>
       <c r="C44" s="8" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="D44" s="12" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="E44" s="12" t="s">
         <v>159</v>
@@ -5831,10 +5831,10 @@
         <v>95</v>
       </c>
       <c r="C45" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D45" s="12" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E45" s="12" t="s">
         <v>160</v>
@@ -5848,10 +5848,10 @@
         <v>96</v>
       </c>
       <c r="C46" s="8" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D46" s="12" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E46" s="12" t="s">
         <v>161</v>
@@ -5865,10 +5865,10 @@
         <v>96</v>
       </c>
       <c r="C47" s="8" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D47" s="12" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E47" s="12" t="s">
         <v>161</v>
@@ -5882,10 +5882,10 @@
         <v>97</v>
       </c>
       <c r="C48" s="8" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D48" s="12" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E48" s="12" t="s">
         <v>162</v>
@@ -5893,16 +5893,16 @@
     </row>
     <row r="49" spans="1:5" ht="12" customHeight="1">
       <c r="A49" s="2" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B49" s="1" t="s">
         <v>97</v>
       </c>
       <c r="C49" s="8" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D49" s="12" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="E49" s="12" t="s">
         <v>162</v>
@@ -5916,10 +5916,10 @@
         <v>98</v>
       </c>
       <c r="C50" s="8" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D50" s="12" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E50" s="12" t="s">
         <v>163</v>
@@ -5933,13 +5933,13 @@
         <v>110</v>
       </c>
       <c r="C51" s="8" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="D51" s="12" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E51" s="12" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="52" spans="1:5" ht="14">
@@ -5950,10 +5950,10 @@
         <v>99</v>
       </c>
       <c r="C52" s="8" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D52" s="12" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E52" s="12" t="s">
         <v>164</v>
@@ -5967,10 +5967,10 @@
         <v>100</v>
       </c>
       <c r="C53" s="8" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D53" s="12" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E53" s="12" t="s">
         <v>165</v>
@@ -5984,10 +5984,10 @@
         <v>101</v>
       </c>
       <c r="C54" s="8" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D54" s="12" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E54" s="12" t="s">
         <v>166</v>
@@ -6001,10 +6001,10 @@
         <v>101</v>
       </c>
       <c r="C55" s="8" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D55" s="12" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E55" s="12" t="s">
         <v>166</v>
@@ -6018,10 +6018,10 @@
         <v>102</v>
       </c>
       <c r="C56" s="8" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D56" s="12" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E56" s="12" t="s">
         <v>167</v>
@@ -6035,13 +6035,13 @@
         <v>103</v>
       </c>
       <c r="C57" s="8" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D57" s="12" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E57" s="12" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="58" spans="1:5" ht="14">
@@ -6049,13 +6049,13 @@
         <v>48</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C58" s="8" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D58" s="12" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E58" s="12" t="s">
         <v>168</v>
@@ -6066,13 +6066,13 @@
         <v>49</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C59" s="8" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D59" s="12" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="E59" s="12" t="s">
         <v>169</v>
@@ -6083,13 +6083,13 @@
         <v>60</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C60" s="8" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D60" s="12" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="E60" s="12" t="s">
         <v>170</v>
@@ -6100,16 +6100,16 @@
         <v>50</v>
       </c>
       <c r="B61" s="8" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="C61" s="8" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D61" s="12" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="E61" s="12" t="s">
-        <v>171</v>
+        <v>340</v>
       </c>
     </row>
     <row r="70" spans="2:7" ht="14">
@@ -6146,31 +6146,31 @@
         <v>120</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>53</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>54</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>55</v>
       </c>
       <c r="H1" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="I1" s="4" t="s">
         <v>321</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="J1" s="4" t="s">
         <v>322</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>323</v>
       </c>
     </row>
     <row r="2" spans="1:14" s="11" customFormat="1" ht="19" customHeight="1">
@@ -6210,10 +6210,10 @@
         <v>0</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>52</v>
@@ -6234,7 +6234,7 @@
         <v>52</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="16" customHeight="1">
@@ -6707,19 +6707,19 @@
         <v>32143</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H18" s="5">
         <v>32143</v>
@@ -6905,7 +6905,7 @@
         <v>34367</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D24" s="5">
         <v>40325</v>
@@ -7001,10 +7001,10 @@
         <v>22</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D27" s="5" t="s">
         <v>52</v>
@@ -7019,7 +7019,7 @@
         <v>52</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="I27" s="5" t="s">
         <v>52</v>
@@ -7095,10 +7095,10 @@
     </row>
     <row r="30" spans="1:14" ht="16" customHeight="1">
       <c r="A30" s="3" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>52</v>
@@ -7116,7 +7116,7 @@
         <v>52</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="I30" s="5" t="s">
         <v>52</v>
@@ -7130,16 +7130,16 @@
         <v>26</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="F31" s="5" t="s">
         <v>52</v>
@@ -7151,7 +7151,7 @@
         <v>52</v>
       </c>
       <c r="I31" s="5" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="J31" s="5" t="s">
         <v>52</v>
@@ -7191,7 +7191,7 @@
     </row>
     <row r="33" spans="1:10" ht="16" customHeight="1">
       <c r="A33" s="2" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>52</v>
@@ -7200,7 +7200,7 @@
         <v>52</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="E33" s="5" t="s">
         <v>52</v>
@@ -7226,10 +7226,10 @@
         <v>28</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>52</v>
@@ -7354,10 +7354,10 @@
         <v>32</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>52</v>
@@ -7375,7 +7375,7 @@
         <v>52</v>
       </c>
       <c r="I38" s="5" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="J38" s="5" t="s">
         <v>52</v>
@@ -7485,7 +7485,7 @@
         <v>32143</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D42" s="5">
         <v>35765</v>
@@ -7546,10 +7546,10 @@
         <v>38</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D44" s="5" t="s">
         <v>52</v>
@@ -7564,7 +7564,7 @@
         <v>52</v>
       </c>
       <c r="H44" s="5" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="I44" s="5" t="s">
         <v>52</v>
@@ -7671,16 +7671,16 @@
     </row>
     <row r="48" spans="1:10" ht="16" customHeight="1">
       <c r="A48" s="2" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C48" s="5" t="s">
         <v>52</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E48" s="5" t="s">
         <v>52</v>
@@ -7738,10 +7738,10 @@
         <v>42</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="D50" s="5" t="s">
         <v>52</v>
@@ -7759,7 +7759,7 @@
         <v>52</v>
       </c>
       <c r="I50" s="5" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="J50" s="5" t="s">
         <v>52</v>
@@ -7866,10 +7866,10 @@
         <v>59</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="D54" s="5" t="s">
         <v>52</v>
@@ -7887,7 +7887,7 @@
         <v>52</v>
       </c>
       <c r="I54" s="5" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="J54" s="5" t="s">
         <v>52</v>
@@ -8058,10 +8058,10 @@
         <v>50</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D60" s="5" t="s">
         <v>52</v>
@@ -8082,7 +8082,7 @@
         <v>52</v>
       </c>
       <c r="J60" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
   </sheetData>

</xml_diff>